<commit_message>
Log Week 1 Day 1 training (Wed 22 Jul)
Push gym session completed in full; easy 4km run completed as
planned, RPE 4, felt great.
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1200" yWindow="680" windowWidth="33000" windowHeight="21460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workouts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Changelog" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weekly Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Workouts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Weekly Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Plan Changelog" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Weekly Plan'!$A$1:$Q$199</definedName>
@@ -1233,13 +1233,21 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L2" s="15" t="n"/>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M2" s="15" t="n"/>
       <c r="N2" s="15" t="n"/>
       <c r="O2" s="15" t="n"/>
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="15" t="n"/>
-      <c r="R2" s="15" t="n"/>
+      <c r="R2" s="15" t="inlineStr">
+        <is>
+          <t>Full session completed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="n">
@@ -1291,12 +1299,24 @@
           <t>Easy run</t>
         </is>
       </c>
-      <c r="L3" s="15" t="n"/>
-      <c r="M3" s="15" t="n"/>
+      <c r="L3" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M3" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="N3" s="15" t="n"/>
       <c r="O3" s="15" t="n"/>
-      <c r="P3" s="15" t="n"/>
-      <c r="Q3" s="15" t="n"/>
+      <c r="P3" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q3" s="15" t="inlineStr">
+        <is>
+          <t>Great</t>
+        </is>
+      </c>
       <c r="R3" s="15" t="n"/>
     </row>
     <row r="4">
@@ -14546,7 +14566,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="43" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add actual pace/duration for Week 1 easy run (6:00/km)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -1307,8 +1307,16 @@
       <c r="M3" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="N3" s="15" t="n"/>
-      <c r="O3" s="15" t="n"/>
+      <c r="N3" s="15" t="inlineStr">
+        <is>
+          <t>0:24:00</t>
+        </is>
+      </c>
+      <c r="O3" s="15" t="inlineStr">
+        <is>
+          <t>6:00</t>
+        </is>
+      </c>
       <c r="P3" s="15" t="n">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Fix Wk2 Mon log: football fully replaced the run, not completed
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1420" yWindow="680" windowWidth="32780" windowHeight="21460" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1420" yWindow="760" windowWidth="32780" windowHeight="21460" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="168" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
-    <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -342,6 +342,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="20" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -360,14 +368,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="20" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -751,16 +751,16 @@
   <dimension ref="B2:F28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" style="46" min="1" max="1"/>
-    <col width="17" bestFit="1" customWidth="1" style="46" min="2" max="2"/>
-    <col width="32.1640625" bestFit="1" customWidth="1" style="46" min="3" max="3"/>
-    <col width="45.5" bestFit="1" customWidth="1" style="46" min="4" max="4"/>
-    <col width="33" bestFit="1" customWidth="1" style="46" min="5" max="5"/>
-    <col width="10" customWidth="1" style="46" min="6" max="6"/>
+    <col width="2" customWidth="1" style="52" min="1" max="1"/>
+    <col width="17" bestFit="1" customWidth="1" style="52" min="2" max="2"/>
+    <col width="32.1640625" bestFit="1" customWidth="1" style="52" min="3" max="3"/>
+    <col width="45.5" bestFit="1" customWidth="1" style="52" min="4" max="4"/>
+    <col width="33" bestFit="1" customWidth="1" style="52" min="5" max="5"/>
+    <col width="10" customWidth="1" style="52" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="2" ht="18" customHeight="1" s="46">
-      <c r="B2" s="45" t="inlineStr">
+    <row r="2" ht="18" customHeight="1" s="52">
+      <c r="B2" s="51" t="inlineStr">
         <is>
           <t>Abu Dhabi Marathon 2026 — Training Plan</t>
         </is>
@@ -821,7 +821,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16" customHeight="1" s="46">
+    <row r="9" ht="16" customHeight="1" s="52">
       <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Days to race</t>
@@ -844,7 +844,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="47" t="inlineStr">
+      <c r="B12" s="53" t="inlineStr">
         <is>
           <t>Pace zones (CALIBRATED after Wk1 5K time trial 24 Jul 2026: 5 km in 23:20 @ 4:40/km, RPE 7. Conservative interpretation. Recheck at the Wk13 half-marathon time trial on Sat 17 Oct.)</t>
         </is>
@@ -964,7 +964,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="29" customHeight="1" s="46">
+    <row r="21" ht="29" customHeight="1" s="52">
       <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Base building</t>
@@ -986,7 +986,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="29" customHeight="1" s="46">
+    <row r="22" ht="29" customHeight="1" s="52">
       <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Aerobic build</t>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="29" customHeight="1" s="46">
+    <row r="23" ht="29" customHeight="1" s="52">
       <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Peak</t>
@@ -1053,14 +1053,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="49" t="inlineStr">
+      <c r="B26" s="55" t="inlineStr">
         <is>
           <t>Deload weeks: 5, 10, 14 (volume cut ~20-25%). Checkpoints: Wk1 baseline 5K, Wk13 half-marathon time trial.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="48" t="inlineStr">
+      <c r="B28" s="54" t="inlineStr">
         <is>
           <t>Yellow cells are yours to edit (pace zones as you calibrate them). Everything else on this sheet is a formula or fixed reference.</t>
         </is>
@@ -1086,25 +1086,25 @@
   <dimension ref="A1:R199"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="46" min="1" max="1"/>
-    <col width="14" customWidth="1" style="46" min="2" max="2"/>
-    <col width="8" customWidth="1" style="46" min="3" max="3"/>
-    <col width="12" customWidth="1" style="46" min="4" max="4"/>
-    <col width="10" customWidth="1" style="46" min="5" max="5"/>
-    <col width="11" customWidth="1" style="46" min="6" max="6"/>
-    <col width="18" customWidth="1" style="46" min="7" max="7"/>
-    <col width="10" customWidth="1" style="46" min="8" max="8"/>
-    <col width="14" customWidth="1" style="46" min="9" max="9"/>
-    <col width="30" customWidth="1" style="46" min="10" max="10"/>
-    <col width="24" customWidth="1" style="46" min="11" max="11"/>
-    <col width="12" customWidth="1" style="46" min="12" max="13"/>
-    <col width="11.6640625" bestFit="1" customWidth="1" style="59" min="14" max="14"/>
-    <col width="13.1640625" bestFit="1" customWidth="1" style="46" min="15" max="15"/>
-    <col width="9" customWidth="1" style="46" min="16" max="16"/>
-    <col width="24" customWidth="1" style="46" min="17" max="17"/>
+    <col width="6" customWidth="1" style="52" min="1" max="1"/>
+    <col width="14" customWidth="1" style="52" min="2" max="2"/>
+    <col width="8" customWidth="1" style="52" min="3" max="3"/>
+    <col width="12" customWidth="1" style="52" min="4" max="4"/>
+    <col width="10" customWidth="1" style="52" min="5" max="5"/>
+    <col width="11" customWidth="1" style="52" min="6" max="6"/>
+    <col width="18" customWidth="1" style="52" min="7" max="7"/>
+    <col width="10" customWidth="1" style="52" min="8" max="8"/>
+    <col width="14" customWidth="1" style="52" min="9" max="9"/>
+    <col width="30" customWidth="1" style="52" min="10" max="10"/>
+    <col width="24" customWidth="1" style="52" min="11" max="11"/>
+    <col width="12" customWidth="1" style="52" min="12" max="13"/>
+    <col width="11.6640625" bestFit="1" customWidth="1" style="49" min="14" max="14"/>
+    <col width="13.1640625" bestFit="1" customWidth="1" style="52" min="15" max="15"/>
+    <col width="9" customWidth="1" style="52" min="16" max="16"/>
+    <col width="24" customWidth="1" style="52" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1" s="46">
+    <row r="1" ht="42" customHeight="1" s="52">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Week</t>
@@ -1170,7 +1170,7 @@
           <t>Actual (km)</t>
         </is>
       </c>
-      <c r="N1" s="56" t="inlineStr">
+      <c r="N1" s="46" t="inlineStr">
         <is>
           <t>Actual Duration (h:mm:ss)</t>
         </is>
@@ -1254,7 +1254,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N2" s="57" t="inlineStr">
+      <c r="N2" s="47" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1332,12 +1332,12 @@
       <c r="M3" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="N3" s="57" t="inlineStr">
+      <c r="N3" s="47" t="inlineStr">
         <is>
           <t>0:24:00</t>
         </is>
       </c>
-      <c r="O3" s="55" t="n">
+      <c r="O3" s="45" t="n">
         <v>0.25</v>
       </c>
       <c r="P3" s="15" t="n">
@@ -1408,12 +1408,12 @@
       <c r="M4" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="N4" s="57" t="inlineStr">
+      <c r="N4" s="47" t="inlineStr">
         <is>
           <t>0:24:00</t>
         </is>
       </c>
-      <c r="O4" s="55" t="n">
+      <c r="O4" s="45" t="n">
         <v>0.25</v>
       </c>
       <c r="P4" s="15" t="n">
@@ -1488,12 +1488,12 @@
       <c r="M5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="N5" s="57" t="inlineStr">
+      <c r="N5" s="47" t="inlineStr">
         <is>
           <t>0:23:20</t>
         </is>
       </c>
-      <c r="O5" s="55" t="n">
+      <c r="O5" s="45" t="n">
         <v>0.003240740740740741</v>
       </c>
       <c r="P5" s="15" t="n">
@@ -1554,9 +1554,13 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L6" s="15" t="n"/>
+      <c r="L6" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M6" s="15" t="n"/>
-      <c r="N6" s="57" t="n"/>
+      <c r="N6" s="47" t="n"/>
       <c r="O6" s="15" t="n"/>
       <c r="P6" s="15" t="n"/>
       <c r="Q6" s="15" t="n"/>
@@ -1612,13 +1616,35 @@
           <t>Long run - easy</t>
         </is>
       </c>
-      <c r="L7" s="15" t="n"/>
-      <c r="M7" s="15" t="n"/>
-      <c r="N7" s="57" t="n"/>
-      <c r="O7" s="15" t="n"/>
-      <c r="P7" s="15" t="n"/>
-      <c r="Q7" s="15" t="n"/>
-      <c r="R7" s="15" t="n"/>
+      <c r="L7" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="N7" s="47" t="inlineStr">
+        <is>
+          <t>4:00:00</t>
+        </is>
+      </c>
+      <c r="O7" s="45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P7" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="15" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="R7" s="15" t="inlineStr">
+        <is>
+          <t>Walked while playing Golf</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="n">
@@ -1668,12 +1694,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L8" s="15" t="n"/>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M8" s="15" t="n"/>
-      <c r="N8" s="57" t="n"/>
+      <c r="N8" s="47" t="n"/>
       <c r="O8" s="15" t="n"/>
       <c r="P8" s="15" t="n"/>
-      <c r="Q8" s="15" t="n"/>
+      <c r="Q8" s="15" t="inlineStr">
+        <is>
+          <t>Great</t>
+        </is>
+      </c>
       <c r="R8" s="15" t="n"/>
     </row>
     <row r="9">
@@ -1726,7 +1760,7 @@
       </c>
       <c r="L9" s="15" t="n"/>
       <c r="M9" s="15" t="n"/>
-      <c r="N9" s="57" t="n"/>
+      <c r="N9" s="47" t="n"/>
       <c r="O9" s="15" t="n"/>
       <c r="P9" s="15" t="n"/>
       <c r="Q9" s="15" t="n"/>
@@ -1782,13 +1816,21 @@
           <t>Easy run</t>
         </is>
       </c>
-      <c r="L10" s="15" t="n"/>
+      <c r="L10" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M10" s="15" t="n"/>
-      <c r="N10" s="57" t="n"/>
+      <c r="N10" s="47" t="n"/>
       <c r="O10" s="15" t="n"/>
       <c r="P10" s="15" t="n"/>
       <c r="Q10" s="15" t="n"/>
-      <c r="R10" s="15" t="n"/>
+      <c r="R10" s="15" t="inlineStr">
+        <is>
+          <t>Replaced by football game</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="n">
@@ -1842,7 +1884,7 @@
       </c>
       <c r="L11" s="15" t="n"/>
       <c r="M11" s="15" t="n"/>
-      <c r="N11" s="57" t="n"/>
+      <c r="N11" s="47" t="n"/>
       <c r="O11" s="15" t="n"/>
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="15" t="n"/>
@@ -1898,7 +1940,7 @@
       </c>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
-      <c r="N12" s="57" t="n"/>
+      <c r="N12" s="47" t="n"/>
       <c r="O12" s="15" t="n"/>
       <c r="P12" s="15" t="n"/>
       <c r="Q12" s="15" t="n"/>
@@ -1956,7 +1998,7 @@
       </c>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
-      <c r="N13" s="57" t="n"/>
+      <c r="N13" s="47" t="n"/>
       <c r="O13" s="15" t="n"/>
       <c r="P13" s="15" t="n"/>
       <c r="Q13" s="15" t="n"/>
@@ -2014,7 +2056,7 @@
       </c>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
-      <c r="N14" s="57" t="n"/>
+      <c r="N14" s="47" t="n"/>
       <c r="O14" s="15" t="n"/>
       <c r="P14" s="15" t="n"/>
       <c r="Q14" s="15" t="n"/>
@@ -2070,7 +2112,7 @@
       </c>
       <c r="L15" s="15" t="n"/>
       <c r="M15" s="15" t="n"/>
-      <c r="N15" s="57" t="n"/>
+      <c r="N15" s="47" t="n"/>
       <c r="O15" s="15" t="n"/>
       <c r="P15" s="15" t="n"/>
       <c r="Q15" s="15" t="n"/>
@@ -2128,7 +2170,7 @@
       </c>
       <c r="L16" s="15" t="n"/>
       <c r="M16" s="15" t="n"/>
-      <c r="N16" s="57" t="n"/>
+      <c r="N16" s="47" t="n"/>
       <c r="O16" s="15" t="n"/>
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
@@ -2184,7 +2226,7 @@
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
-      <c r="N17" s="57" t="n"/>
+      <c r="N17" s="47" t="n"/>
       <c r="O17" s="15" t="n"/>
       <c r="P17" s="15" t="n"/>
       <c r="Q17" s="15" t="n"/>
@@ -2240,7 +2282,7 @@
       </c>
       <c r="L18" s="15" t="n"/>
       <c r="M18" s="15" t="n"/>
-      <c r="N18" s="57" t="n"/>
+      <c r="N18" s="47" t="n"/>
       <c r="O18" s="15" t="n"/>
       <c r="P18" s="15" t="n"/>
       <c r="Q18" s="15" t="n"/>
@@ -2298,7 +2340,7 @@
       </c>
       <c r="L19" s="15" t="n"/>
       <c r="M19" s="15" t="n"/>
-      <c r="N19" s="57" t="n"/>
+      <c r="N19" s="47" t="n"/>
       <c r="O19" s="15" t="n"/>
       <c r="P19" s="15" t="n"/>
       <c r="Q19" s="15" t="n"/>
@@ -2356,7 +2398,7 @@
       </c>
       <c r="L20" s="15" t="n"/>
       <c r="M20" s="15" t="n"/>
-      <c r="N20" s="57" t="n"/>
+      <c r="N20" s="47" t="n"/>
       <c r="O20" s="15" t="n"/>
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="15" t="n"/>
@@ -2412,7 +2454,7 @@
       </c>
       <c r="L21" s="15" t="n"/>
       <c r="M21" s="15" t="n"/>
-      <c r="N21" s="57" t="n"/>
+      <c r="N21" s="47" t="n"/>
       <c r="O21" s="15" t="n"/>
       <c r="P21" s="15" t="n"/>
       <c r="Q21" s="15" t="n"/>
@@ -2470,7 +2512,7 @@
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>
-      <c r="N22" s="57" t="n"/>
+      <c r="N22" s="47" t="n"/>
       <c r="O22" s="15" t="n"/>
       <c r="P22" s="15" t="n"/>
       <c r="Q22" s="15" t="n"/>
@@ -2528,7 +2570,7 @@
       </c>
       <c r="L23" s="15" t="n"/>
       <c r="M23" s="15" t="n"/>
-      <c r="N23" s="57" t="n"/>
+      <c r="N23" s="47" t="n"/>
       <c r="O23" s="15" t="n"/>
       <c r="P23" s="15" t="n"/>
       <c r="Q23" s="15" t="n"/>
@@ -2584,7 +2626,7 @@
       </c>
       <c r="L24" s="15" t="n"/>
       <c r="M24" s="15" t="n"/>
-      <c r="N24" s="57" t="n"/>
+      <c r="N24" s="47" t="n"/>
       <c r="O24" s="15" t="n"/>
       <c r="P24" s="15" t="n"/>
       <c r="Q24" s="15" t="n"/>
@@ -2642,7 +2684,7 @@
       </c>
       <c r="L25" s="15" t="n"/>
       <c r="M25" s="15" t="n"/>
-      <c r="N25" s="57" t="n"/>
+      <c r="N25" s="47" t="n"/>
       <c r="O25" s="15" t="n"/>
       <c r="P25" s="15" t="n"/>
       <c r="Q25" s="15" t="n"/>
@@ -2698,7 +2740,7 @@
       </c>
       <c r="L26" s="15" t="n"/>
       <c r="M26" s="15" t="n"/>
-      <c r="N26" s="57" t="n"/>
+      <c r="N26" s="47" t="n"/>
       <c r="O26" s="15" t="n"/>
       <c r="P26" s="15" t="n"/>
       <c r="Q26" s="15" t="n"/>
@@ -2754,7 +2796,7 @@
       </c>
       <c r="L27" s="15" t="n"/>
       <c r="M27" s="15" t="n"/>
-      <c r="N27" s="57" t="n"/>
+      <c r="N27" s="47" t="n"/>
       <c r="O27" s="15" t="n"/>
       <c r="P27" s="15" t="n"/>
       <c r="Q27" s="15" t="n"/>
@@ -2812,7 +2854,7 @@
       </c>
       <c r="L28" s="15" t="n"/>
       <c r="M28" s="15" t="n"/>
-      <c r="N28" s="57" t="n"/>
+      <c r="N28" s="47" t="n"/>
       <c r="O28" s="15" t="n"/>
       <c r="P28" s="15" t="n"/>
       <c r="Q28" s="15" t="n"/>
@@ -2870,7 +2912,7 @@
       </c>
       <c r="L29" s="15" t="n"/>
       <c r="M29" s="15" t="n"/>
-      <c r="N29" s="57" t="n"/>
+      <c r="N29" s="47" t="n"/>
       <c r="O29" s="15" t="n"/>
       <c r="P29" s="15" t="n"/>
       <c r="Q29" s="15" t="n"/>
@@ -2926,7 +2968,7 @@
       </c>
       <c r="L30" s="15" t="n"/>
       <c r="M30" s="15" t="n"/>
-      <c r="N30" s="57" t="n"/>
+      <c r="N30" s="47" t="n"/>
       <c r="O30" s="15" t="n"/>
       <c r="P30" s="15" t="n"/>
       <c r="Q30" s="15" t="n"/>
@@ -2984,7 +3026,7 @@
       </c>
       <c r="L31" s="15" t="n"/>
       <c r="M31" s="15" t="n"/>
-      <c r="N31" s="57" t="n"/>
+      <c r="N31" s="47" t="n"/>
       <c r="O31" s="15" t="n"/>
       <c r="P31" s="15" t="n"/>
       <c r="Q31" s="15" t="n"/>
@@ -3042,7 +3084,7 @@
       </c>
       <c r="L32" s="15" t="n"/>
       <c r="M32" s="15" t="n"/>
-      <c r="N32" s="57" t="n"/>
+      <c r="N32" s="47" t="n"/>
       <c r="O32" s="15" t="n"/>
       <c r="P32" s="15" t="n"/>
       <c r="Q32" s="15" t="n"/>
@@ -3098,7 +3140,7 @@
       </c>
       <c r="L33" s="15" t="n"/>
       <c r="M33" s="15" t="n"/>
-      <c r="N33" s="57" t="n"/>
+      <c r="N33" s="47" t="n"/>
       <c r="O33" s="15" t="n"/>
       <c r="P33" s="15" t="n"/>
       <c r="Q33" s="15" t="n"/>
@@ -3156,7 +3198,7 @@
       </c>
       <c r="L34" s="15" t="n"/>
       <c r="M34" s="15" t="n"/>
-      <c r="N34" s="57" t="n"/>
+      <c r="N34" s="47" t="n"/>
       <c r="O34" s="15" t="n"/>
       <c r="P34" s="15" t="n"/>
       <c r="Q34" s="15" t="n"/>
@@ -3212,7 +3254,7 @@
       </c>
       <c r="L35" s="20" t="n"/>
       <c r="M35" s="20" t="n"/>
-      <c r="N35" s="58" t="n"/>
+      <c r="N35" s="48" t="n"/>
       <c r="O35" s="20" t="n"/>
       <c r="P35" s="20" t="n"/>
       <c r="Q35" s="20" t="n"/>
@@ -3268,7 +3310,7 @@
       </c>
       <c r="L36" s="20" t="n"/>
       <c r="M36" s="20" t="n"/>
-      <c r="N36" s="58" t="n"/>
+      <c r="N36" s="48" t="n"/>
       <c r="O36" s="20" t="n"/>
       <c r="P36" s="20" t="n"/>
       <c r="Q36" s="20" t="n"/>
@@ -3326,7 +3368,7 @@
       </c>
       <c r="L37" s="20" t="n"/>
       <c r="M37" s="20" t="n"/>
-      <c r="N37" s="58" t="n"/>
+      <c r="N37" s="48" t="n"/>
       <c r="O37" s="20" t="n"/>
       <c r="P37" s="20" t="n"/>
       <c r="Q37" s="20" t="n"/>
@@ -3384,7 +3426,7 @@
       </c>
       <c r="L38" s="20" t="n"/>
       <c r="M38" s="20" t="n"/>
-      <c r="N38" s="58" t="n"/>
+      <c r="N38" s="48" t="n"/>
       <c r="O38" s="20" t="n"/>
       <c r="P38" s="20" t="n"/>
       <c r="Q38" s="20" t="n"/>
@@ -3440,7 +3482,7 @@
       </c>
       <c r="L39" s="20" t="n"/>
       <c r="M39" s="20" t="n"/>
-      <c r="N39" s="58" t="n"/>
+      <c r="N39" s="48" t="n"/>
       <c r="O39" s="20" t="n"/>
       <c r="P39" s="20" t="n"/>
       <c r="Q39" s="20" t="n"/>
@@ -3498,7 +3540,7 @@
       </c>
       <c r="L40" s="20" t="n"/>
       <c r="M40" s="20" t="n"/>
-      <c r="N40" s="58" t="n"/>
+      <c r="N40" s="48" t="n"/>
       <c r="O40" s="20" t="n"/>
       <c r="P40" s="20" t="n"/>
       <c r="Q40" s="20" t="n"/>
@@ -3556,7 +3598,7 @@
       </c>
       <c r="L41" s="20" t="n"/>
       <c r="M41" s="20" t="n"/>
-      <c r="N41" s="58" t="n"/>
+      <c r="N41" s="48" t="n"/>
       <c r="O41" s="20" t="n"/>
       <c r="P41" s="20" t="n"/>
       <c r="Q41" s="20" t="n"/>
@@ -3612,7 +3654,7 @@
       </c>
       <c r="L42" s="20" t="n"/>
       <c r="M42" s="20" t="n"/>
-      <c r="N42" s="58" t="n"/>
+      <c r="N42" s="48" t="n"/>
       <c r="O42" s="20" t="n"/>
       <c r="P42" s="20" t="n"/>
       <c r="Q42" s="20" t="n"/>
@@ -3670,7 +3712,7 @@
       </c>
       <c r="L43" s="20" t="n"/>
       <c r="M43" s="20" t="n"/>
-      <c r="N43" s="58" t="n"/>
+      <c r="N43" s="48" t="n"/>
       <c r="O43" s="20" t="n"/>
       <c r="P43" s="20" t="n"/>
       <c r="Q43" s="20" t="n"/>
@@ -3726,7 +3768,7 @@
       </c>
       <c r="L44" s="15" t="n"/>
       <c r="M44" s="15" t="n"/>
-      <c r="N44" s="57" t="n"/>
+      <c r="N44" s="47" t="n"/>
       <c r="O44" s="15" t="n"/>
       <c r="P44" s="15" t="n"/>
       <c r="Q44" s="15" t="n"/>
@@ -3782,7 +3824,7 @@
       </c>
       <c r="L45" s="15" t="n"/>
       <c r="M45" s="15" t="n"/>
-      <c r="N45" s="57" t="n"/>
+      <c r="N45" s="47" t="n"/>
       <c r="O45" s="15" t="n"/>
       <c r="P45" s="15" t="n"/>
       <c r="Q45" s="15" t="n"/>
@@ -3840,7 +3882,7 @@
       </c>
       <c r="L46" s="15" t="n"/>
       <c r="M46" s="15" t="n"/>
-      <c r="N46" s="57" t="n"/>
+      <c r="N46" s="47" t="n"/>
       <c r="O46" s="15" t="n"/>
       <c r="P46" s="15" t="n"/>
       <c r="Q46" s="15" t="n"/>
@@ -3898,7 +3940,7 @@
       </c>
       <c r="L47" s="15" t="n"/>
       <c r="M47" s="15" t="n"/>
-      <c r="N47" s="57" t="n"/>
+      <c r="N47" s="47" t="n"/>
       <c r="O47" s="15" t="n"/>
       <c r="P47" s="15" t="n"/>
       <c r="Q47" s="15" t="n"/>
@@ -3954,7 +3996,7 @@
       </c>
       <c r="L48" s="15" t="n"/>
       <c r="M48" s="15" t="n"/>
-      <c r="N48" s="57" t="n"/>
+      <c r="N48" s="47" t="n"/>
       <c r="O48" s="15" t="n"/>
       <c r="P48" s="15" t="n"/>
       <c r="Q48" s="15" t="n"/>
@@ -4012,7 +4054,7 @@
       </c>
       <c r="L49" s="15" t="n"/>
       <c r="M49" s="15" t="n"/>
-      <c r="N49" s="57" t="n"/>
+      <c r="N49" s="47" t="n"/>
       <c r="O49" s="15" t="n"/>
       <c r="P49" s="15" t="n"/>
       <c r="Q49" s="15" t="n"/>
@@ -4070,7 +4112,7 @@
       </c>
       <c r="L50" s="15" t="n"/>
       <c r="M50" s="15" t="n"/>
-      <c r="N50" s="57" t="n"/>
+      <c r="N50" s="47" t="n"/>
       <c r="O50" s="15" t="n"/>
       <c r="P50" s="15" t="n"/>
       <c r="Q50" s="15" t="n"/>
@@ -4126,7 +4168,7 @@
       </c>
       <c r="L51" s="15" t="n"/>
       <c r="M51" s="15" t="n"/>
-      <c r="N51" s="57" t="n"/>
+      <c r="N51" s="47" t="n"/>
       <c r="O51" s="15" t="n"/>
       <c r="P51" s="15" t="n"/>
       <c r="Q51" s="15" t="n"/>
@@ -4184,7 +4226,7 @@
       </c>
       <c r="L52" s="15" t="n"/>
       <c r="M52" s="15" t="n"/>
-      <c r="N52" s="57" t="n"/>
+      <c r="N52" s="47" t="n"/>
       <c r="O52" s="15" t="n"/>
       <c r="P52" s="15" t="n"/>
       <c r="Q52" s="15" t="n"/>
@@ -4240,7 +4282,7 @@
       </c>
       <c r="L53" s="15" t="n"/>
       <c r="M53" s="15" t="n"/>
-      <c r="N53" s="57" t="n"/>
+      <c r="N53" s="47" t="n"/>
       <c r="O53" s="15" t="n"/>
       <c r="P53" s="15" t="n"/>
       <c r="Q53" s="15" t="n"/>
@@ -4296,7 +4338,7 @@
       </c>
       <c r="L54" s="15" t="n"/>
       <c r="M54" s="15" t="n"/>
-      <c r="N54" s="57" t="n"/>
+      <c r="N54" s="47" t="n"/>
       <c r="O54" s="15" t="n"/>
       <c r="P54" s="15" t="n"/>
       <c r="Q54" s="15" t="n"/>
@@ -4354,7 +4396,7 @@
       </c>
       <c r="L55" s="15" t="n"/>
       <c r="M55" s="15" t="n"/>
-      <c r="N55" s="57" t="n"/>
+      <c r="N55" s="47" t="n"/>
       <c r="O55" s="15" t="n"/>
       <c r="P55" s="15" t="n"/>
       <c r="Q55" s="15" t="n"/>
@@ -4412,7 +4454,7 @@
       </c>
       <c r="L56" s="15" t="n"/>
       <c r="M56" s="15" t="n"/>
-      <c r="N56" s="57" t="n"/>
+      <c r="N56" s="47" t="n"/>
       <c r="O56" s="15" t="n"/>
       <c r="P56" s="15" t="n"/>
       <c r="Q56" s="15" t="n"/>
@@ -4468,7 +4510,7 @@
       </c>
       <c r="L57" s="15" t="n"/>
       <c r="M57" s="15" t="n"/>
-      <c r="N57" s="57" t="n"/>
+      <c r="N57" s="47" t="n"/>
       <c r="O57" s="15" t="n"/>
       <c r="P57" s="15" t="n"/>
       <c r="Q57" s="15" t="n"/>
@@ -4526,7 +4568,7 @@
       </c>
       <c r="L58" s="15" t="n"/>
       <c r="M58" s="15" t="n"/>
-      <c r="N58" s="57" t="n"/>
+      <c r="N58" s="47" t="n"/>
       <c r="O58" s="15" t="n"/>
       <c r="P58" s="15" t="n"/>
       <c r="Q58" s="15" t="n"/>
@@ -4584,7 +4626,7 @@
       </c>
       <c r="L59" s="15" t="n"/>
       <c r="M59" s="15" t="n"/>
-      <c r="N59" s="57" t="n"/>
+      <c r="N59" s="47" t="n"/>
       <c r="O59" s="15" t="n"/>
       <c r="P59" s="15" t="n"/>
       <c r="Q59" s="15" t="n"/>
@@ -4640,7 +4682,7 @@
       </c>
       <c r="L60" s="15" t="n"/>
       <c r="M60" s="15" t="n"/>
-      <c r="N60" s="57" t="n"/>
+      <c r="N60" s="47" t="n"/>
       <c r="O60" s="15" t="n"/>
       <c r="P60" s="15" t="n"/>
       <c r="Q60" s="15" t="n"/>
@@ -4698,7 +4740,7 @@
       </c>
       <c r="L61" s="15" t="n"/>
       <c r="M61" s="15" t="n"/>
-      <c r="N61" s="57" t="n"/>
+      <c r="N61" s="47" t="n"/>
       <c r="O61" s="15" t="n"/>
       <c r="P61" s="15" t="n"/>
       <c r="Q61" s="15" t="n"/>
@@ -4754,7 +4796,7 @@
       </c>
       <c r="L62" s="15" t="n"/>
       <c r="M62" s="15" t="n"/>
-      <c r="N62" s="57" t="n"/>
+      <c r="N62" s="47" t="n"/>
       <c r="O62" s="15" t="n"/>
       <c r="P62" s="15" t="n"/>
       <c r="Q62" s="15" t="n"/>
@@ -4810,7 +4852,7 @@
       </c>
       <c r="L63" s="15" t="n"/>
       <c r="M63" s="15" t="n"/>
-      <c r="N63" s="57" t="n"/>
+      <c r="N63" s="47" t="n"/>
       <c r="O63" s="15" t="n"/>
       <c r="P63" s="15" t="n"/>
       <c r="Q63" s="15" t="n"/>
@@ -4868,7 +4910,7 @@
       </c>
       <c r="L64" s="15" t="n"/>
       <c r="M64" s="15" t="n"/>
-      <c r="N64" s="57" t="n"/>
+      <c r="N64" s="47" t="n"/>
       <c r="O64" s="15" t="n"/>
       <c r="P64" s="15" t="n"/>
       <c r="Q64" s="15" t="n"/>
@@ -4926,7 +4968,7 @@
       </c>
       <c r="L65" s="15" t="n"/>
       <c r="M65" s="15" t="n"/>
-      <c r="N65" s="57" t="n"/>
+      <c r="N65" s="47" t="n"/>
       <c r="O65" s="15" t="n"/>
       <c r="P65" s="15" t="n"/>
       <c r="Q65" s="15" t="n"/>
@@ -4982,7 +5024,7 @@
       </c>
       <c r="L66" s="15" t="n"/>
       <c r="M66" s="15" t="n"/>
-      <c r="N66" s="57" t="n"/>
+      <c r="N66" s="47" t="n"/>
       <c r="O66" s="15" t="n"/>
       <c r="P66" s="15" t="n"/>
       <c r="Q66" s="15" t="n"/>
@@ -5040,7 +5082,7 @@
       </c>
       <c r="L67" s="15" t="n"/>
       <c r="M67" s="15" t="n"/>
-      <c r="N67" s="57" t="n"/>
+      <c r="N67" s="47" t="n"/>
       <c r="O67" s="15" t="n"/>
       <c r="P67" s="15" t="n"/>
       <c r="Q67" s="15" t="n"/>
@@ -5098,7 +5140,7 @@
       </c>
       <c r="L68" s="15" t="n"/>
       <c r="M68" s="15" t="n"/>
-      <c r="N68" s="57" t="n"/>
+      <c r="N68" s="47" t="n"/>
       <c r="O68" s="15" t="n"/>
       <c r="P68" s="15" t="n"/>
       <c r="Q68" s="15" t="n"/>
@@ -5154,7 +5196,7 @@
       </c>
       <c r="L69" s="15" t="n"/>
       <c r="M69" s="15" t="n"/>
-      <c r="N69" s="57" t="n"/>
+      <c r="N69" s="47" t="n"/>
       <c r="O69" s="15" t="n"/>
       <c r="P69" s="15" t="n"/>
       <c r="Q69" s="15" t="n"/>
@@ -5212,7 +5254,7 @@
       </c>
       <c r="L70" s="15" t="n"/>
       <c r="M70" s="15" t="n"/>
-      <c r="N70" s="57" t="n"/>
+      <c r="N70" s="47" t="n"/>
       <c r="O70" s="15" t="n"/>
       <c r="P70" s="15" t="n"/>
       <c r="Q70" s="15" t="n"/>
@@ -5270,7 +5312,7 @@
       </c>
       <c r="L71" s="15" t="n"/>
       <c r="M71" s="15" t="n"/>
-      <c r="N71" s="57" t="n"/>
+      <c r="N71" s="47" t="n"/>
       <c r="O71" s="15" t="n"/>
       <c r="P71" s="15" t="n"/>
       <c r="Q71" s="15" t="n"/>
@@ -5326,7 +5368,7 @@
       </c>
       <c r="L72" s="15" t="n"/>
       <c r="M72" s="15" t="n"/>
-      <c r="N72" s="57" t="n"/>
+      <c r="N72" s="47" t="n"/>
       <c r="O72" s="15" t="n"/>
       <c r="P72" s="15" t="n"/>
       <c r="Q72" s="15" t="n"/>
@@ -5382,7 +5424,7 @@
       </c>
       <c r="L73" s="15" t="n"/>
       <c r="M73" s="15" t="n"/>
-      <c r="N73" s="57" t="n"/>
+      <c r="N73" s="47" t="n"/>
       <c r="O73" s="15" t="n"/>
       <c r="P73" s="15" t="n"/>
       <c r="Q73" s="15" t="n"/>
@@ -5440,7 +5482,7 @@
       </c>
       <c r="L74" s="15" t="n"/>
       <c r="M74" s="15" t="n"/>
-      <c r="N74" s="57" t="n"/>
+      <c r="N74" s="47" t="n"/>
       <c r="O74" s="15" t="n"/>
       <c r="P74" s="15" t="n"/>
       <c r="Q74" s="15" t="n"/>
@@ -5498,7 +5540,7 @@
       </c>
       <c r="L75" s="15" t="n"/>
       <c r="M75" s="15" t="n"/>
-      <c r="N75" s="57" t="n"/>
+      <c r="N75" s="47" t="n"/>
       <c r="O75" s="15" t="n"/>
       <c r="P75" s="15" t="n"/>
       <c r="Q75" s="15" t="n"/>
@@ -5554,7 +5596,7 @@
       </c>
       <c r="L76" s="15" t="n"/>
       <c r="M76" s="15" t="n"/>
-      <c r="N76" s="57" t="n"/>
+      <c r="N76" s="47" t="n"/>
       <c r="O76" s="15" t="n"/>
       <c r="P76" s="15" t="n"/>
       <c r="Q76" s="15" t="n"/>
@@ -5612,7 +5654,7 @@
       </c>
       <c r="L77" s="15" t="n"/>
       <c r="M77" s="15" t="n"/>
-      <c r="N77" s="57" t="n"/>
+      <c r="N77" s="47" t="n"/>
       <c r="O77" s="15" t="n"/>
       <c r="P77" s="15" t="n"/>
       <c r="Q77" s="15" t="n"/>
@@ -5670,7 +5712,7 @@
       </c>
       <c r="L78" s="15" t="n"/>
       <c r="M78" s="15" t="n"/>
-      <c r="N78" s="57" t="n"/>
+      <c r="N78" s="47" t="n"/>
       <c r="O78" s="15" t="n"/>
       <c r="P78" s="15" t="n"/>
       <c r="Q78" s="15" t="n"/>
@@ -5726,7 +5768,7 @@
       </c>
       <c r="L79" s="15" t="n"/>
       <c r="M79" s="15" t="n"/>
-      <c r="N79" s="57" t="n"/>
+      <c r="N79" s="47" t="n"/>
       <c r="O79" s="15" t="n"/>
       <c r="P79" s="15" t="n"/>
       <c r="Q79" s="15" t="n"/>
@@ -5784,7 +5826,7 @@
       </c>
       <c r="L80" s="15" t="n"/>
       <c r="M80" s="15" t="n"/>
-      <c r="N80" s="57" t="n"/>
+      <c r="N80" s="47" t="n"/>
       <c r="O80" s="15" t="n"/>
       <c r="P80" s="15" t="n"/>
       <c r="Q80" s="15" t="n"/>
@@ -5842,7 +5884,7 @@
       </c>
       <c r="L81" s="15" t="n"/>
       <c r="M81" s="15" t="n"/>
-      <c r="N81" s="57" t="n"/>
+      <c r="N81" s="47" t="n"/>
       <c r="O81" s="15" t="n"/>
       <c r="P81" s="15" t="n"/>
       <c r="Q81" s="15" t="n"/>
@@ -5898,7 +5940,7 @@
       </c>
       <c r="L82" s="20" t="n"/>
       <c r="M82" s="20" t="n"/>
-      <c r="N82" s="58" t="n"/>
+      <c r="N82" s="48" t="n"/>
       <c r="O82" s="20" t="n"/>
       <c r="P82" s="20" t="n"/>
       <c r="Q82" s="20" t="n"/>
@@ -5954,7 +5996,7 @@
       </c>
       <c r="L83" s="20" t="n"/>
       <c r="M83" s="20" t="n"/>
-      <c r="N83" s="58" t="n"/>
+      <c r="N83" s="48" t="n"/>
       <c r="O83" s="20" t="n"/>
       <c r="P83" s="20" t="n"/>
       <c r="Q83" s="20" t="n"/>
@@ -6012,7 +6054,7 @@
       </c>
       <c r="L84" s="20" t="n"/>
       <c r="M84" s="20" t="n"/>
-      <c r="N84" s="58" t="n"/>
+      <c r="N84" s="48" t="n"/>
       <c r="O84" s="20" t="n"/>
       <c r="P84" s="20" t="n"/>
       <c r="Q84" s="20" t="n"/>
@@ -6070,7 +6112,7 @@
       </c>
       <c r="L85" s="20" t="n"/>
       <c r="M85" s="20" t="n"/>
-      <c r="N85" s="58" t="n"/>
+      <c r="N85" s="48" t="n"/>
       <c r="O85" s="20" t="n"/>
       <c r="P85" s="20" t="n"/>
       <c r="Q85" s="20" t="n"/>
@@ -6126,7 +6168,7 @@
       </c>
       <c r="L86" s="20" t="n"/>
       <c r="M86" s="20" t="n"/>
-      <c r="N86" s="58" t="n"/>
+      <c r="N86" s="48" t="n"/>
       <c r="O86" s="20" t="n"/>
       <c r="P86" s="20" t="n"/>
       <c r="Q86" s="20" t="n"/>
@@ -6184,7 +6226,7 @@
       </c>
       <c r="L87" s="20" t="n"/>
       <c r="M87" s="20" t="n"/>
-      <c r="N87" s="58" t="n"/>
+      <c r="N87" s="48" t="n"/>
       <c r="O87" s="20" t="n"/>
       <c r="P87" s="20" t="n"/>
       <c r="Q87" s="20" t="n"/>
@@ -6242,7 +6284,7 @@
       </c>
       <c r="L88" s="20" t="n"/>
       <c r="M88" s="20" t="n"/>
-      <c r="N88" s="58" t="n"/>
+      <c r="N88" s="48" t="n"/>
       <c r="O88" s="20" t="n"/>
       <c r="P88" s="20" t="n"/>
       <c r="Q88" s="20" t="n"/>
@@ -6298,7 +6340,7 @@
       </c>
       <c r="L89" s="20" t="n"/>
       <c r="M89" s="20" t="n"/>
-      <c r="N89" s="58" t="n"/>
+      <c r="N89" s="48" t="n"/>
       <c r="O89" s="20" t="n"/>
       <c r="P89" s="20" t="n"/>
       <c r="Q89" s="20" t="n"/>
@@ -6356,7 +6398,7 @@
       </c>
       <c r="L90" s="20" t="n"/>
       <c r="M90" s="20" t="n"/>
-      <c r="N90" s="58" t="n"/>
+      <c r="N90" s="48" t="n"/>
       <c r="O90" s="20" t="n"/>
       <c r="P90" s="20" t="n"/>
       <c r="Q90" s="20" t="n"/>
@@ -6414,7 +6456,7 @@
       </c>
       <c r="L91" s="20" t="n"/>
       <c r="M91" s="20" t="n"/>
-      <c r="N91" s="58" t="n"/>
+      <c r="N91" s="48" t="n"/>
       <c r="O91" s="20" t="n"/>
       <c r="P91" s="20" t="n"/>
       <c r="Q91" s="20" t="n"/>
@@ -6470,7 +6512,7 @@
       </c>
       <c r="L92" s="15" t="n"/>
       <c r="M92" s="15" t="n"/>
-      <c r="N92" s="57" t="n"/>
+      <c r="N92" s="47" t="n"/>
       <c r="O92" s="15" t="n"/>
       <c r="P92" s="15" t="n"/>
       <c r="Q92" s="15" t="n"/>
@@ -6526,7 +6568,7 @@
       </c>
       <c r="L93" s="15" t="n"/>
       <c r="M93" s="15" t="n"/>
-      <c r="N93" s="57" t="n"/>
+      <c r="N93" s="47" t="n"/>
       <c r="O93" s="15" t="n"/>
       <c r="P93" s="15" t="n"/>
       <c r="Q93" s="15" t="n"/>
@@ -6584,7 +6626,7 @@
       </c>
       <c r="L94" s="15" t="n"/>
       <c r="M94" s="15" t="n"/>
-      <c r="N94" s="57" t="n"/>
+      <c r="N94" s="47" t="n"/>
       <c r="O94" s="15" t="n"/>
       <c r="P94" s="15" t="n"/>
       <c r="Q94" s="15" t="n"/>
@@ -6642,7 +6684,7 @@
       </c>
       <c r="L95" s="15" t="n"/>
       <c r="M95" s="15" t="n"/>
-      <c r="N95" s="57" t="n"/>
+      <c r="N95" s="47" t="n"/>
       <c r="O95" s="15" t="n"/>
       <c r="P95" s="15" t="n"/>
       <c r="Q95" s="15" t="n"/>
@@ -6698,7 +6740,7 @@
       </c>
       <c r="L96" s="15" t="n"/>
       <c r="M96" s="15" t="n"/>
-      <c r="N96" s="57" t="n"/>
+      <c r="N96" s="47" t="n"/>
       <c r="O96" s="15" t="n"/>
       <c r="P96" s="15" t="n"/>
       <c r="Q96" s="15" t="n"/>
@@ -6756,7 +6798,7 @@
       </c>
       <c r="L97" s="15" t="n"/>
       <c r="M97" s="15" t="n"/>
-      <c r="N97" s="57" t="n"/>
+      <c r="N97" s="47" t="n"/>
       <c r="O97" s="15" t="n"/>
       <c r="P97" s="15" t="n"/>
       <c r="Q97" s="15" t="n"/>
@@ -6814,7 +6856,7 @@
       </c>
       <c r="L98" s="15" t="n"/>
       <c r="M98" s="15" t="n"/>
-      <c r="N98" s="57" t="n"/>
+      <c r="N98" s="47" t="n"/>
       <c r="O98" s="15" t="n"/>
       <c r="P98" s="15" t="n"/>
       <c r="Q98" s="15" t="n"/>
@@ -6870,7 +6912,7 @@
       </c>
       <c r="L99" s="15" t="n"/>
       <c r="M99" s="15" t="n"/>
-      <c r="N99" s="57" t="n"/>
+      <c r="N99" s="47" t="n"/>
       <c r="O99" s="15" t="n"/>
       <c r="P99" s="15" t="n"/>
       <c r="Q99" s="15" t="n"/>
@@ -6928,7 +6970,7 @@
       </c>
       <c r="L100" s="15" t="n"/>
       <c r="M100" s="15" t="n"/>
-      <c r="N100" s="57" t="n"/>
+      <c r="N100" s="47" t="n"/>
       <c r="O100" s="15" t="n"/>
       <c r="P100" s="15" t="n"/>
       <c r="Q100" s="15" t="n"/>
@@ -6986,7 +7028,7 @@
       </c>
       <c r="L101" s="15" t="n"/>
       <c r="M101" s="15" t="n"/>
-      <c r="N101" s="57" t="n"/>
+      <c r="N101" s="47" t="n"/>
       <c r="O101" s="15" t="n"/>
       <c r="P101" s="15" t="n"/>
       <c r="Q101" s="15" t="n"/>
@@ -7042,7 +7084,7 @@
       </c>
       <c r="L102" s="15" t="n"/>
       <c r="M102" s="15" t="n"/>
-      <c r="N102" s="57" t="n"/>
+      <c r="N102" s="47" t="n"/>
       <c r="O102" s="15" t="n"/>
       <c r="P102" s="15" t="n"/>
       <c r="Q102" s="15" t="n"/>
@@ -7098,7 +7140,7 @@
       </c>
       <c r="L103" s="15" t="n"/>
       <c r="M103" s="15" t="n"/>
-      <c r="N103" s="57" t="n"/>
+      <c r="N103" s="47" t="n"/>
       <c r="O103" s="15" t="n"/>
       <c r="P103" s="15" t="n"/>
       <c r="Q103" s="15" t="n"/>
@@ -7156,7 +7198,7 @@
       </c>
       <c r="L104" s="15" t="n"/>
       <c r="M104" s="15" t="n"/>
-      <c r="N104" s="57" t="n"/>
+      <c r="N104" s="47" t="n"/>
       <c r="O104" s="15" t="n"/>
       <c r="P104" s="15" t="n"/>
       <c r="Q104" s="15" t="n"/>
@@ -7214,7 +7256,7 @@
       </c>
       <c r="L105" s="15" t="n"/>
       <c r="M105" s="15" t="n"/>
-      <c r="N105" s="57" t="n"/>
+      <c r="N105" s="47" t="n"/>
       <c r="O105" s="15" t="n"/>
       <c r="P105" s="15" t="n"/>
       <c r="Q105" s="15" t="n"/>
@@ -7270,7 +7312,7 @@
       </c>
       <c r="L106" s="15" t="n"/>
       <c r="M106" s="15" t="n"/>
-      <c r="N106" s="57" t="n"/>
+      <c r="N106" s="47" t="n"/>
       <c r="O106" s="15" t="n"/>
       <c r="P106" s="15" t="n"/>
       <c r="Q106" s="15" t="n"/>
@@ -7328,7 +7370,7 @@
       </c>
       <c r="L107" s="15" t="n"/>
       <c r="M107" s="15" t="n"/>
-      <c r="N107" s="57" t="n"/>
+      <c r="N107" s="47" t="n"/>
       <c r="O107" s="15" t="n"/>
       <c r="P107" s="15" t="n"/>
       <c r="Q107" s="15" t="n"/>
@@ -7386,7 +7428,7 @@
       </c>
       <c r="L108" s="15" t="n"/>
       <c r="M108" s="15" t="n"/>
-      <c r="N108" s="57" t="n"/>
+      <c r="N108" s="47" t="n"/>
       <c r="O108" s="15" t="n"/>
       <c r="P108" s="15" t="n"/>
       <c r="Q108" s="15" t="n"/>
@@ -7442,7 +7484,7 @@
       </c>
       <c r="L109" s="15" t="n"/>
       <c r="M109" s="15" t="n"/>
-      <c r="N109" s="57" t="n"/>
+      <c r="N109" s="47" t="n"/>
       <c r="O109" s="15" t="n"/>
       <c r="P109" s="15" t="n"/>
       <c r="Q109" s="15" t="n"/>
@@ -7500,7 +7542,7 @@
       </c>
       <c r="L110" s="15" t="n"/>
       <c r="M110" s="15" t="n"/>
-      <c r="N110" s="57" t="n"/>
+      <c r="N110" s="47" t="n"/>
       <c r="O110" s="15" t="n"/>
       <c r="P110" s="15" t="n"/>
       <c r="Q110" s="15" t="n"/>
@@ -7558,7 +7600,7 @@
       </c>
       <c r="L111" s="15" t="n"/>
       <c r="M111" s="15" t="n"/>
-      <c r="N111" s="57" t="n"/>
+      <c r="N111" s="47" t="n"/>
       <c r="O111" s="15" t="n"/>
       <c r="P111" s="15" t="n"/>
       <c r="Q111" s="15" t="n"/>
@@ -7614,7 +7656,7 @@
       </c>
       <c r="L112" s="15" t="n"/>
       <c r="M112" s="15" t="n"/>
-      <c r="N112" s="57" t="n"/>
+      <c r="N112" s="47" t="n"/>
       <c r="O112" s="15" t="n"/>
       <c r="P112" s="15" t="n"/>
       <c r="Q112" s="15" t="n"/>
@@ -7670,7 +7712,7 @@
       </c>
       <c r="L113" s="15" t="n"/>
       <c r="M113" s="15" t="n"/>
-      <c r="N113" s="57" t="n"/>
+      <c r="N113" s="47" t="n"/>
       <c r="O113" s="15" t="n"/>
       <c r="P113" s="15" t="n"/>
       <c r="Q113" s="15" t="n"/>
@@ -7728,7 +7770,7 @@
       </c>
       <c r="L114" s="15" t="n"/>
       <c r="M114" s="15" t="n"/>
-      <c r="N114" s="57" t="n"/>
+      <c r="N114" s="47" t="n"/>
       <c r="O114" s="15" t="n"/>
       <c r="P114" s="15" t="n"/>
       <c r="Q114" s="15" t="n"/>
@@ -7786,7 +7828,7 @@
       </c>
       <c r="L115" s="15" t="n"/>
       <c r="M115" s="15" t="n"/>
-      <c r="N115" s="57" t="n"/>
+      <c r="N115" s="47" t="n"/>
       <c r="O115" s="15" t="n"/>
       <c r="P115" s="15" t="n"/>
       <c r="Q115" s="15" t="n"/>
@@ -7842,7 +7884,7 @@
       </c>
       <c r="L116" s="15" t="n"/>
       <c r="M116" s="15" t="n"/>
-      <c r="N116" s="57" t="n"/>
+      <c r="N116" s="47" t="n"/>
       <c r="O116" s="15" t="n"/>
       <c r="P116" s="15" t="n"/>
       <c r="Q116" s="15" t="n"/>
@@ -7900,7 +7942,7 @@
       </c>
       <c r="L117" s="15" t="n"/>
       <c r="M117" s="15" t="n"/>
-      <c r="N117" s="57" t="n"/>
+      <c r="N117" s="47" t="n"/>
       <c r="O117" s="15" t="n"/>
       <c r="P117" s="15" t="n"/>
       <c r="Q117" s="15" t="n"/>
@@ -7958,7 +8000,7 @@
       </c>
       <c r="L118" s="15" t="n"/>
       <c r="M118" s="15" t="n"/>
-      <c r="N118" s="57" t="n"/>
+      <c r="N118" s="47" t="n"/>
       <c r="O118" s="15" t="n"/>
       <c r="P118" s="15" t="n"/>
       <c r="Q118" s="15" t="n"/>
@@ -8014,7 +8056,7 @@
       </c>
       <c r="L119" s="15" t="n"/>
       <c r="M119" s="15" t="n"/>
-      <c r="N119" s="57" t="n"/>
+      <c r="N119" s="47" t="n"/>
       <c r="O119" s="15" t="n"/>
       <c r="P119" s="15" t="n"/>
       <c r="Q119" s="15" t="n"/>
@@ -8072,7 +8114,7 @@
       </c>
       <c r="L120" s="15" t="n"/>
       <c r="M120" s="15" t="n"/>
-      <c r="N120" s="57" t="n"/>
+      <c r="N120" s="47" t="n"/>
       <c r="O120" s="15" t="n"/>
       <c r="P120" s="15" t="n"/>
       <c r="Q120" s="15" t="n"/>
@@ -8130,7 +8172,7 @@
       </c>
       <c r="L121" s="15" t="n"/>
       <c r="M121" s="15" t="n"/>
-      <c r="N121" s="57" t="n"/>
+      <c r="N121" s="47" t="n"/>
       <c r="O121" s="15" t="n"/>
       <c r="P121" s="15" t="n"/>
       <c r="Q121" s="15" t="n"/>
@@ -8186,7 +8228,7 @@
       </c>
       <c r="L122" s="20" t="n"/>
       <c r="M122" s="20" t="n"/>
-      <c r="N122" s="58" t="n"/>
+      <c r="N122" s="48" t="n"/>
       <c r="O122" s="20" t="n"/>
       <c r="P122" s="20" t="n"/>
       <c r="Q122" s="20" t="n"/>
@@ -8242,7 +8284,7 @@
       </c>
       <c r="L123" s="20" t="n"/>
       <c r="M123" s="20" t="n"/>
-      <c r="N123" s="58" t="n"/>
+      <c r="N123" s="48" t="n"/>
       <c r="O123" s="20" t="n"/>
       <c r="P123" s="20" t="n"/>
       <c r="Q123" s="20" t="n"/>
@@ -8300,7 +8342,7 @@
       </c>
       <c r="L124" s="20" t="n"/>
       <c r="M124" s="20" t="n"/>
-      <c r="N124" s="58" t="n"/>
+      <c r="N124" s="48" t="n"/>
       <c r="O124" s="20" t="n"/>
       <c r="P124" s="20" t="n"/>
       <c r="Q124" s="20" t="n"/>
@@ -8358,7 +8400,7 @@
       </c>
       <c r="L125" s="20" t="n"/>
       <c r="M125" s="20" t="n"/>
-      <c r="N125" s="58" t="n"/>
+      <c r="N125" s="48" t="n"/>
       <c r="O125" s="20" t="n"/>
       <c r="P125" s="20" t="n"/>
       <c r="Q125" s="20" t="n"/>
@@ -8414,7 +8456,7 @@
       </c>
       <c r="L126" s="20" t="n"/>
       <c r="M126" s="20" t="n"/>
-      <c r="N126" s="58" t="n"/>
+      <c r="N126" s="48" t="n"/>
       <c r="O126" s="20" t="n"/>
       <c r="P126" s="20" t="n"/>
       <c r="Q126" s="20" t="n"/>
@@ -8472,7 +8514,7 @@
       </c>
       <c r="L127" s="20" t="n"/>
       <c r="M127" s="20" t="n"/>
-      <c r="N127" s="58" t="n"/>
+      <c r="N127" s="48" t="n"/>
       <c r="O127" s="20" t="n"/>
       <c r="P127" s="20" t="n"/>
       <c r="Q127" s="20" t="n"/>
@@ -8530,7 +8572,7 @@
       </c>
       <c r="L128" s="20" t="n"/>
       <c r="M128" s="20" t="n"/>
-      <c r="N128" s="58" t="n"/>
+      <c r="N128" s="48" t="n"/>
       <c r="O128" s="20" t="n"/>
       <c r="P128" s="20" t="n"/>
       <c r="Q128" s="20" t="n"/>
@@ -8586,7 +8628,7 @@
       </c>
       <c r="L129" s="20" t="n"/>
       <c r="M129" s="20" t="n"/>
-      <c r="N129" s="58" t="n"/>
+      <c r="N129" s="48" t="n"/>
       <c r="O129" s="20" t="n"/>
       <c r="P129" s="20" t="n"/>
       <c r="Q129" s="20" t="n"/>
@@ -8644,7 +8686,7 @@
       </c>
       <c r="L130" s="20" t="n"/>
       <c r="M130" s="20" t="n"/>
-      <c r="N130" s="58" t="n"/>
+      <c r="N130" s="48" t="n"/>
       <c r="O130" s="20" t="n"/>
       <c r="P130" s="20" t="n"/>
       <c r="Q130" s="20" t="n"/>
@@ -8702,7 +8744,7 @@
       </c>
       <c r="L131" s="20" t="n"/>
       <c r="M131" s="20" t="n"/>
-      <c r="N131" s="58" t="n"/>
+      <c r="N131" s="48" t="n"/>
       <c r="O131" s="20" t="n"/>
       <c r="P131" s="20" t="n"/>
       <c r="Q131" s="20" t="n"/>
@@ -8758,7 +8800,7 @@
       </c>
       <c r="L132" s="15" t="n"/>
       <c r="M132" s="15" t="n"/>
-      <c r="N132" s="57" t="n"/>
+      <c r="N132" s="47" t="n"/>
       <c r="O132" s="15" t="n"/>
       <c r="P132" s="15" t="n"/>
       <c r="Q132" s="15" t="n"/>
@@ -8814,7 +8856,7 @@
       </c>
       <c r="L133" s="15" t="n"/>
       <c r="M133" s="15" t="n"/>
-      <c r="N133" s="57" t="n"/>
+      <c r="N133" s="47" t="n"/>
       <c r="O133" s="15" t="n"/>
       <c r="P133" s="15" t="n"/>
       <c r="Q133" s="15" t="n"/>
@@ -8872,7 +8914,7 @@
       </c>
       <c r="L134" s="15" t="n"/>
       <c r="M134" s="15" t="n"/>
-      <c r="N134" s="57" t="n"/>
+      <c r="N134" s="47" t="n"/>
       <c r="O134" s="15" t="n"/>
       <c r="P134" s="15" t="n"/>
       <c r="Q134" s="15" t="n"/>
@@ -8930,7 +8972,7 @@
       </c>
       <c r="L135" s="15" t="n"/>
       <c r="M135" s="15" t="n"/>
-      <c r="N135" s="57" t="n"/>
+      <c r="N135" s="47" t="n"/>
       <c r="O135" s="15" t="n"/>
       <c r="P135" s="15" t="n"/>
       <c r="Q135" s="15" t="n"/>
@@ -8986,7 +9028,7 @@
       </c>
       <c r="L136" s="15" t="n"/>
       <c r="M136" s="15" t="n"/>
-      <c r="N136" s="57" t="n"/>
+      <c r="N136" s="47" t="n"/>
       <c r="O136" s="15" t="n"/>
       <c r="P136" s="15" t="n"/>
       <c r="Q136" s="15" t="n"/>
@@ -9044,7 +9086,7 @@
       </c>
       <c r="L137" s="15" t="n"/>
       <c r="M137" s="15" t="n"/>
-      <c r="N137" s="57" t="n"/>
+      <c r="N137" s="47" t="n"/>
       <c r="O137" s="15" t="n"/>
       <c r="P137" s="15" t="n"/>
       <c r="Q137" s="15" t="n"/>
@@ -9102,7 +9144,7 @@
       </c>
       <c r="L138" s="15" t="n"/>
       <c r="M138" s="15" t="n"/>
-      <c r="N138" s="57" t="n"/>
+      <c r="N138" s="47" t="n"/>
       <c r="O138" s="15" t="n"/>
       <c r="P138" s="15" t="n"/>
       <c r="Q138" s="15" t="n"/>
@@ -9158,7 +9200,7 @@
       </c>
       <c r="L139" s="15" t="n"/>
       <c r="M139" s="15" t="n"/>
-      <c r="N139" s="57" t="n"/>
+      <c r="N139" s="47" t="n"/>
       <c r="O139" s="15" t="n"/>
       <c r="P139" s="15" t="n"/>
       <c r="Q139" s="15" t="n"/>
@@ -9216,7 +9258,7 @@
       </c>
       <c r="L140" s="15" t="n"/>
       <c r="M140" s="15" t="n"/>
-      <c r="N140" s="57" t="n"/>
+      <c r="N140" s="47" t="n"/>
       <c r="O140" s="15" t="n"/>
       <c r="P140" s="15" t="n"/>
       <c r="Q140" s="15" t="n"/>
@@ -9274,7 +9316,7 @@
       </c>
       <c r="L141" s="15" t="n"/>
       <c r="M141" s="15" t="n"/>
-      <c r="N141" s="57" t="n"/>
+      <c r="N141" s="47" t="n"/>
       <c r="O141" s="15" t="n"/>
       <c r="P141" s="15" t="n"/>
       <c r="Q141" s="15" t="n"/>
@@ -9330,7 +9372,7 @@
       </c>
       <c r="L142" s="15" t="n"/>
       <c r="M142" s="15" t="n"/>
-      <c r="N142" s="57" t="n"/>
+      <c r="N142" s="47" t="n"/>
       <c r="O142" s="15" t="n"/>
       <c r="P142" s="15" t="n"/>
       <c r="Q142" s="15" t="n"/>
@@ -9386,7 +9428,7 @@
       </c>
       <c r="L143" s="15" t="n"/>
       <c r="M143" s="15" t="n"/>
-      <c r="N143" s="57" t="n"/>
+      <c r="N143" s="47" t="n"/>
       <c r="O143" s="15" t="n"/>
       <c r="P143" s="15" t="n"/>
       <c r="Q143" s="15" t="n"/>
@@ -9444,7 +9486,7 @@
       </c>
       <c r="L144" s="15" t="n"/>
       <c r="M144" s="15" t="n"/>
-      <c r="N144" s="57" t="n"/>
+      <c r="N144" s="47" t="n"/>
       <c r="O144" s="15" t="n"/>
       <c r="P144" s="15" t="n"/>
       <c r="Q144" s="15" t="n"/>
@@ -9502,7 +9544,7 @@
       </c>
       <c r="L145" s="15" t="n"/>
       <c r="M145" s="15" t="n"/>
-      <c r="N145" s="57" t="n"/>
+      <c r="N145" s="47" t="n"/>
       <c r="O145" s="15" t="n"/>
       <c r="P145" s="15" t="n"/>
       <c r="Q145" s="15" t="n"/>
@@ -9558,7 +9600,7 @@
       </c>
       <c r="L146" s="15" t="n"/>
       <c r="M146" s="15" t="n"/>
-      <c r="N146" s="57" t="n"/>
+      <c r="N146" s="47" t="n"/>
       <c r="O146" s="15" t="n"/>
       <c r="P146" s="15" t="n"/>
       <c r="Q146" s="15" t="n"/>
@@ -9616,7 +9658,7 @@
       </c>
       <c r="L147" s="15" t="n"/>
       <c r="M147" s="15" t="n"/>
-      <c r="N147" s="57" t="n"/>
+      <c r="N147" s="47" t="n"/>
       <c r="O147" s="15" t="n"/>
       <c r="P147" s="15" t="n"/>
       <c r="Q147" s="15" t="n"/>
@@ -9674,7 +9716,7 @@
       </c>
       <c r="L148" s="15" t="n"/>
       <c r="M148" s="15" t="n"/>
-      <c r="N148" s="57" t="n"/>
+      <c r="N148" s="47" t="n"/>
       <c r="O148" s="15" t="n"/>
       <c r="P148" s="15" t="n"/>
       <c r="Q148" s="15" t="n"/>
@@ -9730,7 +9772,7 @@
       </c>
       <c r="L149" s="15" t="n"/>
       <c r="M149" s="15" t="n"/>
-      <c r="N149" s="57" t="n"/>
+      <c r="N149" s="47" t="n"/>
       <c r="O149" s="15" t="n"/>
       <c r="P149" s="15" t="n"/>
       <c r="Q149" s="15" t="n"/>
@@ -9788,7 +9830,7 @@
       </c>
       <c r="L150" s="15" t="n"/>
       <c r="M150" s="15" t="n"/>
-      <c r="N150" s="57" t="n"/>
+      <c r="N150" s="47" t="n"/>
       <c r="O150" s="15" t="n"/>
       <c r="P150" s="15" t="n"/>
       <c r="Q150" s="15" t="n"/>
@@ -9846,7 +9888,7 @@
       </c>
       <c r="L151" s="15" t="n"/>
       <c r="M151" s="15" t="n"/>
-      <c r="N151" s="57" t="n"/>
+      <c r="N151" s="47" t="n"/>
       <c r="O151" s="15" t="n"/>
       <c r="P151" s="15" t="n"/>
       <c r="Q151" s="15" t="n"/>
@@ -9902,7 +9944,7 @@
       </c>
       <c r="L152" s="15" t="n"/>
       <c r="M152" s="15" t="n"/>
-      <c r="N152" s="57" t="n"/>
+      <c r="N152" s="47" t="n"/>
       <c r="O152" s="15" t="n"/>
       <c r="P152" s="15" t="n"/>
       <c r="Q152" s="15" t="n"/>
@@ -9958,7 +10000,7 @@
       </c>
       <c r="L153" s="15" t="n"/>
       <c r="M153" s="15" t="n"/>
-      <c r="N153" s="57" t="n"/>
+      <c r="N153" s="47" t="n"/>
       <c r="O153" s="15" t="n"/>
       <c r="P153" s="15" t="n"/>
       <c r="Q153" s="15" t="n"/>
@@ -10016,7 +10058,7 @@
       </c>
       <c r="L154" s="15" t="n"/>
       <c r="M154" s="15" t="n"/>
-      <c r="N154" s="57" t="n"/>
+      <c r="N154" s="47" t="n"/>
       <c r="O154" s="15" t="n"/>
       <c r="P154" s="15" t="n"/>
       <c r="Q154" s="15" t="n"/>
@@ -10074,7 +10116,7 @@
       </c>
       <c r="L155" s="15" t="n"/>
       <c r="M155" s="15" t="n"/>
-      <c r="N155" s="57" t="n"/>
+      <c r="N155" s="47" t="n"/>
       <c r="O155" s="15" t="n"/>
       <c r="P155" s="15" t="n"/>
       <c r="Q155" s="15" t="n"/>
@@ -10130,7 +10172,7 @@
       </c>
       <c r="L156" s="15" t="n"/>
       <c r="M156" s="15" t="n"/>
-      <c r="N156" s="57" t="n"/>
+      <c r="N156" s="47" t="n"/>
       <c r="O156" s="15" t="n"/>
       <c r="P156" s="15" t="n"/>
       <c r="Q156" s="15" t="n"/>
@@ -10188,7 +10230,7 @@
       </c>
       <c r="L157" s="15" t="n"/>
       <c r="M157" s="15" t="n"/>
-      <c r="N157" s="57" t="n"/>
+      <c r="N157" s="47" t="n"/>
       <c r="O157" s="15" t="n"/>
       <c r="P157" s="15" t="n"/>
       <c r="Q157" s="15" t="n"/>
@@ -10246,7 +10288,7 @@
       </c>
       <c r="L158" s="15" t="n"/>
       <c r="M158" s="15" t="n"/>
-      <c r="N158" s="57" t="n"/>
+      <c r="N158" s="47" t="n"/>
       <c r="O158" s="15" t="n"/>
       <c r="P158" s="15" t="n"/>
       <c r="Q158" s="15" t="n"/>
@@ -10302,7 +10344,7 @@
       </c>
       <c r="L159" s="15" t="n"/>
       <c r="M159" s="15" t="n"/>
-      <c r="N159" s="57" t="n"/>
+      <c r="N159" s="47" t="n"/>
       <c r="O159" s="15" t="n"/>
       <c r="P159" s="15" t="n"/>
       <c r="Q159" s="15" t="n"/>
@@ -10360,7 +10402,7 @@
       </c>
       <c r="L160" s="15" t="n"/>
       <c r="M160" s="15" t="n"/>
-      <c r="N160" s="57" t="n"/>
+      <c r="N160" s="47" t="n"/>
       <c r="O160" s="15" t="n"/>
       <c r="P160" s="15" t="n"/>
       <c r="Q160" s="15" t="n"/>
@@ -10418,7 +10460,7 @@
       </c>
       <c r="L161" s="15" t="n"/>
       <c r="M161" s="15" t="n"/>
-      <c r="N161" s="57" t="n"/>
+      <c r="N161" s="47" t="n"/>
       <c r="O161" s="15" t="n"/>
       <c r="P161" s="15" t="n"/>
       <c r="Q161" s="15" t="n"/>
@@ -10474,7 +10516,7 @@
       </c>
       <c r="L162" s="15" t="n"/>
       <c r="M162" s="15" t="n"/>
-      <c r="N162" s="57" t="n"/>
+      <c r="N162" s="47" t="n"/>
       <c r="O162" s="15" t="n"/>
       <c r="P162" s="15" t="n"/>
       <c r="Q162" s="15" t="n"/>
@@ -10530,7 +10572,7 @@
       </c>
       <c r="L163" s="15" t="n"/>
       <c r="M163" s="15" t="n"/>
-      <c r="N163" s="57" t="n"/>
+      <c r="N163" s="47" t="n"/>
       <c r="O163" s="15" t="n"/>
       <c r="P163" s="15" t="n"/>
       <c r="Q163" s="15" t="n"/>
@@ -10588,7 +10630,7 @@
       </c>
       <c r="L164" s="15" t="n"/>
       <c r="M164" s="15" t="n"/>
-      <c r="N164" s="57" t="n"/>
+      <c r="N164" s="47" t="n"/>
       <c r="O164" s="15" t="n"/>
       <c r="P164" s="15" t="n"/>
       <c r="Q164" s="15" t="n"/>
@@ -10646,7 +10688,7 @@
       </c>
       <c r="L165" s="15" t="n"/>
       <c r="M165" s="15" t="n"/>
-      <c r="N165" s="57" t="n"/>
+      <c r="N165" s="47" t="n"/>
       <c r="O165" s="15" t="n"/>
       <c r="P165" s="15" t="n"/>
       <c r="Q165" s="15" t="n"/>
@@ -10702,7 +10744,7 @@
       </c>
       <c r="L166" s="15" t="n"/>
       <c r="M166" s="15" t="n"/>
-      <c r="N166" s="57" t="n"/>
+      <c r="N166" s="47" t="n"/>
       <c r="O166" s="15" t="n"/>
       <c r="P166" s="15" t="n"/>
       <c r="Q166" s="15" t="n"/>
@@ -10760,7 +10802,7 @@
       </c>
       <c r="L167" s="15" t="n"/>
       <c r="M167" s="15" t="n"/>
-      <c r="N167" s="57" t="n"/>
+      <c r="N167" s="47" t="n"/>
       <c r="O167" s="15" t="n"/>
       <c r="P167" s="15" t="n"/>
       <c r="Q167" s="15" t="n"/>
@@ -10818,7 +10860,7 @@
       </c>
       <c r="L168" s="15" t="n"/>
       <c r="M168" s="15" t="n"/>
-      <c r="N168" s="57" t="n"/>
+      <c r="N168" s="47" t="n"/>
       <c r="O168" s="15" t="n"/>
       <c r="P168" s="15" t="n"/>
       <c r="Q168" s="15" t="n"/>
@@ -10874,7 +10916,7 @@
       </c>
       <c r="L169" s="15" t="n"/>
       <c r="M169" s="15" t="n"/>
-      <c r="N169" s="57" t="n"/>
+      <c r="N169" s="47" t="n"/>
       <c r="O169" s="15" t="n"/>
       <c r="P169" s="15" t="n"/>
       <c r="Q169" s="15" t="n"/>
@@ -10932,7 +10974,7 @@
       </c>
       <c r="L170" s="15" t="n"/>
       <c r="M170" s="15" t="n"/>
-      <c r="N170" s="57" t="n"/>
+      <c r="N170" s="47" t="n"/>
       <c r="O170" s="15" t="n"/>
       <c r="P170" s="15" t="n"/>
       <c r="Q170" s="15" t="n"/>
@@ -10990,7 +11032,7 @@
       </c>
       <c r="L171" s="15" t="n"/>
       <c r="M171" s="15" t="n"/>
-      <c r="N171" s="57" t="n"/>
+      <c r="N171" s="47" t="n"/>
       <c r="O171" s="15" t="n"/>
       <c r="P171" s="15" t="n"/>
       <c r="Q171" s="15" t="n"/>
@@ -11046,7 +11088,7 @@
       </c>
       <c r="L172" s="15" t="n"/>
       <c r="M172" s="15" t="n"/>
-      <c r="N172" s="57" t="n"/>
+      <c r="N172" s="47" t="n"/>
       <c r="O172" s="15" t="n"/>
       <c r="P172" s="15" t="n"/>
       <c r="Q172" s="15" t="n"/>
@@ -11102,7 +11144,7 @@
       </c>
       <c r="L173" s="15" t="n"/>
       <c r="M173" s="15" t="n"/>
-      <c r="N173" s="57" t="n"/>
+      <c r="N173" s="47" t="n"/>
       <c r="O173" s="15" t="n"/>
       <c r="P173" s="15" t="n"/>
       <c r="Q173" s="15" t="n"/>
@@ -11160,7 +11202,7 @@
       </c>
       <c r="L174" s="15" t="n"/>
       <c r="M174" s="15" t="n"/>
-      <c r="N174" s="57" t="n"/>
+      <c r="N174" s="47" t="n"/>
       <c r="O174" s="15" t="n"/>
       <c r="P174" s="15" t="n"/>
       <c r="Q174" s="15" t="n"/>
@@ -11218,7 +11260,7 @@
       </c>
       <c r="L175" s="15" t="n"/>
       <c r="M175" s="15" t="n"/>
-      <c r="N175" s="57" t="n"/>
+      <c r="N175" s="47" t="n"/>
       <c r="O175" s="15" t="n"/>
       <c r="P175" s="15" t="n"/>
       <c r="Q175" s="15" t="n"/>
@@ -11274,7 +11316,7 @@
       </c>
       <c r="L176" s="15" t="n"/>
       <c r="M176" s="15" t="n"/>
-      <c r="N176" s="57" t="n"/>
+      <c r="N176" s="47" t="n"/>
       <c r="O176" s="15" t="n"/>
       <c r="P176" s="15" t="n"/>
       <c r="Q176" s="15" t="n"/>
@@ -11332,7 +11374,7 @@
       </c>
       <c r="L177" s="15" t="n"/>
       <c r="M177" s="15" t="n"/>
-      <c r="N177" s="57" t="n"/>
+      <c r="N177" s="47" t="n"/>
       <c r="O177" s="15" t="n"/>
       <c r="P177" s="15" t="n"/>
       <c r="Q177" s="15" t="n"/>
@@ -11390,7 +11432,7 @@
       </c>
       <c r="L178" s="15" t="n"/>
       <c r="M178" s="15" t="n"/>
-      <c r="N178" s="57" t="n"/>
+      <c r="N178" s="47" t="n"/>
       <c r="O178" s="15" t="n"/>
       <c r="P178" s="15" t="n"/>
       <c r="Q178" s="15" t="n"/>
@@ -11446,7 +11488,7 @@
       </c>
       <c r="L179" s="15" t="n"/>
       <c r="M179" s="15" t="n"/>
-      <c r="N179" s="57" t="n"/>
+      <c r="N179" s="47" t="n"/>
       <c r="O179" s="15" t="n"/>
       <c r="P179" s="15" t="n"/>
       <c r="Q179" s="15" t="n"/>
@@ -11504,7 +11546,7 @@
       </c>
       <c r="L180" s="15" t="n"/>
       <c r="M180" s="15" t="n"/>
-      <c r="N180" s="57" t="n"/>
+      <c r="N180" s="47" t="n"/>
       <c r="O180" s="15" t="n"/>
       <c r="P180" s="15" t="n"/>
       <c r="Q180" s="15" t="n"/>
@@ -11562,7 +11604,7 @@
       </c>
       <c r="L181" s="15" t="n"/>
       <c r="M181" s="15" t="n"/>
-      <c r="N181" s="57" t="n"/>
+      <c r="N181" s="47" t="n"/>
       <c r="O181" s="15" t="n"/>
       <c r="P181" s="15" t="n"/>
       <c r="Q181" s="15" t="n"/>
@@ -11618,7 +11660,7 @@
       </c>
       <c r="L182" s="15" t="n"/>
       <c r="M182" s="15" t="n"/>
-      <c r="N182" s="57" t="n"/>
+      <c r="N182" s="47" t="n"/>
       <c r="O182" s="15" t="n"/>
       <c r="P182" s="15" t="n"/>
       <c r="Q182" s="15" t="n"/>
@@ -11674,7 +11716,7 @@
       </c>
       <c r="L183" s="15" t="n"/>
       <c r="M183" s="15" t="n"/>
-      <c r="N183" s="57" t="n"/>
+      <c r="N183" s="47" t="n"/>
       <c r="O183" s="15" t="n"/>
       <c r="P183" s="15" t="n"/>
       <c r="Q183" s="15" t="n"/>
@@ -11732,7 +11774,7 @@
       </c>
       <c r="L184" s="15" t="n"/>
       <c r="M184" s="15" t="n"/>
-      <c r="N184" s="57" t="n"/>
+      <c r="N184" s="47" t="n"/>
       <c r="O184" s="15" t="n"/>
       <c r="P184" s="15" t="n"/>
       <c r="Q184" s="15" t="n"/>
@@ -11790,7 +11832,7 @@
       </c>
       <c r="L185" s="15" t="n"/>
       <c r="M185" s="15" t="n"/>
-      <c r="N185" s="57" t="n"/>
+      <c r="N185" s="47" t="n"/>
       <c r="O185" s="15" t="n"/>
       <c r="P185" s="15" t="n"/>
       <c r="Q185" s="15" t="n"/>
@@ -11846,7 +11888,7 @@
       </c>
       <c r="L186" s="15" t="n"/>
       <c r="M186" s="15" t="n"/>
-      <c r="N186" s="57" t="n"/>
+      <c r="N186" s="47" t="n"/>
       <c r="O186" s="15" t="n"/>
       <c r="P186" s="15" t="n"/>
       <c r="Q186" s="15" t="n"/>
@@ -11904,7 +11946,7 @@
       </c>
       <c r="L187" s="15" t="n"/>
       <c r="M187" s="15" t="n"/>
-      <c r="N187" s="57" t="n"/>
+      <c r="N187" s="47" t="n"/>
       <c r="O187" s="15" t="n"/>
       <c r="P187" s="15" t="n"/>
       <c r="Q187" s="15" t="n"/>
@@ -11962,7 +12004,7 @@
       </c>
       <c r="L188" s="15" t="n"/>
       <c r="M188" s="15" t="n"/>
-      <c r="N188" s="57" t="n"/>
+      <c r="N188" s="47" t="n"/>
       <c r="O188" s="15" t="n"/>
       <c r="P188" s="15" t="n"/>
       <c r="Q188" s="15" t="n"/>
@@ -12018,7 +12060,7 @@
       </c>
       <c r="L189" s="15" t="n"/>
       <c r="M189" s="15" t="n"/>
-      <c r="N189" s="57" t="n"/>
+      <c r="N189" s="47" t="n"/>
       <c r="O189" s="15" t="n"/>
       <c r="P189" s="15" t="n"/>
       <c r="Q189" s="15" t="n"/>
@@ -12076,7 +12118,7 @@
       </c>
       <c r="L190" s="15" t="n"/>
       <c r="M190" s="15" t="n"/>
-      <c r="N190" s="57" t="n"/>
+      <c r="N190" s="47" t="n"/>
       <c r="O190" s="15" t="n"/>
       <c r="P190" s="15" t="n"/>
       <c r="Q190" s="15" t="n"/>
@@ -12134,7 +12176,7 @@
       </c>
       <c r="L191" s="15" t="n"/>
       <c r="M191" s="15" t="n"/>
-      <c r="N191" s="57" t="n"/>
+      <c r="N191" s="47" t="n"/>
       <c r="O191" s="15" t="n"/>
       <c r="P191" s="15" t="n"/>
       <c r="Q191" s="15" t="n"/>
@@ -12190,7 +12232,7 @@
       </c>
       <c r="L192" s="15" t="n"/>
       <c r="M192" s="15" t="n"/>
-      <c r="N192" s="57" t="n"/>
+      <c r="N192" s="47" t="n"/>
       <c r="O192" s="15" t="n"/>
       <c r="P192" s="15" t="n"/>
       <c r="Q192" s="15" t="n"/>
@@ -12246,7 +12288,7 @@
       </c>
       <c r="L193" s="15" t="n"/>
       <c r="M193" s="15" t="n"/>
-      <c r="N193" s="57" t="n"/>
+      <c r="N193" s="47" t="n"/>
       <c r="O193" s="15" t="n"/>
       <c r="P193" s="15" t="n"/>
       <c r="Q193" s="15" t="n"/>
@@ -12304,7 +12346,7 @@
       </c>
       <c r="L194" s="15" t="n"/>
       <c r="M194" s="15" t="n"/>
-      <c r="N194" s="57" t="n"/>
+      <c r="N194" s="47" t="n"/>
       <c r="O194" s="15" t="n"/>
       <c r="P194" s="15" t="n"/>
       <c r="Q194" s="15" t="n"/>
@@ -12362,7 +12404,7 @@
       </c>
       <c r="L195" s="15" t="n"/>
       <c r="M195" s="15" t="n"/>
-      <c r="N195" s="57" t="n"/>
+      <c r="N195" s="47" t="n"/>
       <c r="O195" s="15" t="n"/>
       <c r="P195" s="15" t="n"/>
       <c r="Q195" s="15" t="n"/>
@@ -12418,7 +12460,7 @@
       </c>
       <c r="L196" s="15" t="n"/>
       <c r="M196" s="15" t="n"/>
-      <c r="N196" s="57" t="n"/>
+      <c r="N196" s="47" t="n"/>
       <c r="O196" s="15" t="n"/>
       <c r="P196" s="15" t="n"/>
       <c r="Q196" s="15" t="n"/>
@@ -12474,7 +12516,7 @@
       </c>
       <c r="L197" s="15" t="n"/>
       <c r="M197" s="15" t="n"/>
-      <c r="N197" s="57" t="n"/>
+      <c r="N197" s="47" t="n"/>
       <c r="O197" s="15" t="n"/>
       <c r="P197" s="15" t="n"/>
       <c r="Q197" s="15" t="n"/>
@@ -12532,7 +12574,7 @@
       </c>
       <c r="L198" s="15" t="n"/>
       <c r="M198" s="15" t="n"/>
-      <c r="N198" s="57" t="n"/>
+      <c r="N198" s="47" t="n"/>
       <c r="O198" s="15" t="n"/>
       <c r="P198" s="15" t="n"/>
       <c r="Q198" s="15" t="n"/>
@@ -12590,7 +12632,7 @@
       </c>
       <c r="L199" s="15" t="n"/>
       <c r="M199" s="15" t="n"/>
-      <c r="N199" s="57" t="n"/>
+      <c r="N199" s="47" t="n"/>
       <c r="O199" s="15" t="n"/>
       <c r="P199" s="15" t="n"/>
       <c r="Q199" s="15" t="n"/>
@@ -12621,32 +12663,32 @@
   <dimension ref="B2:I37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" style="46" min="1" max="1"/>
-    <col width="26" customWidth="1" style="46" min="2" max="2"/>
-    <col width="16" customWidth="1" style="46" min="3" max="3"/>
-    <col width="22" customWidth="1" style="46" min="4" max="4"/>
-    <col width="40" customWidth="1" style="46" min="5" max="5"/>
-    <col width="20" customWidth="1" style="46" min="6" max="6"/>
-    <col width="22" customWidth="1" style="46" min="7" max="7"/>
-    <col width="11" customWidth="1" style="46" min="8" max="8"/>
-    <col width="40" customWidth="1" style="46" min="9" max="9"/>
+    <col width="2" customWidth="1" style="52" min="1" max="1"/>
+    <col width="26" customWidth="1" style="52" min="2" max="2"/>
+    <col width="16" customWidth="1" style="52" min="3" max="3"/>
+    <col width="22" customWidth="1" style="52" min="4" max="4"/>
+    <col width="40" customWidth="1" style="52" min="5" max="5"/>
+    <col width="20" customWidth="1" style="52" min="6" max="6"/>
+    <col width="22" customWidth="1" style="52" min="7" max="7"/>
+    <col width="11" customWidth="1" style="52" min="8" max="8"/>
+    <col width="40" customWidth="1" style="52" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="2" ht="17" customHeight="1" s="46">
+    <row r="2" ht="17" customHeight="1" s="52">
       <c r="B2" s="40" t="inlineStr">
         <is>
           <t>Workout Library</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1" s="46">
-      <c r="B3" s="53" t="inlineStr">
+    <row r="3" ht="58" customHeight="1" s="52">
+      <c r="B3" s="59" t="inlineStr">
         <is>
           <t>Named, spelled-out sessions referenced by the 'Workout' column on the Weekly Plan. All paces are in min/km, CALIBRATED to the Wk1 5K baseline (24 Jul 2026: 4:40/km, RPE 7) with a conservative interpretation. MP band shifted to the sub-3:50 goal (5:27/km). Recheck after the Wk13 half-marathon time trial.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1" s="46">
+    <row r="5" ht="16" customHeight="1" s="52">
       <c r="B5" s="41" t="inlineStr">
         <is>
           <t>Workout</t>
@@ -12689,20 +12731,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="50" t="inlineStr">
+      <c r="B6" s="56" t="inlineStr">
         <is>
           <t>EASY / STEADY / LONG (aerobic base - reference by distance on the plan)</t>
         </is>
       </c>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="51" t="n"/>
-      <c r="E6" s="51" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="51" t="n"/>
-      <c r="H6" s="51" t="n"/>
-      <c r="I6" s="52" t="n"/>
-    </row>
-    <row r="7" ht="32" customHeight="1" s="46">
+      <c r="C6" s="57" t="n"/>
+      <c r="D6" s="57" t="n"/>
+      <c r="E6" s="57" t="n"/>
+      <c r="F6" s="57" t="n"/>
+      <c r="G6" s="57" t="n"/>
+      <c r="H6" s="57" t="n"/>
+      <c r="I6" s="58" t="n"/>
+    </row>
+    <row r="7" ht="32" customHeight="1" s="52">
       <c r="B7" s="42" t="inlineStr">
         <is>
           <t>Easy run</t>
@@ -12744,7 +12786,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1" s="46">
+    <row r="8" ht="32" customHeight="1" s="52">
       <c r="B8" s="42" t="inlineStr">
         <is>
           <t>Medium-long - steady</t>
@@ -12786,7 +12828,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1" s="46">
+    <row r="9" ht="32" customHeight="1" s="52">
       <c r="B9" s="42" t="inlineStr">
         <is>
           <t>Medium-long + MP finish</t>
@@ -12828,7 +12870,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1" s="46">
+    <row r="10" ht="32" customHeight="1" s="52">
       <c r="B10" s="42" t="inlineStr">
         <is>
           <t>Long run - easy</t>
@@ -12870,7 +12912,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1" s="46">
+    <row r="11" ht="32" customHeight="1" s="52">
       <c r="B11" s="42" t="inlineStr">
         <is>
           <t>Long run + MP segments</t>
@@ -12913,20 +12955,20 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="50" t="inlineStr">
+      <c r="B12" s="56" t="inlineStr">
         <is>
           <t>TEMPO (sustained 'comfortably hard' - Tuesday quality)</t>
         </is>
       </c>
-      <c r="C12" s="51" t="n"/>
-      <c r="D12" s="51" t="n"/>
-      <c r="E12" s="51" t="n"/>
-      <c r="F12" s="51" t="n"/>
-      <c r="G12" s="51" t="n"/>
-      <c r="H12" s="51" t="n"/>
-      <c r="I12" s="52" t="n"/>
-    </row>
-    <row r="13" ht="32" customHeight="1" s="46">
+      <c r="C12" s="57" t="n"/>
+      <c r="D12" s="57" t="n"/>
+      <c r="E12" s="57" t="n"/>
+      <c r="F12" s="57" t="n"/>
+      <c r="G12" s="57" t="n"/>
+      <c r="H12" s="57" t="n"/>
+      <c r="I12" s="58" t="n"/>
+    </row>
+    <row r="13" ht="32" customHeight="1" s="52">
       <c r="B13" s="42" t="inlineStr">
         <is>
           <t>12-min tempo</t>
@@ -12966,7 +13008,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1" s="46">
+    <row r="14" ht="16" customHeight="1" s="52">
       <c r="B14" s="42" t="inlineStr">
         <is>
           <t>15-min tempo</t>
@@ -13006,7 +13048,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1" s="46">
+    <row r="15" ht="16" customHeight="1" s="52">
       <c r="B15" s="42" t="inlineStr">
         <is>
           <t>18-min tempo</t>
@@ -13046,7 +13088,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1" s="46">
+    <row r="16" ht="32" customHeight="1" s="52">
       <c r="B16" s="42" t="inlineStr">
         <is>
           <t>2 x 10-min tempo</t>
@@ -13086,7 +13128,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1" s="46">
+    <row r="17" ht="16" customHeight="1" s="52">
       <c r="B17" s="42" t="inlineStr">
         <is>
           <t>18-min tempo (deload)</t>
@@ -13126,7 +13168,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1" s="46">
+    <row r="18" ht="16" customHeight="1" s="52">
       <c r="B18" s="42" t="inlineStr">
         <is>
           <t>25-min tempo</t>
@@ -13166,7 +13208,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1" s="46">
+    <row r="19" ht="16" customHeight="1" s="52">
       <c r="B19" s="42" t="inlineStr">
         <is>
           <t>2 x 10-min tempo (deload)</t>
@@ -13206,7 +13248,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1" s="46">
+    <row r="20" ht="32" customHeight="1" s="52">
       <c r="B20" s="42" t="inlineStr">
         <is>
           <t>3 x 8-min cruise</t>
@@ -13246,7 +13288,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1" s="46">
+    <row r="21" ht="16" customHeight="1" s="52">
       <c r="B21" s="42" t="inlineStr">
         <is>
           <t>3 x 10-min tempo</t>
@@ -13286,7 +13328,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1" s="46">
+    <row r="22" ht="16" customHeight="1" s="52">
       <c r="B22" s="42" t="inlineStr">
         <is>
           <t>15-min tempo (sharpener)</t>
@@ -13327,20 +13369,20 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="50" t="inlineStr">
+      <c r="B23" s="56" t="inlineStr">
         <is>
           <t>INTERVALS (faster reps with jog recovery - Tuesday quality)</t>
         </is>
       </c>
-      <c r="C23" s="51" t="n"/>
-      <c r="D23" s="51" t="n"/>
-      <c r="E23" s="51" t="n"/>
-      <c r="F23" s="51" t="n"/>
-      <c r="G23" s="51" t="n"/>
-      <c r="H23" s="51" t="n"/>
-      <c r="I23" s="52" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1" s="46">
+      <c r="C23" s="57" t="n"/>
+      <c r="D23" s="57" t="n"/>
+      <c r="E23" s="57" t="n"/>
+      <c r="F23" s="57" t="n"/>
+      <c r="G23" s="57" t="n"/>
+      <c r="H23" s="57" t="n"/>
+      <c r="I23" s="58" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1" s="52">
       <c r="B24" s="42" t="inlineStr">
         <is>
           <t>6 x 400 m</t>
@@ -13380,7 +13422,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1" s="46">
+    <row r="25" ht="16" customHeight="1" s="52">
       <c r="B25" s="42" t="inlineStr">
         <is>
           <t>5 x 400 m (deload)</t>
@@ -13420,7 +13462,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1" s="46">
+    <row r="26" ht="16" customHeight="1" s="52">
       <c r="B26" s="42" t="inlineStr">
         <is>
           <t>6 x 500 m</t>
@@ -13460,7 +13502,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1" s="46">
+    <row r="27" ht="16" customHeight="1" s="52">
       <c r="B27" s="42" t="inlineStr">
         <is>
           <t>5 x 800 m</t>
@@ -13500,7 +13542,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1" s="46">
+    <row r="28" ht="16" customHeight="1" s="52">
       <c r="B28" s="42" t="inlineStr">
         <is>
           <t>6 x 600 m</t>
@@ -13540,7 +13582,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="32" customHeight="1" s="46">
+    <row r="29" ht="32" customHeight="1" s="52">
       <c r="B29" s="42" t="inlineStr">
         <is>
           <t>10 x 2 min</t>
@@ -13580,7 +13622,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1" s="46">
+    <row r="30" ht="16" customHeight="1" s="52">
       <c r="B30" s="42" t="inlineStr">
         <is>
           <t>5 x 1 km</t>
@@ -13620,7 +13662,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1" s="46">
+    <row r="31" ht="16" customHeight="1" s="52">
       <c r="B31" s="42" t="inlineStr">
         <is>
           <t>6 x 2 min (sharpener)</t>
@@ -13661,20 +13703,20 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="50" t="inlineStr">
+      <c r="B32" s="56" t="inlineStr">
         <is>
           <t>TIME TRIALS, STRIDES &amp; RACE</t>
         </is>
       </c>
-      <c r="C32" s="51" t="n"/>
-      <c r="D32" s="51" t="n"/>
-      <c r="E32" s="51" t="n"/>
-      <c r="F32" s="51" t="n"/>
-      <c r="G32" s="51" t="n"/>
-      <c r="H32" s="51" t="n"/>
-      <c r="I32" s="52" t="n"/>
-    </row>
-    <row r="33" ht="32" customHeight="1" s="46">
+      <c r="C32" s="57" t="n"/>
+      <c r="D32" s="57" t="n"/>
+      <c r="E32" s="57" t="n"/>
+      <c r="F32" s="57" t="n"/>
+      <c r="G32" s="57" t="n"/>
+      <c r="H32" s="57" t="n"/>
+      <c r="I32" s="58" t="n"/>
+    </row>
+    <row r="33" ht="32" customHeight="1" s="52">
       <c r="B33" s="42" t="inlineStr">
         <is>
           <t>Baseline 5K time trial</t>
@@ -13714,7 +13756,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1" s="46">
+    <row r="34" ht="32" customHeight="1" s="52">
       <c r="B34" s="42" t="inlineStr">
         <is>
           <t>Half-marathon time trial</t>
@@ -13754,7 +13796,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="32" customHeight="1" s="46">
+    <row r="35" ht="32" customHeight="1" s="52">
       <c r="B35" s="42" t="inlineStr">
         <is>
           <t>Shakeout + strides</t>
@@ -13794,7 +13836,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="32" customHeight="1" s="46">
+    <row r="36" ht="32" customHeight="1" s="52">
       <c r="B36" s="42" t="inlineStr">
         <is>
           <t>Pre-race shakeout</t>
@@ -13834,7 +13876,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="32" customHeight="1" s="46">
+    <row r="37" ht="32" customHeight="1" s="52">
       <c r="B37" s="42" t="inlineStr">
         <is>
           <t>Marathon - race day</t>
@@ -13895,12 +13937,12 @@
   <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" style="46" min="1" max="1"/>
-    <col width="14" customWidth="1" style="46" min="2" max="3"/>
-    <col width="16" customWidth="1" style="46" min="4" max="4"/>
-    <col width="12" customWidth="1" style="46" min="5" max="6"/>
-    <col width="9" customWidth="1" style="46" min="7" max="7"/>
-    <col width="10" customWidth="1" style="46" min="8" max="8"/>
+    <col width="6" customWidth="1" style="52" min="1" max="1"/>
+    <col width="14" customWidth="1" style="52" min="2" max="3"/>
+    <col width="16" customWidth="1" style="52" min="4" max="4"/>
+    <col width="12" customWidth="1" style="52" min="5" max="6"/>
+    <col width="9" customWidth="1" style="52" min="7" max="7"/>
+    <col width="10" customWidth="1" style="52" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14639,7 +14681,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="54" t="inlineStr">
+      <c r="A24" s="60" t="inlineStr">
         <is>
           <t>Planned/Completed exclude Rest rows. Adherence = Completed / Planned sessions for the week.</t>
         </is>
@@ -14663,11 +14705,11 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="46" min="1" max="1"/>
-    <col width="16" customWidth="1" style="46" min="2" max="2"/>
-    <col width="34" customWidth="1" style="46" min="3" max="3"/>
-    <col width="50" customWidth="1" style="46" min="4" max="4"/>
-    <col width="16" customWidth="1" style="46" min="5" max="5"/>
+    <col width="12" customWidth="1" style="52" min="1" max="1"/>
+    <col width="16" customWidth="1" style="52" min="2" max="2"/>
+    <col width="34" customWidth="1" style="52" min="3" max="3"/>
+    <col width="50" customWidth="1" style="52" min="4" max="4"/>
+    <col width="16" customWidth="1" style="52" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14748,14 +14790,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="54" t="inlineStr">
+      <c r="A10" s="60" t="inlineStr">
         <is>
           <t>The adapt-training-plan skill logs an entry here every time it adjusts an upcoming week. Add your own rows too if you tweak things manually.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="60" t="n">
+      <c r="A11" s="50" t="n">
         <v>46227</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -14780,7 +14822,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="60" t="n">
+      <c r="A12" s="50" t="n">
         <v>46227</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -14805,7 +14847,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="60" t="n">
+      <c r="A13" s="50" t="n">
         <v>46227</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -14830,7 +14872,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="60" t="n">
+      <c r="A14" s="50" t="n">
         <v>46227</v>
       </c>
       <c r="B14" t="inlineStr">

</xml_diff>

<commit_message>
Log Week 2 long run; switch duration/pace to minutes + formula
Actual Duration is now logged in whole minutes only, and Actual
Pace is calculated from Duration/Distance instead of typed in
directly. Converts the existing Week 1 log entry to the new format
and logs today's 10km long run (55min -> ~5:30/km, rounded from the
reported 5:27/km since whole-minute duration can't hold seconds
precision). Updates CLAUDE.md and the adapt-training-plan skill to
match.
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -259,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -356,6 +356,10 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="45" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="45" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1161,12 +1165,12 @@
       </c>
       <c r="N1" s="12" t="inlineStr">
         <is>
-          <t>Actual Duration (h:mm:ss)</t>
+          <t>Actual Duration (min)</t>
         </is>
       </c>
       <c r="O1" s="12" t="inlineStr">
         <is>
-          <t>Actual Pace (mm:ss/km)</t>
+          <t>Actual Pace (min/km)</t>
         </is>
       </c>
       <c r="P1" s="12" t="inlineStr">
@@ -1239,8 +1243,11 @@
         </is>
       </c>
       <c r="M2" s="15" t="n"/>
-      <c r="N2" s="15" t="n"/>
-      <c r="O2" s="15" t="n"/>
+      <c r="N2" s="68" t="n"/>
+      <c r="O2" s="69">
+        <f>IF(OR(M2="",N2="",M2=0),"",(N2/M2)/1440)</f>
+        <v/>
+      </c>
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="15" t="n"/>
       <c r="R2" s="15" t="inlineStr">
@@ -1307,15 +1314,12 @@
       <c r="M3" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="N3" s="15" t="inlineStr">
-        <is>
-          <t>0:24:00</t>
-        </is>
-      </c>
-      <c r="O3" s="15" t="inlineStr">
-        <is>
-          <t>6:00</t>
-        </is>
+      <c r="N3" s="68" t="n">
+        <v>24</v>
+      </c>
+      <c r="O3" s="69">
+        <f>IF(OR(M3="",N3="",M3=0),"",(N3/M3)/1440)</f>
+        <v/>
       </c>
       <c r="P3" s="15" t="n">
         <v>4</v>
@@ -1377,8 +1381,11 @@
       </c>
       <c r="L4" s="15" t="n"/>
       <c r="M4" s="15" t="n"/>
-      <c r="N4" s="15" t="n"/>
-      <c r="O4" s="15" t="n"/>
+      <c r="N4" s="68" t="n"/>
+      <c r="O4" s="69">
+        <f>IF(OR(M4="",N4="",M4=0),"",(N4/M4)/1440)</f>
+        <v/>
+      </c>
       <c r="P4" s="15" t="n"/>
       <c r="Q4" s="15" t="n"/>
       <c r="R4" s="15" t="n"/>
@@ -1435,8 +1442,11 @@
       </c>
       <c r="L5" s="15" t="n"/>
       <c r="M5" s="15" t="n"/>
-      <c r="N5" s="15" t="n"/>
-      <c r="O5" s="15" t="n"/>
+      <c r="N5" s="68" t="n"/>
+      <c r="O5" s="69">
+        <f>IF(OR(M5="",N5="",M5=0),"",(N5/M5)/1440)</f>
+        <v/>
+      </c>
       <c r="P5" s="15" t="n"/>
       <c r="Q5" s="15" t="n"/>
       <c r="R5" s="15" t="n"/>
@@ -1493,8 +1503,11 @@
       </c>
       <c r="L6" s="15" t="n"/>
       <c r="M6" s="15" t="n"/>
-      <c r="N6" s="15" t="n"/>
-      <c r="O6" s="15" t="n"/>
+      <c r="N6" s="68" t="n"/>
+      <c r="O6" s="69">
+        <f>IF(OR(M6="",N6="",M6=0),"",(N6/M6)/1440)</f>
+        <v/>
+      </c>
       <c r="P6" s="15" t="n"/>
       <c r="Q6" s="15" t="n"/>
       <c r="R6" s="15" t="n"/>
@@ -1551,8 +1564,11 @@
       </c>
       <c r="L7" s="15" t="n"/>
       <c r="M7" s="15" t="n"/>
-      <c r="N7" s="15" t="n"/>
-      <c r="O7" s="15" t="n"/>
+      <c r="N7" s="68" t="n"/>
+      <c r="O7" s="69">
+        <f>IF(OR(M7="",N7="",M7=0),"",(N7/M7)/1440)</f>
+        <v/>
+      </c>
       <c r="P7" s="15" t="n"/>
       <c r="Q7" s="15" t="n"/>
       <c r="R7" s="15" t="n"/>
@@ -1607,8 +1623,11 @@
       </c>
       <c r="L8" s="15" t="n"/>
       <c r="M8" s="15" t="n"/>
-      <c r="N8" s="15" t="n"/>
-      <c r="O8" s="15" t="n"/>
+      <c r="N8" s="68" t="n"/>
+      <c r="O8" s="69">
+        <f>IF(OR(M8="",N8="",M8=0),"",(N8/M8)/1440)</f>
+        <v/>
+      </c>
       <c r="P8" s="15" t="n"/>
       <c r="Q8" s="15" t="n"/>
       <c r="R8" s="15" t="n"/>
@@ -1663,8 +1682,11 @@
       </c>
       <c r="L9" s="15" t="n"/>
       <c r="M9" s="15" t="n"/>
-      <c r="N9" s="15" t="n"/>
-      <c r="O9" s="15" t="n"/>
+      <c r="N9" s="68" t="n"/>
+      <c r="O9" s="69">
+        <f>IF(OR(M9="",N9="",M9=0),"",(N9/M9)/1440)</f>
+        <v/>
+      </c>
       <c r="P9" s="15" t="n"/>
       <c r="Q9" s="15" t="n"/>
       <c r="R9" s="15" t="n"/>
@@ -1721,8 +1743,11 @@
       </c>
       <c r="L10" s="15" t="n"/>
       <c r="M10" s="15" t="n"/>
-      <c r="N10" s="15" t="n"/>
-      <c r="O10" s="15" t="n"/>
+      <c r="N10" s="68" t="n"/>
+      <c r="O10" s="69">
+        <f>IF(OR(M10="",N10="",M10=0),"",(N10/M10)/1440)</f>
+        <v/>
+      </c>
       <c r="P10" s="15" t="n"/>
       <c r="Q10" s="15" t="n"/>
       <c r="R10" s="15" t="n"/>
@@ -1779,8 +1804,11 @@
       </c>
       <c r="L11" s="15" t="n"/>
       <c r="M11" s="15" t="n"/>
-      <c r="N11" s="15" t="n"/>
-      <c r="O11" s="15" t="n"/>
+      <c r="N11" s="68" t="n"/>
+      <c r="O11" s="69">
+        <f>IF(OR(M11="",N11="",M11=0),"",(N11/M11)/1440)</f>
+        <v/>
+      </c>
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="15" t="n"/>
       <c r="R11" s="15" t="n"/>
@@ -1835,8 +1863,11 @@
       </c>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
-      <c r="N12" s="15" t="n"/>
-      <c r="O12" s="15" t="n"/>
+      <c r="N12" s="68" t="n"/>
+      <c r="O12" s="69">
+        <f>IF(OR(M12="",N12="",M12=0),"",(N12/M12)/1440)</f>
+        <v/>
+      </c>
       <c r="P12" s="15" t="n"/>
       <c r="Q12" s="15" t="n"/>
       <c r="R12" s="15" t="n"/>
@@ -1893,8 +1924,11 @@
       </c>
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
-      <c r="N13" s="15" t="n"/>
-      <c r="O13" s="15" t="n"/>
+      <c r="N13" s="68" t="n"/>
+      <c r="O13" s="69">
+        <f>IF(OR(M13="",N13="",M13=0),"",(N13/M13)/1440)</f>
+        <v/>
+      </c>
       <c r="P13" s="15" t="n"/>
       <c r="Q13" s="15" t="n"/>
       <c r="R13" s="15" t="n"/>
@@ -1949,8 +1983,11 @@
       </c>
       <c r="L14" s="15" t="n"/>
       <c r="M14" s="15" t="n"/>
-      <c r="N14" s="15" t="n"/>
-      <c r="O14" s="15" t="n"/>
+      <c r="N14" s="68" t="n"/>
+      <c r="O14" s="69">
+        <f>IF(OR(M14="",N14="",M14=0),"",(N14/M14)/1440)</f>
+        <v/>
+      </c>
       <c r="P14" s="15" t="n"/>
       <c r="Q14" s="15" t="n"/>
       <c r="R14" s="15" t="n"/>
@@ -2007,8 +2044,11 @@
       </c>
       <c r="L15" s="15" t="n"/>
       <c r="M15" s="15" t="n"/>
-      <c r="N15" s="15" t="n"/>
-      <c r="O15" s="15" t="n"/>
+      <c r="N15" s="68" t="n"/>
+      <c r="O15" s="69">
+        <f>IF(OR(M15="",N15="",M15=0),"",(N15/M15)/1440)</f>
+        <v/>
+      </c>
       <c r="P15" s="15" t="n"/>
       <c r="Q15" s="15" t="n"/>
       <c r="R15" s="15" t="n"/>
@@ -2063,10 +2103,21 @@
           <t>Long run - easy</t>
         </is>
       </c>
-      <c r="L16" s="15" t="n"/>
-      <c r="M16" s="15" t="n"/>
-      <c r="N16" s="15" t="n"/>
-      <c r="O16" s="15" t="n"/>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M16" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N16" s="68" t="n">
+        <v>55</v>
+      </c>
+      <c r="O16" s="69">
+        <f>IF(OR(M16="",N16="",M16=0),"",(N16/M16)/1440)</f>
+        <v/>
+      </c>
       <c r="P16" s="15" t="n"/>
       <c r="Q16" s="15" t="n"/>
       <c r="R16" s="15" t="n"/>
@@ -2121,8 +2172,11 @@
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
-      <c r="N17" s="15" t="n"/>
-      <c r="O17" s="15" t="n"/>
+      <c r="N17" s="68" t="n"/>
+      <c r="O17" s="69">
+        <f>IF(OR(M17="",N17="",M17=0),"",(N17/M17)/1440)</f>
+        <v/>
+      </c>
       <c r="P17" s="15" t="n"/>
       <c r="Q17" s="15" t="n"/>
       <c r="R17" s="15" t="n"/>
@@ -2177,8 +2231,11 @@
       </c>
       <c r="L18" s="15" t="n"/>
       <c r="M18" s="15" t="n"/>
-      <c r="N18" s="15" t="n"/>
-      <c r="O18" s="15" t="n"/>
+      <c r="N18" s="68" t="n"/>
+      <c r="O18" s="69">
+        <f>IF(OR(M18="",N18="",M18=0),"",(N18/M18)/1440)</f>
+        <v/>
+      </c>
       <c r="P18" s="15" t="n"/>
       <c r="Q18" s="15" t="n"/>
       <c r="R18" s="15" t="n"/>
@@ -2235,8 +2292,11 @@
       </c>
       <c r="L19" s="15" t="n"/>
       <c r="M19" s="15" t="n"/>
-      <c r="N19" s="15" t="n"/>
-      <c r="O19" s="15" t="n"/>
+      <c r="N19" s="68" t="n"/>
+      <c r="O19" s="69">
+        <f>IF(OR(M19="",N19="",M19=0),"",(N19/M19)/1440)</f>
+        <v/>
+      </c>
       <c r="P19" s="15" t="n"/>
       <c r="Q19" s="15" t="n"/>
       <c r="R19" s="15" t="n"/>
@@ -2293,8 +2353,11 @@
       </c>
       <c r="L20" s="15" t="n"/>
       <c r="M20" s="15" t="n"/>
-      <c r="N20" s="15" t="n"/>
-      <c r="O20" s="15" t="n"/>
+      <c r="N20" s="68" t="n"/>
+      <c r="O20" s="69">
+        <f>IF(OR(M20="",N20="",M20=0),"",(N20/M20)/1440)</f>
+        <v/>
+      </c>
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="15" t="n"/>
       <c r="R20" s="15" t="n"/>
@@ -2349,8 +2412,11 @@
       </c>
       <c r="L21" s="15" t="n"/>
       <c r="M21" s="15" t="n"/>
-      <c r="N21" s="15" t="n"/>
-      <c r="O21" s="15" t="n"/>
+      <c r="N21" s="68" t="n"/>
+      <c r="O21" s="69">
+        <f>IF(OR(M21="",N21="",M21=0),"",(N21/M21)/1440)</f>
+        <v/>
+      </c>
       <c r="P21" s="15" t="n"/>
       <c r="Q21" s="15" t="n"/>
       <c r="R21" s="15" t="n"/>
@@ -2407,8 +2473,11 @@
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>
-      <c r="N22" s="15" t="n"/>
-      <c r="O22" s="15" t="n"/>
+      <c r="N22" s="68" t="n"/>
+      <c r="O22" s="69">
+        <f>IF(OR(M22="",N22="",M22=0),"",(N22/M22)/1440)</f>
+        <v/>
+      </c>
       <c r="P22" s="15" t="n"/>
       <c r="Q22" s="15" t="n"/>
       <c r="R22" s="15" t="n"/>
@@ -2463,8 +2532,11 @@
       </c>
       <c r="L23" s="15" t="n"/>
       <c r="M23" s="15" t="n"/>
-      <c r="N23" s="15" t="n"/>
-      <c r="O23" s="15" t="n"/>
+      <c r="N23" s="68" t="n"/>
+      <c r="O23" s="69">
+        <f>IF(OR(M23="",N23="",M23=0),"",(N23/M23)/1440)</f>
+        <v/>
+      </c>
       <c r="P23" s="15" t="n"/>
       <c r="Q23" s="15" t="n"/>
       <c r="R23" s="15" t="n"/>
@@ -2521,8 +2593,11 @@
       </c>
       <c r="L24" s="15" t="n"/>
       <c r="M24" s="15" t="n"/>
-      <c r="N24" s="15" t="n"/>
-      <c r="O24" s="15" t="n"/>
+      <c r="N24" s="68" t="n"/>
+      <c r="O24" s="69">
+        <f>IF(OR(M24="",N24="",M24=0),"",(N24/M24)/1440)</f>
+        <v/>
+      </c>
       <c r="P24" s="15" t="n"/>
       <c r="Q24" s="15" t="n"/>
       <c r="R24" s="15" t="n"/>
@@ -2579,8 +2654,11 @@
       </c>
       <c r="L25" s="15" t="n"/>
       <c r="M25" s="15" t="n"/>
-      <c r="N25" s="15" t="n"/>
-      <c r="O25" s="15" t="n"/>
+      <c r="N25" s="68" t="n"/>
+      <c r="O25" s="69">
+        <f>IF(OR(M25="",N25="",M25=0),"",(N25/M25)/1440)</f>
+        <v/>
+      </c>
       <c r="P25" s="15" t="n"/>
       <c r="Q25" s="15" t="n"/>
       <c r="R25" s="15" t="n"/>
@@ -2635,8 +2713,11 @@
       </c>
       <c r="L26" s="15" t="n"/>
       <c r="M26" s="15" t="n"/>
-      <c r="N26" s="15" t="n"/>
-      <c r="O26" s="15" t="n"/>
+      <c r="N26" s="68" t="n"/>
+      <c r="O26" s="69">
+        <f>IF(OR(M26="",N26="",M26=0),"",(N26/M26)/1440)</f>
+        <v/>
+      </c>
       <c r="P26" s="15" t="n"/>
       <c r="Q26" s="15" t="n"/>
       <c r="R26" s="15" t="n"/>
@@ -2691,8 +2772,11 @@
       </c>
       <c r="L27" s="15" t="n"/>
       <c r="M27" s="15" t="n"/>
-      <c r="N27" s="15" t="n"/>
-      <c r="O27" s="15" t="n"/>
+      <c r="N27" s="68" t="n"/>
+      <c r="O27" s="69">
+        <f>IF(OR(M27="",N27="",M27=0),"",(N27/M27)/1440)</f>
+        <v/>
+      </c>
       <c r="P27" s="15" t="n"/>
       <c r="Q27" s="15" t="n"/>
       <c r="R27" s="15" t="n"/>
@@ -2749,8 +2833,11 @@
       </c>
       <c r="L28" s="15" t="n"/>
       <c r="M28" s="15" t="n"/>
-      <c r="N28" s="15" t="n"/>
-      <c r="O28" s="15" t="n"/>
+      <c r="N28" s="68" t="n"/>
+      <c r="O28" s="69">
+        <f>IF(OR(M28="",N28="",M28=0),"",(N28/M28)/1440)</f>
+        <v/>
+      </c>
       <c r="P28" s="15" t="n"/>
       <c r="Q28" s="15" t="n"/>
       <c r="R28" s="15" t="n"/>
@@ -2807,8 +2894,11 @@
       </c>
       <c r="L29" s="15" t="n"/>
       <c r="M29" s="15" t="n"/>
-      <c r="N29" s="15" t="n"/>
-      <c r="O29" s="15" t="n"/>
+      <c r="N29" s="68" t="n"/>
+      <c r="O29" s="69">
+        <f>IF(OR(M29="",N29="",M29=0),"",(N29/M29)/1440)</f>
+        <v/>
+      </c>
       <c r="P29" s="15" t="n"/>
       <c r="Q29" s="15" t="n"/>
       <c r="R29" s="15" t="n"/>
@@ -2863,8 +2953,11 @@
       </c>
       <c r="L30" s="15" t="n"/>
       <c r="M30" s="15" t="n"/>
-      <c r="N30" s="15" t="n"/>
-      <c r="O30" s="15" t="n"/>
+      <c r="N30" s="68" t="n"/>
+      <c r="O30" s="69">
+        <f>IF(OR(M30="",N30="",M30=0),"",(N30/M30)/1440)</f>
+        <v/>
+      </c>
       <c r="P30" s="15" t="n"/>
       <c r="Q30" s="15" t="n"/>
       <c r="R30" s="15" t="n"/>
@@ -2921,8 +3014,11 @@
       </c>
       <c r="L31" s="15" t="n"/>
       <c r="M31" s="15" t="n"/>
-      <c r="N31" s="15" t="n"/>
-      <c r="O31" s="15" t="n"/>
+      <c r="N31" s="68" t="n"/>
+      <c r="O31" s="69">
+        <f>IF(OR(M31="",N31="",M31=0),"",(N31/M31)/1440)</f>
+        <v/>
+      </c>
       <c r="P31" s="15" t="n"/>
       <c r="Q31" s="15" t="n"/>
       <c r="R31" s="15" t="n"/>
@@ -2977,8 +3073,11 @@
       </c>
       <c r="L32" s="15" t="n"/>
       <c r="M32" s="15" t="n"/>
-      <c r="N32" s="15" t="n"/>
-      <c r="O32" s="15" t="n"/>
+      <c r="N32" s="68" t="n"/>
+      <c r="O32" s="69">
+        <f>IF(OR(M32="",N32="",M32=0),"",(N32/M32)/1440)</f>
+        <v/>
+      </c>
       <c r="P32" s="15" t="n"/>
       <c r="Q32" s="15" t="n"/>
       <c r="R32" s="15" t="n"/>
@@ -3035,8 +3134,11 @@
       </c>
       <c r="L33" s="15" t="n"/>
       <c r="M33" s="15" t="n"/>
-      <c r="N33" s="15" t="n"/>
-      <c r="O33" s="15" t="n"/>
+      <c r="N33" s="68" t="n"/>
+      <c r="O33" s="69">
+        <f>IF(OR(M33="",N33="",M33=0),"",(N33/M33)/1440)</f>
+        <v/>
+      </c>
       <c r="P33" s="15" t="n"/>
       <c r="Q33" s="15" t="n"/>
       <c r="R33" s="15" t="n"/>
@@ -3093,8 +3195,11 @@
       </c>
       <c r="L34" s="15" t="n"/>
       <c r="M34" s="15" t="n"/>
-      <c r="N34" s="15" t="n"/>
-      <c r="O34" s="15" t="n"/>
+      <c r="N34" s="68" t="n"/>
+      <c r="O34" s="69">
+        <f>IF(OR(M34="",N34="",M34=0),"",(N34/M34)/1440)</f>
+        <v/>
+      </c>
       <c r="P34" s="15" t="n"/>
       <c r="Q34" s="15" t="n"/>
       <c r="R34" s="15" t="n"/>
@@ -3149,8 +3254,11 @@
       </c>
       <c r="L35" s="20" t="n"/>
       <c r="M35" s="20" t="n"/>
-      <c r="N35" s="20" t="n"/>
-      <c r="O35" s="20" t="n"/>
+      <c r="N35" s="70" t="n"/>
+      <c r="O35" s="71">
+        <f>IF(OR(M35="",N35="",M35=0),"",(N35/M35)/1440)</f>
+        <v/>
+      </c>
       <c r="P35" s="20" t="n"/>
       <c r="Q35" s="20" t="n"/>
       <c r="R35" s="20" t="n"/>
@@ -3205,8 +3313,11 @@
       </c>
       <c r="L36" s="20" t="n"/>
       <c r="M36" s="20" t="n"/>
-      <c r="N36" s="20" t="n"/>
-      <c r="O36" s="20" t="n"/>
+      <c r="N36" s="70" t="n"/>
+      <c r="O36" s="71">
+        <f>IF(OR(M36="",N36="",M36=0),"",(N36/M36)/1440)</f>
+        <v/>
+      </c>
       <c r="P36" s="20" t="n"/>
       <c r="Q36" s="20" t="n"/>
       <c r="R36" s="20" t="n"/>
@@ -3263,8 +3374,11 @@
       </c>
       <c r="L37" s="20" t="n"/>
       <c r="M37" s="20" t="n"/>
-      <c r="N37" s="20" t="n"/>
-      <c r="O37" s="20" t="n"/>
+      <c r="N37" s="70" t="n"/>
+      <c r="O37" s="71">
+        <f>IF(OR(M37="",N37="",M37=0),"",(N37/M37)/1440)</f>
+        <v/>
+      </c>
       <c r="P37" s="20" t="n"/>
       <c r="Q37" s="20" t="n"/>
       <c r="R37" s="20" t="n"/>
@@ -3321,8 +3435,11 @@
       </c>
       <c r="L38" s="20" t="n"/>
       <c r="M38" s="20" t="n"/>
-      <c r="N38" s="20" t="n"/>
-      <c r="O38" s="20" t="n"/>
+      <c r="N38" s="70" t="n"/>
+      <c r="O38" s="71">
+        <f>IF(OR(M38="",N38="",M38=0),"",(N38/M38)/1440)</f>
+        <v/>
+      </c>
       <c r="P38" s="20" t="n"/>
       <c r="Q38" s="20" t="n"/>
       <c r="R38" s="20" t="n"/>
@@ -3377,8 +3494,11 @@
       </c>
       <c r="L39" s="20" t="n"/>
       <c r="M39" s="20" t="n"/>
-      <c r="N39" s="20" t="n"/>
-      <c r="O39" s="20" t="n"/>
+      <c r="N39" s="70" t="n"/>
+      <c r="O39" s="71">
+        <f>IF(OR(M39="",N39="",M39=0),"",(N39/M39)/1440)</f>
+        <v/>
+      </c>
       <c r="P39" s="20" t="n"/>
       <c r="Q39" s="20" t="n"/>
       <c r="R39" s="20" t="n"/>
@@ -3435,8 +3555,11 @@
       </c>
       <c r="L40" s="20" t="n"/>
       <c r="M40" s="20" t="n"/>
-      <c r="N40" s="20" t="n"/>
-      <c r="O40" s="20" t="n"/>
+      <c r="N40" s="70" t="n"/>
+      <c r="O40" s="71">
+        <f>IF(OR(M40="",N40="",M40=0),"",(N40/M40)/1440)</f>
+        <v/>
+      </c>
       <c r="P40" s="20" t="n"/>
       <c r="Q40" s="20" t="n"/>
       <c r="R40" s="20" t="n"/>
@@ -3491,8 +3614,11 @@
       </c>
       <c r="L41" s="20" t="n"/>
       <c r="M41" s="20" t="n"/>
-      <c r="N41" s="20" t="n"/>
-      <c r="O41" s="20" t="n"/>
+      <c r="N41" s="70" t="n"/>
+      <c r="O41" s="71">
+        <f>IF(OR(M41="",N41="",M41=0),"",(N41/M41)/1440)</f>
+        <v/>
+      </c>
       <c r="P41" s="20" t="n"/>
       <c r="Q41" s="20" t="n"/>
       <c r="R41" s="20" t="n"/>
@@ -3549,8 +3675,11 @@
       </c>
       <c r="L42" s="20" t="n"/>
       <c r="M42" s="20" t="n"/>
-      <c r="N42" s="20" t="n"/>
-      <c r="O42" s="20" t="n"/>
+      <c r="N42" s="70" t="n"/>
+      <c r="O42" s="71">
+        <f>IF(OR(M42="",N42="",M42=0),"",(N42/M42)/1440)</f>
+        <v/>
+      </c>
       <c r="P42" s="20" t="n"/>
       <c r="Q42" s="20" t="n"/>
       <c r="R42" s="20" t="n"/>
@@ -3607,8 +3736,11 @@
       </c>
       <c r="L43" s="20" t="n"/>
       <c r="M43" s="20" t="n"/>
-      <c r="N43" s="20" t="n"/>
-      <c r="O43" s="20" t="n"/>
+      <c r="N43" s="70" t="n"/>
+      <c r="O43" s="71">
+        <f>IF(OR(M43="",N43="",M43=0),"",(N43/M43)/1440)</f>
+        <v/>
+      </c>
       <c r="P43" s="20" t="n"/>
       <c r="Q43" s="20" t="n"/>
       <c r="R43" s="20" t="n"/>
@@ -3663,8 +3795,11 @@
       </c>
       <c r="L44" s="15" t="n"/>
       <c r="M44" s="15" t="n"/>
-      <c r="N44" s="15" t="n"/>
-      <c r="O44" s="15" t="n"/>
+      <c r="N44" s="68" t="n"/>
+      <c r="O44" s="69">
+        <f>IF(OR(M44="",N44="",M44=0),"",(N44/M44)/1440)</f>
+        <v/>
+      </c>
       <c r="P44" s="15" t="n"/>
       <c r="Q44" s="15" t="n"/>
       <c r="R44" s="15" t="n"/>
@@ -3719,8 +3854,11 @@
       </c>
       <c r="L45" s="15" t="n"/>
       <c r="M45" s="15" t="n"/>
-      <c r="N45" s="15" t="n"/>
-      <c r="O45" s="15" t="n"/>
+      <c r="N45" s="68" t="n"/>
+      <c r="O45" s="69">
+        <f>IF(OR(M45="",N45="",M45=0),"",(N45/M45)/1440)</f>
+        <v/>
+      </c>
       <c r="P45" s="15" t="n"/>
       <c r="Q45" s="15" t="n"/>
       <c r="R45" s="15" t="n"/>
@@ -3777,8 +3915,11 @@
       </c>
       <c r="L46" s="15" t="n"/>
       <c r="M46" s="15" t="n"/>
-      <c r="N46" s="15" t="n"/>
-      <c r="O46" s="15" t="n"/>
+      <c r="N46" s="68" t="n"/>
+      <c r="O46" s="69">
+        <f>IF(OR(M46="",N46="",M46=0),"",(N46/M46)/1440)</f>
+        <v/>
+      </c>
       <c r="P46" s="15" t="n"/>
       <c r="Q46" s="15" t="n"/>
       <c r="R46" s="15" t="n"/>
@@ -3835,8 +3976,11 @@
       </c>
       <c r="L47" s="15" t="n"/>
       <c r="M47" s="15" t="n"/>
-      <c r="N47" s="15" t="n"/>
-      <c r="O47" s="15" t="n"/>
+      <c r="N47" s="68" t="n"/>
+      <c r="O47" s="69">
+        <f>IF(OR(M47="",N47="",M47=0),"",(N47/M47)/1440)</f>
+        <v/>
+      </c>
       <c r="P47" s="15" t="n"/>
       <c r="Q47" s="15" t="n"/>
       <c r="R47" s="15" t="n"/>
@@ -3891,8 +4035,11 @@
       </c>
       <c r="L48" s="15" t="n"/>
       <c r="M48" s="15" t="n"/>
-      <c r="N48" s="15" t="n"/>
-      <c r="O48" s="15" t="n"/>
+      <c r="N48" s="68" t="n"/>
+      <c r="O48" s="69">
+        <f>IF(OR(M48="",N48="",M48=0),"",(N48/M48)/1440)</f>
+        <v/>
+      </c>
       <c r="P48" s="15" t="n"/>
       <c r="Q48" s="15" t="n"/>
       <c r="R48" s="15" t="n"/>
@@ -3949,8 +4096,11 @@
       </c>
       <c r="L49" s="15" t="n"/>
       <c r="M49" s="15" t="n"/>
-      <c r="N49" s="15" t="n"/>
-      <c r="O49" s="15" t="n"/>
+      <c r="N49" s="68" t="n"/>
+      <c r="O49" s="69">
+        <f>IF(OR(M49="",N49="",M49=0),"",(N49/M49)/1440)</f>
+        <v/>
+      </c>
       <c r="P49" s="15" t="n"/>
       <c r="Q49" s="15" t="n"/>
       <c r="R49" s="15" t="n"/>
@@ -4005,8 +4155,11 @@
       </c>
       <c r="L50" s="15" t="n"/>
       <c r="M50" s="15" t="n"/>
-      <c r="N50" s="15" t="n"/>
-      <c r="O50" s="15" t="n"/>
+      <c r="N50" s="68" t="n"/>
+      <c r="O50" s="69">
+        <f>IF(OR(M50="",N50="",M50=0),"",(N50/M50)/1440)</f>
+        <v/>
+      </c>
       <c r="P50" s="15" t="n"/>
       <c r="Q50" s="15" t="n"/>
       <c r="R50" s="15" t="n"/>
@@ -4063,8 +4216,11 @@
       </c>
       <c r="L51" s="15" t="n"/>
       <c r="M51" s="15" t="n"/>
-      <c r="N51" s="15" t="n"/>
-      <c r="O51" s="15" t="n"/>
+      <c r="N51" s="68" t="n"/>
+      <c r="O51" s="69">
+        <f>IF(OR(M51="",N51="",M51=0),"",(N51/M51)/1440)</f>
+        <v/>
+      </c>
       <c r="P51" s="15" t="n"/>
       <c r="Q51" s="15" t="n"/>
       <c r="R51" s="15" t="n"/>
@@ -4121,8 +4277,11 @@
       </c>
       <c r="L52" s="15" t="n"/>
       <c r="M52" s="15" t="n"/>
-      <c r="N52" s="15" t="n"/>
-      <c r="O52" s="15" t="n"/>
+      <c r="N52" s="68" t="n"/>
+      <c r="O52" s="69">
+        <f>IF(OR(M52="",N52="",M52=0),"",(N52/M52)/1440)</f>
+        <v/>
+      </c>
       <c r="P52" s="15" t="n"/>
       <c r="Q52" s="15" t="n"/>
       <c r="R52" s="15" t="n"/>
@@ -4177,8 +4336,11 @@
       </c>
       <c r="L53" s="15" t="n"/>
       <c r="M53" s="15" t="n"/>
-      <c r="N53" s="15" t="n"/>
-      <c r="O53" s="15" t="n"/>
+      <c r="N53" s="68" t="n"/>
+      <c r="O53" s="69">
+        <f>IF(OR(M53="",N53="",M53=0),"",(N53/M53)/1440)</f>
+        <v/>
+      </c>
       <c r="P53" s="15" t="n"/>
       <c r="Q53" s="15" t="n"/>
       <c r="R53" s="15" t="n"/>
@@ -4233,8 +4395,11 @@
       </c>
       <c r="L54" s="15" t="n"/>
       <c r="M54" s="15" t="n"/>
-      <c r="N54" s="15" t="n"/>
-      <c r="O54" s="15" t="n"/>
+      <c r="N54" s="68" t="n"/>
+      <c r="O54" s="69">
+        <f>IF(OR(M54="",N54="",M54=0),"",(N54/M54)/1440)</f>
+        <v/>
+      </c>
       <c r="P54" s="15" t="n"/>
       <c r="Q54" s="15" t="n"/>
       <c r="R54" s="15" t="n"/>
@@ -4291,8 +4456,11 @@
       </c>
       <c r="L55" s="15" t="n"/>
       <c r="M55" s="15" t="n"/>
-      <c r="N55" s="15" t="n"/>
-      <c r="O55" s="15" t="n"/>
+      <c r="N55" s="68" t="n"/>
+      <c r="O55" s="69">
+        <f>IF(OR(M55="",N55="",M55=0),"",(N55/M55)/1440)</f>
+        <v/>
+      </c>
       <c r="P55" s="15" t="n"/>
       <c r="Q55" s="15" t="n"/>
       <c r="R55" s="15" t="n"/>
@@ -4349,8 +4517,11 @@
       </c>
       <c r="L56" s="15" t="n"/>
       <c r="M56" s="15" t="n"/>
-      <c r="N56" s="15" t="n"/>
-      <c r="O56" s="15" t="n"/>
+      <c r="N56" s="68" t="n"/>
+      <c r="O56" s="69">
+        <f>IF(OR(M56="",N56="",M56=0),"",(N56/M56)/1440)</f>
+        <v/>
+      </c>
       <c r="P56" s="15" t="n"/>
       <c r="Q56" s="15" t="n"/>
       <c r="R56" s="15" t="n"/>
@@ -4405,8 +4576,11 @@
       </c>
       <c r="L57" s="15" t="n"/>
       <c r="M57" s="15" t="n"/>
-      <c r="N57" s="15" t="n"/>
-      <c r="O57" s="15" t="n"/>
+      <c r="N57" s="68" t="n"/>
+      <c r="O57" s="69">
+        <f>IF(OR(M57="",N57="",M57=0),"",(N57/M57)/1440)</f>
+        <v/>
+      </c>
       <c r="P57" s="15" t="n"/>
       <c r="Q57" s="15" t="n"/>
       <c r="R57" s="15" t="n"/>
@@ -4463,8 +4637,11 @@
       </c>
       <c r="L58" s="15" t="n"/>
       <c r="M58" s="15" t="n"/>
-      <c r="N58" s="15" t="n"/>
-      <c r="O58" s="15" t="n"/>
+      <c r="N58" s="68" t="n"/>
+      <c r="O58" s="69">
+        <f>IF(OR(M58="",N58="",M58=0),"",(N58/M58)/1440)</f>
+        <v/>
+      </c>
       <c r="P58" s="15" t="n"/>
       <c r="Q58" s="15" t="n"/>
       <c r="R58" s="15" t="n"/>
@@ -4519,8 +4696,11 @@
       </c>
       <c r="L59" s="15" t="n"/>
       <c r="M59" s="15" t="n"/>
-      <c r="N59" s="15" t="n"/>
-      <c r="O59" s="15" t="n"/>
+      <c r="N59" s="68" t="n"/>
+      <c r="O59" s="69">
+        <f>IF(OR(M59="",N59="",M59=0),"",(N59/M59)/1440)</f>
+        <v/>
+      </c>
       <c r="P59" s="15" t="n"/>
       <c r="Q59" s="15" t="n"/>
       <c r="R59" s="15" t="n"/>
@@ -4577,8 +4757,11 @@
       </c>
       <c r="L60" s="15" t="n"/>
       <c r="M60" s="15" t="n"/>
-      <c r="N60" s="15" t="n"/>
-      <c r="O60" s="15" t="n"/>
+      <c r="N60" s="68" t="n"/>
+      <c r="O60" s="69">
+        <f>IF(OR(M60="",N60="",M60=0),"",(N60/M60)/1440)</f>
+        <v/>
+      </c>
       <c r="P60" s="15" t="n"/>
       <c r="Q60" s="15" t="n"/>
       <c r="R60" s="15" t="n"/>
@@ -4635,8 +4818,11 @@
       </c>
       <c r="L61" s="15" t="n"/>
       <c r="M61" s="15" t="n"/>
-      <c r="N61" s="15" t="n"/>
-      <c r="O61" s="15" t="n"/>
+      <c r="N61" s="68" t="n"/>
+      <c r="O61" s="69">
+        <f>IF(OR(M61="",N61="",M61=0),"",(N61/M61)/1440)</f>
+        <v/>
+      </c>
       <c r="P61" s="15" t="n"/>
       <c r="Q61" s="15" t="n"/>
       <c r="R61" s="15" t="n"/>
@@ -4691,8 +4877,11 @@
       </c>
       <c r="L62" s="15" t="n"/>
       <c r="M62" s="15" t="n"/>
-      <c r="N62" s="15" t="n"/>
-      <c r="O62" s="15" t="n"/>
+      <c r="N62" s="68" t="n"/>
+      <c r="O62" s="69">
+        <f>IF(OR(M62="",N62="",M62=0),"",(N62/M62)/1440)</f>
+        <v/>
+      </c>
       <c r="P62" s="15" t="n"/>
       <c r="Q62" s="15" t="n"/>
       <c r="R62" s="15" t="n"/>
@@ -4747,8 +4936,11 @@
       </c>
       <c r="L63" s="15" t="n"/>
       <c r="M63" s="15" t="n"/>
-      <c r="N63" s="15" t="n"/>
-      <c r="O63" s="15" t="n"/>
+      <c r="N63" s="68" t="n"/>
+      <c r="O63" s="69">
+        <f>IF(OR(M63="",N63="",M63=0),"",(N63/M63)/1440)</f>
+        <v/>
+      </c>
       <c r="P63" s="15" t="n"/>
       <c r="Q63" s="15" t="n"/>
       <c r="R63" s="15" t="n"/>
@@ -4805,8 +4997,11 @@
       </c>
       <c r="L64" s="15" t="n"/>
       <c r="M64" s="15" t="n"/>
-      <c r="N64" s="15" t="n"/>
-      <c r="O64" s="15" t="n"/>
+      <c r="N64" s="68" t="n"/>
+      <c r="O64" s="69">
+        <f>IF(OR(M64="",N64="",M64=0),"",(N64/M64)/1440)</f>
+        <v/>
+      </c>
       <c r="P64" s="15" t="n"/>
       <c r="Q64" s="15" t="n"/>
       <c r="R64" s="15" t="n"/>
@@ -4863,8 +5058,11 @@
       </c>
       <c r="L65" s="15" t="n"/>
       <c r="M65" s="15" t="n"/>
-      <c r="N65" s="15" t="n"/>
-      <c r="O65" s="15" t="n"/>
+      <c r="N65" s="68" t="n"/>
+      <c r="O65" s="69">
+        <f>IF(OR(M65="",N65="",M65=0),"",(N65/M65)/1440)</f>
+        <v/>
+      </c>
       <c r="P65" s="15" t="n"/>
       <c r="Q65" s="15" t="n"/>
       <c r="R65" s="15" t="n"/>
@@ -4919,8 +5117,11 @@
       </c>
       <c r="L66" s="15" t="n"/>
       <c r="M66" s="15" t="n"/>
-      <c r="N66" s="15" t="n"/>
-      <c r="O66" s="15" t="n"/>
+      <c r="N66" s="68" t="n"/>
+      <c r="O66" s="69">
+        <f>IF(OR(M66="",N66="",M66=0),"",(N66/M66)/1440)</f>
+        <v/>
+      </c>
       <c r="P66" s="15" t="n"/>
       <c r="Q66" s="15" t="n"/>
       <c r="R66" s="15" t="n"/>
@@ -4977,8 +5178,11 @@
       </c>
       <c r="L67" s="15" t="n"/>
       <c r="M67" s="15" t="n"/>
-      <c r="N67" s="15" t="n"/>
-      <c r="O67" s="15" t="n"/>
+      <c r="N67" s="68" t="n"/>
+      <c r="O67" s="69">
+        <f>IF(OR(M67="",N67="",M67=0),"",(N67/M67)/1440)</f>
+        <v/>
+      </c>
       <c r="P67" s="15" t="n"/>
       <c r="Q67" s="15" t="n"/>
       <c r="R67" s="15" t="n"/>
@@ -5033,8 +5237,11 @@
       </c>
       <c r="L68" s="15" t="n"/>
       <c r="M68" s="15" t="n"/>
-      <c r="N68" s="15" t="n"/>
-      <c r="O68" s="15" t="n"/>
+      <c r="N68" s="68" t="n"/>
+      <c r="O68" s="69">
+        <f>IF(OR(M68="",N68="",M68=0),"",(N68/M68)/1440)</f>
+        <v/>
+      </c>
       <c r="P68" s="15" t="n"/>
       <c r="Q68" s="15" t="n"/>
       <c r="R68" s="15" t="n"/>
@@ -5091,8 +5298,11 @@
       </c>
       <c r="L69" s="15" t="n"/>
       <c r="M69" s="15" t="n"/>
-      <c r="N69" s="15" t="n"/>
-      <c r="O69" s="15" t="n"/>
+      <c r="N69" s="68" t="n"/>
+      <c r="O69" s="69">
+        <f>IF(OR(M69="",N69="",M69=0),"",(N69/M69)/1440)</f>
+        <v/>
+      </c>
       <c r="P69" s="15" t="n"/>
       <c r="Q69" s="15" t="n"/>
       <c r="R69" s="15" t="n"/>
@@ -5149,8 +5359,11 @@
       </c>
       <c r="L70" s="15" t="n"/>
       <c r="M70" s="15" t="n"/>
-      <c r="N70" s="15" t="n"/>
-      <c r="O70" s="15" t="n"/>
+      <c r="N70" s="68" t="n"/>
+      <c r="O70" s="69">
+        <f>IF(OR(M70="",N70="",M70=0),"",(N70/M70)/1440)</f>
+        <v/>
+      </c>
       <c r="P70" s="15" t="n"/>
       <c r="Q70" s="15" t="n"/>
       <c r="R70" s="15" t="n"/>
@@ -5207,8 +5420,11 @@
       </c>
       <c r="L71" s="15" t="n"/>
       <c r="M71" s="15" t="n"/>
-      <c r="N71" s="15" t="n"/>
-      <c r="O71" s="15" t="n"/>
+      <c r="N71" s="68" t="n"/>
+      <c r="O71" s="69">
+        <f>IF(OR(M71="",N71="",M71=0),"",(N71/M71)/1440)</f>
+        <v/>
+      </c>
       <c r="P71" s="15" t="n"/>
       <c r="Q71" s="15" t="n"/>
       <c r="R71" s="15" t="n"/>
@@ -5263,8 +5479,11 @@
       </c>
       <c r="L72" s="15" t="n"/>
       <c r="M72" s="15" t="n"/>
-      <c r="N72" s="15" t="n"/>
-      <c r="O72" s="15" t="n"/>
+      <c r="N72" s="68" t="n"/>
+      <c r="O72" s="69">
+        <f>IF(OR(M72="",N72="",M72=0),"",(N72/M72)/1440)</f>
+        <v/>
+      </c>
       <c r="P72" s="15" t="n"/>
       <c r="Q72" s="15" t="n"/>
       <c r="R72" s="15" t="n"/>
@@ -5319,8 +5538,11 @@
       </c>
       <c r="L73" s="15" t="n"/>
       <c r="M73" s="15" t="n"/>
-      <c r="N73" s="15" t="n"/>
-      <c r="O73" s="15" t="n"/>
+      <c r="N73" s="68" t="n"/>
+      <c r="O73" s="69">
+        <f>IF(OR(M73="",N73="",M73=0),"",(N73/M73)/1440)</f>
+        <v/>
+      </c>
       <c r="P73" s="15" t="n"/>
       <c r="Q73" s="15" t="n"/>
       <c r="R73" s="15" t="n"/>
@@ -5377,8 +5599,11 @@
       </c>
       <c r="L74" s="15" t="n"/>
       <c r="M74" s="15" t="n"/>
-      <c r="N74" s="15" t="n"/>
-      <c r="O74" s="15" t="n"/>
+      <c r="N74" s="68" t="n"/>
+      <c r="O74" s="69">
+        <f>IF(OR(M74="",N74="",M74=0),"",(N74/M74)/1440)</f>
+        <v/>
+      </c>
       <c r="P74" s="15" t="n"/>
       <c r="Q74" s="15" t="n"/>
       <c r="R74" s="15" t="n"/>
@@ -5435,8 +5660,11 @@
       </c>
       <c r="L75" s="15" t="n"/>
       <c r="M75" s="15" t="n"/>
-      <c r="N75" s="15" t="n"/>
-      <c r="O75" s="15" t="n"/>
+      <c r="N75" s="68" t="n"/>
+      <c r="O75" s="69">
+        <f>IF(OR(M75="",N75="",M75=0),"",(N75/M75)/1440)</f>
+        <v/>
+      </c>
       <c r="P75" s="15" t="n"/>
       <c r="Q75" s="15" t="n"/>
       <c r="R75" s="15" t="n"/>
@@ -5491,8 +5719,11 @@
       </c>
       <c r="L76" s="15" t="n"/>
       <c r="M76" s="15" t="n"/>
-      <c r="N76" s="15" t="n"/>
-      <c r="O76" s="15" t="n"/>
+      <c r="N76" s="68" t="n"/>
+      <c r="O76" s="69">
+        <f>IF(OR(M76="",N76="",M76=0),"",(N76/M76)/1440)</f>
+        <v/>
+      </c>
       <c r="P76" s="15" t="n"/>
       <c r="Q76" s="15" t="n"/>
       <c r="R76" s="15" t="n"/>
@@ -5549,8 +5780,11 @@
       </c>
       <c r="L77" s="15" t="n"/>
       <c r="M77" s="15" t="n"/>
-      <c r="N77" s="15" t="n"/>
-      <c r="O77" s="15" t="n"/>
+      <c r="N77" s="68" t="n"/>
+      <c r="O77" s="69">
+        <f>IF(OR(M77="",N77="",M77=0),"",(N77/M77)/1440)</f>
+        <v/>
+      </c>
       <c r="P77" s="15" t="n"/>
       <c r="Q77" s="15" t="n"/>
       <c r="R77" s="15" t="n"/>
@@ -5605,8 +5839,11 @@
       </c>
       <c r="L78" s="15" t="n"/>
       <c r="M78" s="15" t="n"/>
-      <c r="N78" s="15" t="n"/>
-      <c r="O78" s="15" t="n"/>
+      <c r="N78" s="68" t="n"/>
+      <c r="O78" s="69">
+        <f>IF(OR(M78="",N78="",M78=0),"",(N78/M78)/1440)</f>
+        <v/>
+      </c>
       <c r="P78" s="15" t="n"/>
       <c r="Q78" s="15" t="n"/>
       <c r="R78" s="15" t="n"/>
@@ -5663,8 +5900,11 @@
       </c>
       <c r="L79" s="15" t="n"/>
       <c r="M79" s="15" t="n"/>
-      <c r="N79" s="15" t="n"/>
-      <c r="O79" s="15" t="n"/>
+      <c r="N79" s="68" t="n"/>
+      <c r="O79" s="69">
+        <f>IF(OR(M79="",N79="",M79=0),"",(N79/M79)/1440)</f>
+        <v/>
+      </c>
       <c r="P79" s="15" t="n"/>
       <c r="Q79" s="15" t="n"/>
       <c r="R79" s="15" t="n"/>
@@ -5721,8 +5961,11 @@
       </c>
       <c r="L80" s="15" t="n"/>
       <c r="M80" s="15" t="n"/>
-      <c r="N80" s="15" t="n"/>
-      <c r="O80" s="15" t="n"/>
+      <c r="N80" s="68" t="n"/>
+      <c r="O80" s="69">
+        <f>IF(OR(M80="",N80="",M80=0),"",(N80/M80)/1440)</f>
+        <v/>
+      </c>
       <c r="P80" s="15" t="n"/>
       <c r="Q80" s="15" t="n"/>
       <c r="R80" s="15" t="n"/>
@@ -5779,8 +6022,11 @@
       </c>
       <c r="L81" s="15" t="n"/>
       <c r="M81" s="15" t="n"/>
-      <c r="N81" s="15" t="n"/>
-      <c r="O81" s="15" t="n"/>
+      <c r="N81" s="68" t="n"/>
+      <c r="O81" s="69">
+        <f>IF(OR(M81="",N81="",M81=0),"",(N81/M81)/1440)</f>
+        <v/>
+      </c>
       <c r="P81" s="15" t="n"/>
       <c r="Q81" s="15" t="n"/>
       <c r="R81" s="15" t="n"/>
@@ -5835,8 +6081,11 @@
       </c>
       <c r="L82" s="20" t="n"/>
       <c r="M82" s="20" t="n"/>
-      <c r="N82" s="20" t="n"/>
-      <c r="O82" s="20" t="n"/>
+      <c r="N82" s="70" t="n"/>
+      <c r="O82" s="71">
+        <f>IF(OR(M82="",N82="",M82=0),"",(N82/M82)/1440)</f>
+        <v/>
+      </c>
       <c r="P82" s="20" t="n"/>
       <c r="Q82" s="20" t="n"/>
       <c r="R82" s="20" t="n"/>
@@ -5891,8 +6140,11 @@
       </c>
       <c r="L83" s="20" t="n"/>
       <c r="M83" s="20" t="n"/>
-      <c r="N83" s="20" t="n"/>
-      <c r="O83" s="20" t="n"/>
+      <c r="N83" s="70" t="n"/>
+      <c r="O83" s="71">
+        <f>IF(OR(M83="",N83="",M83=0),"",(N83/M83)/1440)</f>
+        <v/>
+      </c>
       <c r="P83" s="20" t="n"/>
       <c r="Q83" s="20" t="n"/>
       <c r="R83" s="20" t="n"/>
@@ -5949,8 +6201,11 @@
       </c>
       <c r="L84" s="20" t="n"/>
       <c r="M84" s="20" t="n"/>
-      <c r="N84" s="20" t="n"/>
-      <c r="O84" s="20" t="n"/>
+      <c r="N84" s="70" t="n"/>
+      <c r="O84" s="71">
+        <f>IF(OR(M84="",N84="",M84=0),"",(N84/M84)/1440)</f>
+        <v/>
+      </c>
       <c r="P84" s="20" t="n"/>
       <c r="Q84" s="20" t="n"/>
       <c r="R84" s="20" t="n"/>
@@ -6007,8 +6262,11 @@
       </c>
       <c r="L85" s="20" t="n"/>
       <c r="M85" s="20" t="n"/>
-      <c r="N85" s="20" t="n"/>
-      <c r="O85" s="20" t="n"/>
+      <c r="N85" s="70" t="n"/>
+      <c r="O85" s="71">
+        <f>IF(OR(M85="",N85="",M85=0),"",(N85/M85)/1440)</f>
+        <v/>
+      </c>
       <c r="P85" s="20" t="n"/>
       <c r="Q85" s="20" t="n"/>
       <c r="R85" s="20" t="n"/>
@@ -6063,8 +6321,11 @@
       </c>
       <c r="L86" s="20" t="n"/>
       <c r="M86" s="20" t="n"/>
-      <c r="N86" s="20" t="n"/>
-      <c r="O86" s="20" t="n"/>
+      <c r="N86" s="70" t="n"/>
+      <c r="O86" s="71">
+        <f>IF(OR(M86="",N86="",M86=0),"",(N86/M86)/1440)</f>
+        <v/>
+      </c>
       <c r="P86" s="20" t="n"/>
       <c r="Q86" s="20" t="n"/>
       <c r="R86" s="20" t="n"/>
@@ -6121,8 +6382,11 @@
       </c>
       <c r="L87" s="20" t="n"/>
       <c r="M87" s="20" t="n"/>
-      <c r="N87" s="20" t="n"/>
-      <c r="O87" s="20" t="n"/>
+      <c r="N87" s="70" t="n"/>
+      <c r="O87" s="71">
+        <f>IF(OR(M87="",N87="",M87=0),"",(N87/M87)/1440)</f>
+        <v/>
+      </c>
       <c r="P87" s="20" t="n"/>
       <c r="Q87" s="20" t="n"/>
       <c r="R87" s="20" t="n"/>
@@ -6177,8 +6441,11 @@
       </c>
       <c r="L88" s="20" t="n"/>
       <c r="M88" s="20" t="n"/>
-      <c r="N88" s="20" t="n"/>
-      <c r="O88" s="20" t="n"/>
+      <c r="N88" s="70" t="n"/>
+      <c r="O88" s="71">
+        <f>IF(OR(M88="",N88="",M88=0),"",(N88/M88)/1440)</f>
+        <v/>
+      </c>
       <c r="P88" s="20" t="n"/>
       <c r="Q88" s="20" t="n"/>
       <c r="R88" s="20" t="n"/>
@@ -6235,8 +6502,11 @@
       </c>
       <c r="L89" s="20" t="n"/>
       <c r="M89" s="20" t="n"/>
-      <c r="N89" s="20" t="n"/>
-      <c r="O89" s="20" t="n"/>
+      <c r="N89" s="70" t="n"/>
+      <c r="O89" s="71">
+        <f>IF(OR(M89="",N89="",M89=0),"",(N89/M89)/1440)</f>
+        <v/>
+      </c>
       <c r="P89" s="20" t="n"/>
       <c r="Q89" s="20" t="n"/>
       <c r="R89" s="20" t="n"/>
@@ -6293,8 +6563,11 @@
       </c>
       <c r="L90" s="20" t="n"/>
       <c r="M90" s="20" t="n"/>
-      <c r="N90" s="20" t="n"/>
-      <c r="O90" s="20" t="n"/>
+      <c r="N90" s="70" t="n"/>
+      <c r="O90" s="71">
+        <f>IF(OR(M90="",N90="",M90=0),"",(N90/M90)/1440)</f>
+        <v/>
+      </c>
       <c r="P90" s="20" t="n"/>
       <c r="Q90" s="20" t="n"/>
       <c r="R90" s="20" t="n"/>
@@ -6351,8 +6624,11 @@
       </c>
       <c r="L91" s="20" t="n"/>
       <c r="M91" s="20" t="n"/>
-      <c r="N91" s="20" t="n"/>
-      <c r="O91" s="20" t="n"/>
+      <c r="N91" s="70" t="n"/>
+      <c r="O91" s="71">
+        <f>IF(OR(M91="",N91="",M91=0),"",(N91/M91)/1440)</f>
+        <v/>
+      </c>
       <c r="P91" s="20" t="n"/>
       <c r="Q91" s="20" t="n"/>
       <c r="R91" s="20" t="n"/>
@@ -6407,8 +6683,11 @@
       </c>
       <c r="L92" s="15" t="n"/>
       <c r="M92" s="15" t="n"/>
-      <c r="N92" s="15" t="n"/>
-      <c r="O92" s="15" t="n"/>
+      <c r="N92" s="68" t="n"/>
+      <c r="O92" s="69">
+        <f>IF(OR(M92="",N92="",M92=0),"",(N92/M92)/1440)</f>
+        <v/>
+      </c>
       <c r="P92" s="15" t="n"/>
       <c r="Q92" s="15" t="n"/>
       <c r="R92" s="15" t="n"/>
@@ -6463,8 +6742,11 @@
       </c>
       <c r="L93" s="15" t="n"/>
       <c r="M93" s="15" t="n"/>
-      <c r="N93" s="15" t="n"/>
-      <c r="O93" s="15" t="n"/>
+      <c r="N93" s="68" t="n"/>
+      <c r="O93" s="69">
+        <f>IF(OR(M93="",N93="",M93=0),"",(N93/M93)/1440)</f>
+        <v/>
+      </c>
       <c r="P93" s="15" t="n"/>
       <c r="Q93" s="15" t="n"/>
       <c r="R93" s="15" t="n"/>
@@ -6521,8 +6803,11 @@
       </c>
       <c r="L94" s="15" t="n"/>
       <c r="M94" s="15" t="n"/>
-      <c r="N94" s="15" t="n"/>
-      <c r="O94" s="15" t="n"/>
+      <c r="N94" s="68" t="n"/>
+      <c r="O94" s="69">
+        <f>IF(OR(M94="",N94="",M94=0),"",(N94/M94)/1440)</f>
+        <v/>
+      </c>
       <c r="P94" s="15" t="n"/>
       <c r="Q94" s="15" t="n"/>
       <c r="R94" s="15" t="n"/>
@@ -6579,8 +6864,11 @@
       </c>
       <c r="L95" s="15" t="n"/>
       <c r="M95" s="15" t="n"/>
-      <c r="N95" s="15" t="n"/>
-      <c r="O95" s="15" t="n"/>
+      <c r="N95" s="68" t="n"/>
+      <c r="O95" s="69">
+        <f>IF(OR(M95="",N95="",M95=0),"",(N95/M95)/1440)</f>
+        <v/>
+      </c>
       <c r="P95" s="15" t="n"/>
       <c r="Q95" s="15" t="n"/>
       <c r="R95" s="15" t="n"/>
@@ -6635,8 +6923,11 @@
       </c>
       <c r="L96" s="15" t="n"/>
       <c r="M96" s="15" t="n"/>
-      <c r="N96" s="15" t="n"/>
-      <c r="O96" s="15" t="n"/>
+      <c r="N96" s="68" t="n"/>
+      <c r="O96" s="69">
+        <f>IF(OR(M96="",N96="",M96=0),"",(N96/M96)/1440)</f>
+        <v/>
+      </c>
       <c r="P96" s="15" t="n"/>
       <c r="Q96" s="15" t="n"/>
       <c r="R96" s="15" t="n"/>
@@ -6693,8 +6984,11 @@
       </c>
       <c r="L97" s="15" t="n"/>
       <c r="M97" s="15" t="n"/>
-      <c r="N97" s="15" t="n"/>
-      <c r="O97" s="15" t="n"/>
+      <c r="N97" s="68" t="n"/>
+      <c r="O97" s="69">
+        <f>IF(OR(M97="",N97="",M97=0),"",(N97/M97)/1440)</f>
+        <v/>
+      </c>
       <c r="P97" s="15" t="n"/>
       <c r="Q97" s="15" t="n"/>
       <c r="R97" s="15" t="n"/>
@@ -6749,8 +7043,11 @@
       </c>
       <c r="L98" s="15" t="n"/>
       <c r="M98" s="15" t="n"/>
-      <c r="N98" s="15" t="n"/>
-      <c r="O98" s="15" t="n"/>
+      <c r="N98" s="68" t="n"/>
+      <c r="O98" s="69">
+        <f>IF(OR(M98="",N98="",M98=0),"",(N98/M98)/1440)</f>
+        <v/>
+      </c>
       <c r="P98" s="15" t="n"/>
       <c r="Q98" s="15" t="n"/>
       <c r="R98" s="15" t="n"/>
@@ -6807,8 +7104,11 @@
       </c>
       <c r="L99" s="15" t="n"/>
       <c r="M99" s="15" t="n"/>
-      <c r="N99" s="15" t="n"/>
-      <c r="O99" s="15" t="n"/>
+      <c r="N99" s="68" t="n"/>
+      <c r="O99" s="69">
+        <f>IF(OR(M99="",N99="",M99=0),"",(N99/M99)/1440)</f>
+        <v/>
+      </c>
       <c r="P99" s="15" t="n"/>
       <c r="Q99" s="15" t="n"/>
       <c r="R99" s="15" t="n"/>
@@ -6865,8 +7165,11 @@
       </c>
       <c r="L100" s="15" t="n"/>
       <c r="M100" s="15" t="n"/>
-      <c r="N100" s="15" t="n"/>
-      <c r="O100" s="15" t="n"/>
+      <c r="N100" s="68" t="n"/>
+      <c r="O100" s="69">
+        <f>IF(OR(M100="",N100="",M100=0),"",(N100/M100)/1440)</f>
+        <v/>
+      </c>
       <c r="P100" s="15" t="n"/>
       <c r="Q100" s="15" t="n"/>
       <c r="R100" s="15" t="n"/>
@@ -6923,8 +7226,11 @@
       </c>
       <c r="L101" s="15" t="n"/>
       <c r="M101" s="15" t="n"/>
-      <c r="N101" s="15" t="n"/>
-      <c r="O101" s="15" t="n"/>
+      <c r="N101" s="68" t="n"/>
+      <c r="O101" s="69">
+        <f>IF(OR(M101="",N101="",M101=0),"",(N101/M101)/1440)</f>
+        <v/>
+      </c>
       <c r="P101" s="15" t="n"/>
       <c r="Q101" s="15" t="n"/>
       <c r="R101" s="15" t="n"/>
@@ -6979,8 +7285,11 @@
       </c>
       <c r="L102" s="15" t="n"/>
       <c r="M102" s="15" t="n"/>
-      <c r="N102" s="15" t="n"/>
-      <c r="O102" s="15" t="n"/>
+      <c r="N102" s="68" t="n"/>
+      <c r="O102" s="69">
+        <f>IF(OR(M102="",N102="",M102=0),"",(N102/M102)/1440)</f>
+        <v/>
+      </c>
       <c r="P102" s="15" t="n"/>
       <c r="Q102" s="15" t="n"/>
       <c r="R102" s="15" t="n"/>
@@ -7035,8 +7344,11 @@
       </c>
       <c r="L103" s="15" t="n"/>
       <c r="M103" s="15" t="n"/>
-      <c r="N103" s="15" t="n"/>
-      <c r="O103" s="15" t="n"/>
+      <c r="N103" s="68" t="n"/>
+      <c r="O103" s="69">
+        <f>IF(OR(M103="",N103="",M103=0),"",(N103/M103)/1440)</f>
+        <v/>
+      </c>
       <c r="P103" s="15" t="n"/>
       <c r="Q103" s="15" t="n"/>
       <c r="R103" s="15" t="n"/>
@@ -7093,8 +7405,11 @@
       </c>
       <c r="L104" s="15" t="n"/>
       <c r="M104" s="15" t="n"/>
-      <c r="N104" s="15" t="n"/>
-      <c r="O104" s="15" t="n"/>
+      <c r="N104" s="68" t="n"/>
+      <c r="O104" s="69">
+        <f>IF(OR(M104="",N104="",M104=0),"",(N104/M104)/1440)</f>
+        <v/>
+      </c>
       <c r="P104" s="15" t="n"/>
       <c r="Q104" s="15" t="n"/>
       <c r="R104" s="15" t="n"/>
@@ -7151,8 +7466,11 @@
       </c>
       <c r="L105" s="15" t="n"/>
       <c r="M105" s="15" t="n"/>
-      <c r="N105" s="15" t="n"/>
-      <c r="O105" s="15" t="n"/>
+      <c r="N105" s="68" t="n"/>
+      <c r="O105" s="69">
+        <f>IF(OR(M105="",N105="",M105=0),"",(N105/M105)/1440)</f>
+        <v/>
+      </c>
       <c r="P105" s="15" t="n"/>
       <c r="Q105" s="15" t="n"/>
       <c r="R105" s="15" t="n"/>
@@ -7207,8 +7525,11 @@
       </c>
       <c r="L106" s="15" t="n"/>
       <c r="M106" s="15" t="n"/>
-      <c r="N106" s="15" t="n"/>
-      <c r="O106" s="15" t="n"/>
+      <c r="N106" s="68" t="n"/>
+      <c r="O106" s="69">
+        <f>IF(OR(M106="",N106="",M106=0),"",(N106/M106)/1440)</f>
+        <v/>
+      </c>
       <c r="P106" s="15" t="n"/>
       <c r="Q106" s="15" t="n"/>
       <c r="R106" s="15" t="n"/>
@@ -7265,8 +7586,11 @@
       </c>
       <c r="L107" s="15" t="n"/>
       <c r="M107" s="15" t="n"/>
-      <c r="N107" s="15" t="n"/>
-      <c r="O107" s="15" t="n"/>
+      <c r="N107" s="68" t="n"/>
+      <c r="O107" s="69">
+        <f>IF(OR(M107="",N107="",M107=0),"",(N107/M107)/1440)</f>
+        <v/>
+      </c>
       <c r="P107" s="15" t="n"/>
       <c r="Q107" s="15" t="n"/>
       <c r="R107" s="15" t="n"/>
@@ -7321,8 +7645,11 @@
       </c>
       <c r="L108" s="15" t="n"/>
       <c r="M108" s="15" t="n"/>
-      <c r="N108" s="15" t="n"/>
-      <c r="O108" s="15" t="n"/>
+      <c r="N108" s="68" t="n"/>
+      <c r="O108" s="69">
+        <f>IF(OR(M108="",N108="",M108=0),"",(N108/M108)/1440)</f>
+        <v/>
+      </c>
       <c r="P108" s="15" t="n"/>
       <c r="Q108" s="15" t="n"/>
       <c r="R108" s="15" t="n"/>
@@ -7379,8 +7706,11 @@
       </c>
       <c r="L109" s="15" t="n"/>
       <c r="M109" s="15" t="n"/>
-      <c r="N109" s="15" t="n"/>
-      <c r="O109" s="15" t="n"/>
+      <c r="N109" s="68" t="n"/>
+      <c r="O109" s="69">
+        <f>IF(OR(M109="",N109="",M109=0),"",(N109/M109)/1440)</f>
+        <v/>
+      </c>
       <c r="P109" s="15" t="n"/>
       <c r="Q109" s="15" t="n"/>
       <c r="R109" s="15" t="n"/>
@@ -7437,8 +7767,11 @@
       </c>
       <c r="L110" s="15" t="n"/>
       <c r="M110" s="15" t="n"/>
-      <c r="N110" s="15" t="n"/>
-      <c r="O110" s="15" t="n"/>
+      <c r="N110" s="68" t="n"/>
+      <c r="O110" s="69">
+        <f>IF(OR(M110="",N110="",M110=0),"",(N110/M110)/1440)</f>
+        <v/>
+      </c>
       <c r="P110" s="15" t="n"/>
       <c r="Q110" s="15" t="n"/>
       <c r="R110" s="15" t="n"/>
@@ -7495,8 +7828,11 @@
       </c>
       <c r="L111" s="15" t="n"/>
       <c r="M111" s="15" t="n"/>
-      <c r="N111" s="15" t="n"/>
-      <c r="O111" s="15" t="n"/>
+      <c r="N111" s="68" t="n"/>
+      <c r="O111" s="69">
+        <f>IF(OR(M111="",N111="",M111=0),"",(N111/M111)/1440)</f>
+        <v/>
+      </c>
       <c r="P111" s="15" t="n"/>
       <c r="Q111" s="15" t="n"/>
       <c r="R111" s="15" t="n"/>
@@ -7551,8 +7887,11 @@
       </c>
       <c r="L112" s="15" t="n"/>
       <c r="M112" s="15" t="n"/>
-      <c r="N112" s="15" t="n"/>
-      <c r="O112" s="15" t="n"/>
+      <c r="N112" s="68" t="n"/>
+      <c r="O112" s="69">
+        <f>IF(OR(M112="",N112="",M112=0),"",(N112/M112)/1440)</f>
+        <v/>
+      </c>
       <c r="P112" s="15" t="n"/>
       <c r="Q112" s="15" t="n"/>
       <c r="R112" s="15" t="n"/>
@@ -7607,8 +7946,11 @@
       </c>
       <c r="L113" s="15" t="n"/>
       <c r="M113" s="15" t="n"/>
-      <c r="N113" s="15" t="n"/>
-      <c r="O113" s="15" t="n"/>
+      <c r="N113" s="68" t="n"/>
+      <c r="O113" s="69">
+        <f>IF(OR(M113="",N113="",M113=0),"",(N113/M113)/1440)</f>
+        <v/>
+      </c>
       <c r="P113" s="15" t="n"/>
       <c r="Q113" s="15" t="n"/>
       <c r="R113" s="15" t="n"/>
@@ -7665,8 +8007,11 @@
       </c>
       <c r="L114" s="15" t="n"/>
       <c r="M114" s="15" t="n"/>
-      <c r="N114" s="15" t="n"/>
-      <c r="O114" s="15" t="n"/>
+      <c r="N114" s="68" t="n"/>
+      <c r="O114" s="69">
+        <f>IF(OR(M114="",N114="",M114=0),"",(N114/M114)/1440)</f>
+        <v/>
+      </c>
       <c r="P114" s="15" t="n"/>
       <c r="Q114" s="15" t="n"/>
       <c r="R114" s="15" t="n"/>
@@ -7723,8 +8068,11 @@
       </c>
       <c r="L115" s="15" t="n"/>
       <c r="M115" s="15" t="n"/>
-      <c r="N115" s="15" t="n"/>
-      <c r="O115" s="15" t="n"/>
+      <c r="N115" s="68" t="n"/>
+      <c r="O115" s="69">
+        <f>IF(OR(M115="",N115="",M115=0),"",(N115/M115)/1440)</f>
+        <v/>
+      </c>
       <c r="P115" s="15" t="n"/>
       <c r="Q115" s="15" t="n"/>
       <c r="R115" s="15" t="n"/>
@@ -7779,8 +8127,11 @@
       </c>
       <c r="L116" s="15" t="n"/>
       <c r="M116" s="15" t="n"/>
-      <c r="N116" s="15" t="n"/>
-      <c r="O116" s="15" t="n"/>
+      <c r="N116" s="68" t="n"/>
+      <c r="O116" s="69">
+        <f>IF(OR(M116="",N116="",M116=0),"",(N116/M116)/1440)</f>
+        <v/>
+      </c>
       <c r="P116" s="15" t="n"/>
       <c r="Q116" s="15" t="n"/>
       <c r="R116" s="15" t="n"/>
@@ -7837,8 +8188,11 @@
       </c>
       <c r="L117" s="15" t="n"/>
       <c r="M117" s="15" t="n"/>
-      <c r="N117" s="15" t="n"/>
-      <c r="O117" s="15" t="n"/>
+      <c r="N117" s="68" t="n"/>
+      <c r="O117" s="69">
+        <f>IF(OR(M117="",N117="",M117=0),"",(N117/M117)/1440)</f>
+        <v/>
+      </c>
       <c r="P117" s="15" t="n"/>
       <c r="Q117" s="15" t="n"/>
       <c r="R117" s="15" t="n"/>
@@ -7893,8 +8247,11 @@
       </c>
       <c r="L118" s="15" t="n"/>
       <c r="M118" s="15" t="n"/>
-      <c r="N118" s="15" t="n"/>
-      <c r="O118" s="15" t="n"/>
+      <c r="N118" s="68" t="n"/>
+      <c r="O118" s="69">
+        <f>IF(OR(M118="",N118="",M118=0),"",(N118/M118)/1440)</f>
+        <v/>
+      </c>
       <c r="P118" s="15" t="n"/>
       <c r="Q118" s="15" t="n"/>
       <c r="R118" s="15" t="n"/>
@@ -7951,8 +8308,11 @@
       </c>
       <c r="L119" s="15" t="n"/>
       <c r="M119" s="15" t="n"/>
-      <c r="N119" s="15" t="n"/>
-      <c r="O119" s="15" t="n"/>
+      <c r="N119" s="68" t="n"/>
+      <c r="O119" s="69">
+        <f>IF(OR(M119="",N119="",M119=0),"",(N119/M119)/1440)</f>
+        <v/>
+      </c>
       <c r="P119" s="15" t="n"/>
       <c r="Q119" s="15" t="n"/>
       <c r="R119" s="15" t="n"/>
@@ -8009,8 +8369,11 @@
       </c>
       <c r="L120" s="15" t="n"/>
       <c r="M120" s="15" t="n"/>
-      <c r="N120" s="15" t="n"/>
-      <c r="O120" s="15" t="n"/>
+      <c r="N120" s="68" t="n"/>
+      <c r="O120" s="69">
+        <f>IF(OR(M120="",N120="",M120=0),"",(N120/M120)/1440)</f>
+        <v/>
+      </c>
       <c r="P120" s="15" t="n"/>
       <c r="Q120" s="15" t="n"/>
       <c r="R120" s="15" t="n"/>
@@ -8067,8 +8430,11 @@
       </c>
       <c r="L121" s="15" t="n"/>
       <c r="M121" s="15" t="n"/>
-      <c r="N121" s="15" t="n"/>
-      <c r="O121" s="15" t="n"/>
+      <c r="N121" s="68" t="n"/>
+      <c r="O121" s="69">
+        <f>IF(OR(M121="",N121="",M121=0),"",(N121/M121)/1440)</f>
+        <v/>
+      </c>
       <c r="P121" s="15" t="n"/>
       <c r="Q121" s="15" t="n"/>
       <c r="R121" s="15" t="n"/>
@@ -8123,8 +8489,11 @@
       </c>
       <c r="L122" s="20" t="n"/>
       <c r="M122" s="20" t="n"/>
-      <c r="N122" s="20" t="n"/>
-      <c r="O122" s="20" t="n"/>
+      <c r="N122" s="70" t="n"/>
+      <c r="O122" s="71">
+        <f>IF(OR(M122="",N122="",M122=0),"",(N122/M122)/1440)</f>
+        <v/>
+      </c>
       <c r="P122" s="20" t="n"/>
       <c r="Q122" s="20" t="n"/>
       <c r="R122" s="20" t="n"/>
@@ -8179,8 +8548,11 @@
       </c>
       <c r="L123" s="20" t="n"/>
       <c r="M123" s="20" t="n"/>
-      <c r="N123" s="20" t="n"/>
-      <c r="O123" s="20" t="n"/>
+      <c r="N123" s="70" t="n"/>
+      <c r="O123" s="71">
+        <f>IF(OR(M123="",N123="",M123=0),"",(N123/M123)/1440)</f>
+        <v/>
+      </c>
       <c r="P123" s="20" t="n"/>
       <c r="Q123" s="20" t="n"/>
       <c r="R123" s="20" t="n"/>
@@ -8237,8 +8609,11 @@
       </c>
       <c r="L124" s="20" t="n"/>
       <c r="M124" s="20" t="n"/>
-      <c r="N124" s="20" t="n"/>
-      <c r="O124" s="20" t="n"/>
+      <c r="N124" s="70" t="n"/>
+      <c r="O124" s="71">
+        <f>IF(OR(M124="",N124="",M124=0),"",(N124/M124)/1440)</f>
+        <v/>
+      </c>
       <c r="P124" s="20" t="n"/>
       <c r="Q124" s="20" t="n"/>
       <c r="R124" s="20" t="n"/>
@@ -8295,8 +8670,11 @@
       </c>
       <c r="L125" s="20" t="n"/>
       <c r="M125" s="20" t="n"/>
-      <c r="N125" s="20" t="n"/>
-      <c r="O125" s="20" t="n"/>
+      <c r="N125" s="70" t="n"/>
+      <c r="O125" s="71">
+        <f>IF(OR(M125="",N125="",M125=0),"",(N125/M125)/1440)</f>
+        <v/>
+      </c>
       <c r="P125" s="20" t="n"/>
       <c r="Q125" s="20" t="n"/>
       <c r="R125" s="20" t="n"/>
@@ -8351,8 +8729,11 @@
       </c>
       <c r="L126" s="20" t="n"/>
       <c r="M126" s="20" t="n"/>
-      <c r="N126" s="20" t="n"/>
-      <c r="O126" s="20" t="n"/>
+      <c r="N126" s="70" t="n"/>
+      <c r="O126" s="71">
+        <f>IF(OR(M126="",N126="",M126=0),"",(N126/M126)/1440)</f>
+        <v/>
+      </c>
       <c r="P126" s="20" t="n"/>
       <c r="Q126" s="20" t="n"/>
       <c r="R126" s="20" t="n"/>
@@ -8409,8 +8790,11 @@
       </c>
       <c r="L127" s="20" t="n"/>
       <c r="M127" s="20" t="n"/>
-      <c r="N127" s="20" t="n"/>
-      <c r="O127" s="20" t="n"/>
+      <c r="N127" s="70" t="n"/>
+      <c r="O127" s="71">
+        <f>IF(OR(M127="",N127="",M127=0),"",(N127/M127)/1440)</f>
+        <v/>
+      </c>
       <c r="P127" s="20" t="n"/>
       <c r="Q127" s="20" t="n"/>
       <c r="R127" s="20" t="n"/>
@@ -8465,8 +8849,11 @@
       </c>
       <c r="L128" s="20" t="n"/>
       <c r="M128" s="20" t="n"/>
-      <c r="N128" s="20" t="n"/>
-      <c r="O128" s="20" t="n"/>
+      <c r="N128" s="70" t="n"/>
+      <c r="O128" s="71">
+        <f>IF(OR(M128="",N128="",M128=0),"",(N128/M128)/1440)</f>
+        <v/>
+      </c>
       <c r="P128" s="20" t="n"/>
       <c r="Q128" s="20" t="n"/>
       <c r="R128" s="20" t="n"/>
@@ -8523,8 +8910,11 @@
       </c>
       <c r="L129" s="20" t="n"/>
       <c r="M129" s="20" t="n"/>
-      <c r="N129" s="20" t="n"/>
-      <c r="O129" s="20" t="n"/>
+      <c r="N129" s="70" t="n"/>
+      <c r="O129" s="71">
+        <f>IF(OR(M129="",N129="",M129=0),"",(N129/M129)/1440)</f>
+        <v/>
+      </c>
       <c r="P129" s="20" t="n"/>
       <c r="Q129" s="20" t="n"/>
       <c r="R129" s="20" t="n"/>
@@ -8581,8 +8971,11 @@
       </c>
       <c r="L130" s="20" t="n"/>
       <c r="M130" s="20" t="n"/>
-      <c r="N130" s="20" t="n"/>
-      <c r="O130" s="20" t="n"/>
+      <c r="N130" s="70" t="n"/>
+      <c r="O130" s="71">
+        <f>IF(OR(M130="",N130="",M130=0),"",(N130/M130)/1440)</f>
+        <v/>
+      </c>
       <c r="P130" s="20" t="n"/>
       <c r="Q130" s="20" t="n"/>
       <c r="R130" s="20" t="n"/>
@@ -8639,8 +9032,11 @@
       </c>
       <c r="L131" s="20" t="n"/>
       <c r="M131" s="20" t="n"/>
-      <c r="N131" s="20" t="n"/>
-      <c r="O131" s="20" t="n"/>
+      <c r="N131" s="70" t="n"/>
+      <c r="O131" s="71">
+        <f>IF(OR(M131="",N131="",M131=0),"",(N131/M131)/1440)</f>
+        <v/>
+      </c>
       <c r="P131" s="20" t="n"/>
       <c r="Q131" s="20" t="n"/>
       <c r="R131" s="20" t="n"/>
@@ -8695,8 +9091,11 @@
       </c>
       <c r="L132" s="15" t="n"/>
       <c r="M132" s="15" t="n"/>
-      <c r="N132" s="15" t="n"/>
-      <c r="O132" s="15" t="n"/>
+      <c r="N132" s="68" t="n"/>
+      <c r="O132" s="69">
+        <f>IF(OR(M132="",N132="",M132=0),"",(N132/M132)/1440)</f>
+        <v/>
+      </c>
       <c r="P132" s="15" t="n"/>
       <c r="Q132" s="15" t="n"/>
       <c r="R132" s="15" t="n"/>
@@ -8751,8 +9150,11 @@
       </c>
       <c r="L133" s="15" t="n"/>
       <c r="M133" s="15" t="n"/>
-      <c r="N133" s="15" t="n"/>
-      <c r="O133" s="15" t="n"/>
+      <c r="N133" s="68" t="n"/>
+      <c r="O133" s="69">
+        <f>IF(OR(M133="",N133="",M133=0),"",(N133/M133)/1440)</f>
+        <v/>
+      </c>
       <c r="P133" s="15" t="n"/>
       <c r="Q133" s="15" t="n"/>
       <c r="R133" s="15" t="n"/>
@@ -8809,8 +9211,11 @@
       </c>
       <c r="L134" s="15" t="n"/>
       <c r="M134" s="15" t="n"/>
-      <c r="N134" s="15" t="n"/>
-      <c r="O134" s="15" t="n"/>
+      <c r="N134" s="68" t="n"/>
+      <c r="O134" s="69">
+        <f>IF(OR(M134="",N134="",M134=0),"",(N134/M134)/1440)</f>
+        <v/>
+      </c>
       <c r="P134" s="15" t="n"/>
       <c r="Q134" s="15" t="n"/>
       <c r="R134" s="15" t="n"/>
@@ -8867,8 +9272,11 @@
       </c>
       <c r="L135" s="15" t="n"/>
       <c r="M135" s="15" t="n"/>
-      <c r="N135" s="15" t="n"/>
-      <c r="O135" s="15" t="n"/>
+      <c r="N135" s="68" t="n"/>
+      <c r="O135" s="69">
+        <f>IF(OR(M135="",N135="",M135=0),"",(N135/M135)/1440)</f>
+        <v/>
+      </c>
       <c r="P135" s="15" t="n"/>
       <c r="Q135" s="15" t="n"/>
       <c r="R135" s="15" t="n"/>
@@ -8923,8 +9331,11 @@
       </c>
       <c r="L136" s="15" t="n"/>
       <c r="M136" s="15" t="n"/>
-      <c r="N136" s="15" t="n"/>
-      <c r="O136" s="15" t="n"/>
+      <c r="N136" s="68" t="n"/>
+      <c r="O136" s="69">
+        <f>IF(OR(M136="",N136="",M136=0),"",(N136/M136)/1440)</f>
+        <v/>
+      </c>
       <c r="P136" s="15" t="n"/>
       <c r="Q136" s="15" t="n"/>
       <c r="R136" s="15" t="n"/>
@@ -8981,8 +9392,11 @@
       </c>
       <c r="L137" s="15" t="n"/>
       <c r="M137" s="15" t="n"/>
-      <c r="N137" s="15" t="n"/>
-      <c r="O137" s="15" t="n"/>
+      <c r="N137" s="68" t="n"/>
+      <c r="O137" s="69">
+        <f>IF(OR(M137="",N137="",M137=0),"",(N137/M137)/1440)</f>
+        <v/>
+      </c>
       <c r="P137" s="15" t="n"/>
       <c r="Q137" s="15" t="n"/>
       <c r="R137" s="15" t="n"/>
@@ -9037,8 +9451,11 @@
       </c>
       <c r="L138" s="15" t="n"/>
       <c r="M138" s="15" t="n"/>
-      <c r="N138" s="15" t="n"/>
-      <c r="O138" s="15" t="n"/>
+      <c r="N138" s="68" t="n"/>
+      <c r="O138" s="69">
+        <f>IF(OR(M138="",N138="",M138=0),"",(N138/M138)/1440)</f>
+        <v/>
+      </c>
       <c r="P138" s="15" t="n"/>
       <c r="Q138" s="15" t="n"/>
       <c r="R138" s="15" t="n"/>
@@ -9095,8 +9512,11 @@
       </c>
       <c r="L139" s="15" t="n"/>
       <c r="M139" s="15" t="n"/>
-      <c r="N139" s="15" t="n"/>
-      <c r="O139" s="15" t="n"/>
+      <c r="N139" s="68" t="n"/>
+      <c r="O139" s="69">
+        <f>IF(OR(M139="",N139="",M139=0),"",(N139/M139)/1440)</f>
+        <v/>
+      </c>
       <c r="P139" s="15" t="n"/>
       <c r="Q139" s="15" t="n"/>
       <c r="R139" s="15" t="n"/>
@@ -9153,8 +9573,11 @@
       </c>
       <c r="L140" s="15" t="n"/>
       <c r="M140" s="15" t="n"/>
-      <c r="N140" s="15" t="n"/>
-      <c r="O140" s="15" t="n"/>
+      <c r="N140" s="68" t="n"/>
+      <c r="O140" s="69">
+        <f>IF(OR(M140="",N140="",M140=0),"",(N140/M140)/1440)</f>
+        <v/>
+      </c>
       <c r="P140" s="15" t="n"/>
       <c r="Q140" s="15" t="n"/>
       <c r="R140" s="15" t="n"/>
@@ -9211,8 +9634,11 @@
       </c>
       <c r="L141" s="15" t="n"/>
       <c r="M141" s="15" t="n"/>
-      <c r="N141" s="15" t="n"/>
-      <c r="O141" s="15" t="n"/>
+      <c r="N141" s="68" t="n"/>
+      <c r="O141" s="69">
+        <f>IF(OR(M141="",N141="",M141=0),"",(N141/M141)/1440)</f>
+        <v/>
+      </c>
       <c r="P141" s="15" t="n"/>
       <c r="Q141" s="15" t="n"/>
       <c r="R141" s="15" t="n"/>
@@ -9267,8 +9693,11 @@
       </c>
       <c r="L142" s="15" t="n"/>
       <c r="M142" s="15" t="n"/>
-      <c r="N142" s="15" t="n"/>
-      <c r="O142" s="15" t="n"/>
+      <c r="N142" s="68" t="n"/>
+      <c r="O142" s="69">
+        <f>IF(OR(M142="",N142="",M142=0),"",(N142/M142)/1440)</f>
+        <v/>
+      </c>
       <c r="P142" s="15" t="n"/>
       <c r="Q142" s="15" t="n"/>
       <c r="R142" s="15" t="n"/>
@@ -9323,8 +9752,11 @@
       </c>
       <c r="L143" s="15" t="n"/>
       <c r="M143" s="15" t="n"/>
-      <c r="N143" s="15" t="n"/>
-      <c r="O143" s="15" t="n"/>
+      <c r="N143" s="68" t="n"/>
+      <c r="O143" s="69">
+        <f>IF(OR(M143="",N143="",M143=0),"",(N143/M143)/1440)</f>
+        <v/>
+      </c>
       <c r="P143" s="15" t="n"/>
       <c r="Q143" s="15" t="n"/>
       <c r="R143" s="15" t="n"/>
@@ -9381,8 +9813,11 @@
       </c>
       <c r="L144" s="15" t="n"/>
       <c r="M144" s="15" t="n"/>
-      <c r="N144" s="15" t="n"/>
-      <c r="O144" s="15" t="n"/>
+      <c r="N144" s="68" t="n"/>
+      <c r="O144" s="69">
+        <f>IF(OR(M144="",N144="",M144=0),"",(N144/M144)/1440)</f>
+        <v/>
+      </c>
       <c r="P144" s="15" t="n"/>
       <c r="Q144" s="15" t="n"/>
       <c r="R144" s="15" t="n"/>
@@ -9439,8 +9874,11 @@
       </c>
       <c r="L145" s="15" t="n"/>
       <c r="M145" s="15" t="n"/>
-      <c r="N145" s="15" t="n"/>
-      <c r="O145" s="15" t="n"/>
+      <c r="N145" s="68" t="n"/>
+      <c r="O145" s="69">
+        <f>IF(OR(M145="",N145="",M145=0),"",(N145/M145)/1440)</f>
+        <v/>
+      </c>
       <c r="P145" s="15" t="n"/>
       <c r="Q145" s="15" t="n"/>
       <c r="R145" s="15" t="n"/>
@@ -9495,8 +9933,11 @@
       </c>
       <c r="L146" s="15" t="n"/>
       <c r="M146" s="15" t="n"/>
-      <c r="N146" s="15" t="n"/>
-      <c r="O146" s="15" t="n"/>
+      <c r="N146" s="68" t="n"/>
+      <c r="O146" s="69">
+        <f>IF(OR(M146="",N146="",M146=0),"",(N146/M146)/1440)</f>
+        <v/>
+      </c>
       <c r="P146" s="15" t="n"/>
       <c r="Q146" s="15" t="n"/>
       <c r="R146" s="15" t="n"/>
@@ -9553,8 +9994,11 @@
       </c>
       <c r="L147" s="15" t="n"/>
       <c r="M147" s="15" t="n"/>
-      <c r="N147" s="15" t="n"/>
-      <c r="O147" s="15" t="n"/>
+      <c r="N147" s="68" t="n"/>
+      <c r="O147" s="69">
+        <f>IF(OR(M147="",N147="",M147=0),"",(N147/M147)/1440)</f>
+        <v/>
+      </c>
       <c r="P147" s="15" t="n"/>
       <c r="Q147" s="15" t="n"/>
       <c r="R147" s="15" t="n"/>
@@ -9609,8 +10053,11 @@
       </c>
       <c r="L148" s="15" t="n"/>
       <c r="M148" s="15" t="n"/>
-      <c r="N148" s="15" t="n"/>
-      <c r="O148" s="15" t="n"/>
+      <c r="N148" s="68" t="n"/>
+      <c r="O148" s="69">
+        <f>IF(OR(M148="",N148="",M148=0),"",(N148/M148)/1440)</f>
+        <v/>
+      </c>
       <c r="P148" s="15" t="n"/>
       <c r="Q148" s="15" t="n"/>
       <c r="R148" s="15" t="n"/>
@@ -9667,8 +10114,11 @@
       </c>
       <c r="L149" s="15" t="n"/>
       <c r="M149" s="15" t="n"/>
-      <c r="N149" s="15" t="n"/>
-      <c r="O149" s="15" t="n"/>
+      <c r="N149" s="68" t="n"/>
+      <c r="O149" s="69">
+        <f>IF(OR(M149="",N149="",M149=0),"",(N149/M149)/1440)</f>
+        <v/>
+      </c>
       <c r="P149" s="15" t="n"/>
       <c r="Q149" s="15" t="n"/>
       <c r="R149" s="15" t="n"/>
@@ -9725,8 +10175,11 @@
       </c>
       <c r="L150" s="15" t="n"/>
       <c r="M150" s="15" t="n"/>
-      <c r="N150" s="15" t="n"/>
-      <c r="O150" s="15" t="n"/>
+      <c r="N150" s="68" t="n"/>
+      <c r="O150" s="69">
+        <f>IF(OR(M150="",N150="",M150=0),"",(N150/M150)/1440)</f>
+        <v/>
+      </c>
       <c r="P150" s="15" t="n"/>
       <c r="Q150" s="15" t="n"/>
       <c r="R150" s="15" t="n"/>
@@ -9783,8 +10236,11 @@
       </c>
       <c r="L151" s="15" t="n"/>
       <c r="M151" s="15" t="n"/>
-      <c r="N151" s="15" t="n"/>
-      <c r="O151" s="15" t="n"/>
+      <c r="N151" s="68" t="n"/>
+      <c r="O151" s="69">
+        <f>IF(OR(M151="",N151="",M151=0),"",(N151/M151)/1440)</f>
+        <v/>
+      </c>
       <c r="P151" s="15" t="n"/>
       <c r="Q151" s="15" t="n"/>
       <c r="R151" s="15" t="n"/>
@@ -9839,8 +10295,11 @@
       </c>
       <c r="L152" s="15" t="n"/>
       <c r="M152" s="15" t="n"/>
-      <c r="N152" s="15" t="n"/>
-      <c r="O152" s="15" t="n"/>
+      <c r="N152" s="68" t="n"/>
+      <c r="O152" s="69">
+        <f>IF(OR(M152="",N152="",M152=0),"",(N152/M152)/1440)</f>
+        <v/>
+      </c>
       <c r="P152" s="15" t="n"/>
       <c r="Q152" s="15" t="n"/>
       <c r="R152" s="15" t="n"/>
@@ -9895,8 +10354,11 @@
       </c>
       <c r="L153" s="15" t="n"/>
       <c r="M153" s="15" t="n"/>
-      <c r="N153" s="15" t="n"/>
-      <c r="O153" s="15" t="n"/>
+      <c r="N153" s="68" t="n"/>
+      <c r="O153" s="69">
+        <f>IF(OR(M153="",N153="",M153=0),"",(N153/M153)/1440)</f>
+        <v/>
+      </c>
       <c r="P153" s="15" t="n"/>
       <c r="Q153" s="15" t="n"/>
       <c r="R153" s="15" t="n"/>
@@ -9953,8 +10415,11 @@
       </c>
       <c r="L154" s="15" t="n"/>
       <c r="M154" s="15" t="n"/>
-      <c r="N154" s="15" t="n"/>
-      <c r="O154" s="15" t="n"/>
+      <c r="N154" s="68" t="n"/>
+      <c r="O154" s="69">
+        <f>IF(OR(M154="",N154="",M154=0),"",(N154/M154)/1440)</f>
+        <v/>
+      </c>
       <c r="P154" s="15" t="n"/>
       <c r="Q154" s="15" t="n"/>
       <c r="R154" s="15" t="n"/>
@@ -10011,8 +10476,11 @@
       </c>
       <c r="L155" s="15" t="n"/>
       <c r="M155" s="15" t="n"/>
-      <c r="N155" s="15" t="n"/>
-      <c r="O155" s="15" t="n"/>
+      <c r="N155" s="68" t="n"/>
+      <c r="O155" s="69">
+        <f>IF(OR(M155="",N155="",M155=0),"",(N155/M155)/1440)</f>
+        <v/>
+      </c>
       <c r="P155" s="15" t="n"/>
       <c r="Q155" s="15" t="n"/>
       <c r="R155" s="15" t="n"/>
@@ -10067,8 +10535,11 @@
       </c>
       <c r="L156" s="15" t="n"/>
       <c r="M156" s="15" t="n"/>
-      <c r="N156" s="15" t="n"/>
-      <c r="O156" s="15" t="n"/>
+      <c r="N156" s="68" t="n"/>
+      <c r="O156" s="69">
+        <f>IF(OR(M156="",N156="",M156=0),"",(N156/M156)/1440)</f>
+        <v/>
+      </c>
       <c r="P156" s="15" t="n"/>
       <c r="Q156" s="15" t="n"/>
       <c r="R156" s="15" t="n"/>
@@ -10125,8 +10596,11 @@
       </c>
       <c r="L157" s="15" t="n"/>
       <c r="M157" s="15" t="n"/>
-      <c r="N157" s="15" t="n"/>
-      <c r="O157" s="15" t="n"/>
+      <c r="N157" s="68" t="n"/>
+      <c r="O157" s="69">
+        <f>IF(OR(M157="",N157="",M157=0),"",(N157/M157)/1440)</f>
+        <v/>
+      </c>
       <c r="P157" s="15" t="n"/>
       <c r="Q157" s="15" t="n"/>
       <c r="R157" s="15" t="n"/>
@@ -10181,8 +10655,11 @@
       </c>
       <c r="L158" s="15" t="n"/>
       <c r="M158" s="15" t="n"/>
-      <c r="N158" s="15" t="n"/>
-      <c r="O158" s="15" t="n"/>
+      <c r="N158" s="68" t="n"/>
+      <c r="O158" s="69">
+        <f>IF(OR(M158="",N158="",M158=0),"",(N158/M158)/1440)</f>
+        <v/>
+      </c>
       <c r="P158" s="15" t="n"/>
       <c r="Q158" s="15" t="n"/>
       <c r="R158" s="15" t="n"/>
@@ -10239,8 +10716,11 @@
       </c>
       <c r="L159" s="15" t="n"/>
       <c r="M159" s="15" t="n"/>
-      <c r="N159" s="15" t="n"/>
-      <c r="O159" s="15" t="n"/>
+      <c r="N159" s="68" t="n"/>
+      <c r="O159" s="69">
+        <f>IF(OR(M159="",N159="",M159=0),"",(N159/M159)/1440)</f>
+        <v/>
+      </c>
       <c r="P159" s="15" t="n"/>
       <c r="Q159" s="15" t="n"/>
       <c r="R159" s="15" t="n"/>
@@ -10297,8 +10777,11 @@
       </c>
       <c r="L160" s="15" t="n"/>
       <c r="M160" s="15" t="n"/>
-      <c r="N160" s="15" t="n"/>
-      <c r="O160" s="15" t="n"/>
+      <c r="N160" s="68" t="n"/>
+      <c r="O160" s="69">
+        <f>IF(OR(M160="",N160="",M160=0),"",(N160/M160)/1440)</f>
+        <v/>
+      </c>
       <c r="P160" s="15" t="n"/>
       <c r="Q160" s="15" t="n"/>
       <c r="R160" s="15" t="n"/>
@@ -10355,8 +10838,11 @@
       </c>
       <c r="L161" s="15" t="n"/>
       <c r="M161" s="15" t="n"/>
-      <c r="N161" s="15" t="n"/>
-      <c r="O161" s="15" t="n"/>
+      <c r="N161" s="68" t="n"/>
+      <c r="O161" s="69">
+        <f>IF(OR(M161="",N161="",M161=0),"",(N161/M161)/1440)</f>
+        <v/>
+      </c>
       <c r="P161" s="15" t="n"/>
       <c r="Q161" s="15" t="n"/>
       <c r="R161" s="15" t="n"/>
@@ -10411,8 +10897,11 @@
       </c>
       <c r="L162" s="15" t="n"/>
       <c r="M162" s="15" t="n"/>
-      <c r="N162" s="15" t="n"/>
-      <c r="O162" s="15" t="n"/>
+      <c r="N162" s="68" t="n"/>
+      <c r="O162" s="69">
+        <f>IF(OR(M162="",N162="",M162=0),"",(N162/M162)/1440)</f>
+        <v/>
+      </c>
       <c r="P162" s="15" t="n"/>
       <c r="Q162" s="15" t="n"/>
       <c r="R162" s="15" t="n"/>
@@ -10467,8 +10956,11 @@
       </c>
       <c r="L163" s="15" t="n"/>
       <c r="M163" s="15" t="n"/>
-      <c r="N163" s="15" t="n"/>
-      <c r="O163" s="15" t="n"/>
+      <c r="N163" s="68" t="n"/>
+      <c r="O163" s="69">
+        <f>IF(OR(M163="",N163="",M163=0),"",(N163/M163)/1440)</f>
+        <v/>
+      </c>
       <c r="P163" s="15" t="n"/>
       <c r="Q163" s="15" t="n"/>
       <c r="R163" s="15" t="n"/>
@@ -10525,8 +11017,11 @@
       </c>
       <c r="L164" s="15" t="n"/>
       <c r="M164" s="15" t="n"/>
-      <c r="N164" s="15" t="n"/>
-      <c r="O164" s="15" t="n"/>
+      <c r="N164" s="68" t="n"/>
+      <c r="O164" s="69">
+        <f>IF(OR(M164="",N164="",M164=0),"",(N164/M164)/1440)</f>
+        <v/>
+      </c>
       <c r="P164" s="15" t="n"/>
       <c r="Q164" s="15" t="n"/>
       <c r="R164" s="15" t="n"/>
@@ -10583,8 +11078,11 @@
       </c>
       <c r="L165" s="15" t="n"/>
       <c r="M165" s="15" t="n"/>
-      <c r="N165" s="15" t="n"/>
-      <c r="O165" s="15" t="n"/>
+      <c r="N165" s="68" t="n"/>
+      <c r="O165" s="69">
+        <f>IF(OR(M165="",N165="",M165=0),"",(N165/M165)/1440)</f>
+        <v/>
+      </c>
       <c r="P165" s="15" t="n"/>
       <c r="Q165" s="15" t="n"/>
       <c r="R165" s="15" t="n"/>
@@ -10639,8 +11137,11 @@
       </c>
       <c r="L166" s="15" t="n"/>
       <c r="M166" s="15" t="n"/>
-      <c r="N166" s="15" t="n"/>
-      <c r="O166" s="15" t="n"/>
+      <c r="N166" s="68" t="n"/>
+      <c r="O166" s="69">
+        <f>IF(OR(M166="",N166="",M166=0),"",(N166/M166)/1440)</f>
+        <v/>
+      </c>
       <c r="P166" s="15" t="n"/>
       <c r="Q166" s="15" t="n"/>
       <c r="R166" s="15" t="n"/>
@@ -10697,8 +11198,11 @@
       </c>
       <c r="L167" s="15" t="n"/>
       <c r="M167" s="15" t="n"/>
-      <c r="N167" s="15" t="n"/>
-      <c r="O167" s="15" t="n"/>
+      <c r="N167" s="68" t="n"/>
+      <c r="O167" s="69">
+        <f>IF(OR(M167="",N167="",M167=0),"",(N167/M167)/1440)</f>
+        <v/>
+      </c>
       <c r="P167" s="15" t="n"/>
       <c r="Q167" s="15" t="n"/>
       <c r="R167" s="15" t="n"/>
@@ -10753,8 +11257,11 @@
       </c>
       <c r="L168" s="15" t="n"/>
       <c r="M168" s="15" t="n"/>
-      <c r="N168" s="15" t="n"/>
-      <c r="O168" s="15" t="n"/>
+      <c r="N168" s="68" t="n"/>
+      <c r="O168" s="69">
+        <f>IF(OR(M168="",N168="",M168=0),"",(N168/M168)/1440)</f>
+        <v/>
+      </c>
       <c r="P168" s="15" t="n"/>
       <c r="Q168" s="15" t="n"/>
       <c r="R168" s="15" t="n"/>
@@ -10811,8 +11318,11 @@
       </c>
       <c r="L169" s="15" t="n"/>
       <c r="M169" s="15" t="n"/>
-      <c r="N169" s="15" t="n"/>
-      <c r="O169" s="15" t="n"/>
+      <c r="N169" s="68" t="n"/>
+      <c r="O169" s="69">
+        <f>IF(OR(M169="",N169="",M169=0),"",(N169/M169)/1440)</f>
+        <v/>
+      </c>
       <c r="P169" s="15" t="n"/>
       <c r="Q169" s="15" t="n"/>
       <c r="R169" s="15" t="n"/>
@@ -10869,8 +11379,11 @@
       </c>
       <c r="L170" s="15" t="n"/>
       <c r="M170" s="15" t="n"/>
-      <c r="N170" s="15" t="n"/>
-      <c r="O170" s="15" t="n"/>
+      <c r="N170" s="68" t="n"/>
+      <c r="O170" s="69">
+        <f>IF(OR(M170="",N170="",M170=0),"",(N170/M170)/1440)</f>
+        <v/>
+      </c>
       <c r="P170" s="15" t="n"/>
       <c r="Q170" s="15" t="n"/>
       <c r="R170" s="15" t="n"/>
@@ -10927,8 +11440,11 @@
       </c>
       <c r="L171" s="15" t="n"/>
       <c r="M171" s="15" t="n"/>
-      <c r="N171" s="15" t="n"/>
-      <c r="O171" s="15" t="n"/>
+      <c r="N171" s="68" t="n"/>
+      <c r="O171" s="69">
+        <f>IF(OR(M171="",N171="",M171=0),"",(N171/M171)/1440)</f>
+        <v/>
+      </c>
       <c r="P171" s="15" t="n"/>
       <c r="Q171" s="15" t="n"/>
       <c r="R171" s="15" t="n"/>
@@ -10983,8 +11499,11 @@
       </c>
       <c r="L172" s="15" t="n"/>
       <c r="M172" s="15" t="n"/>
-      <c r="N172" s="15" t="n"/>
-      <c r="O172" s="15" t="n"/>
+      <c r="N172" s="68" t="n"/>
+      <c r="O172" s="69">
+        <f>IF(OR(M172="",N172="",M172=0),"",(N172/M172)/1440)</f>
+        <v/>
+      </c>
       <c r="P172" s="15" t="n"/>
       <c r="Q172" s="15" t="n"/>
       <c r="R172" s="15" t="n"/>
@@ -11039,8 +11558,11 @@
       </c>
       <c r="L173" s="15" t="n"/>
       <c r="M173" s="15" t="n"/>
-      <c r="N173" s="15" t="n"/>
-      <c r="O173" s="15" t="n"/>
+      <c r="N173" s="68" t="n"/>
+      <c r="O173" s="69">
+        <f>IF(OR(M173="",N173="",M173=0),"",(N173/M173)/1440)</f>
+        <v/>
+      </c>
       <c r="P173" s="15" t="n"/>
       <c r="Q173" s="15" t="n"/>
       <c r="R173" s="15" t="n"/>
@@ -11097,8 +11619,11 @@
       </c>
       <c r="L174" s="15" t="n"/>
       <c r="M174" s="15" t="n"/>
-      <c r="N174" s="15" t="n"/>
-      <c r="O174" s="15" t="n"/>
+      <c r="N174" s="68" t="n"/>
+      <c r="O174" s="69">
+        <f>IF(OR(M174="",N174="",M174=0),"",(N174/M174)/1440)</f>
+        <v/>
+      </c>
       <c r="P174" s="15" t="n"/>
       <c r="Q174" s="15" t="n"/>
       <c r="R174" s="15" t="n"/>
@@ -11155,8 +11680,11 @@
       </c>
       <c r="L175" s="15" t="n"/>
       <c r="M175" s="15" t="n"/>
-      <c r="N175" s="15" t="n"/>
-      <c r="O175" s="15" t="n"/>
+      <c r="N175" s="68" t="n"/>
+      <c r="O175" s="69">
+        <f>IF(OR(M175="",N175="",M175=0),"",(N175/M175)/1440)</f>
+        <v/>
+      </c>
       <c r="P175" s="15" t="n"/>
       <c r="Q175" s="15" t="n"/>
       <c r="R175" s="15" t="n"/>
@@ -11211,8 +11739,11 @@
       </c>
       <c r="L176" s="15" t="n"/>
       <c r="M176" s="15" t="n"/>
-      <c r="N176" s="15" t="n"/>
-      <c r="O176" s="15" t="n"/>
+      <c r="N176" s="68" t="n"/>
+      <c r="O176" s="69">
+        <f>IF(OR(M176="",N176="",M176=0),"",(N176/M176)/1440)</f>
+        <v/>
+      </c>
       <c r="P176" s="15" t="n"/>
       <c r="Q176" s="15" t="n"/>
       <c r="R176" s="15" t="n"/>
@@ -11269,8 +11800,11 @@
       </c>
       <c r="L177" s="15" t="n"/>
       <c r="M177" s="15" t="n"/>
-      <c r="N177" s="15" t="n"/>
-      <c r="O177" s="15" t="n"/>
+      <c r="N177" s="68" t="n"/>
+      <c r="O177" s="69">
+        <f>IF(OR(M177="",N177="",M177=0),"",(N177/M177)/1440)</f>
+        <v/>
+      </c>
       <c r="P177" s="15" t="n"/>
       <c r="Q177" s="15" t="n"/>
       <c r="R177" s="15" t="n"/>
@@ -11325,8 +11859,11 @@
       </c>
       <c r="L178" s="15" t="n"/>
       <c r="M178" s="15" t="n"/>
-      <c r="N178" s="15" t="n"/>
-      <c r="O178" s="15" t="n"/>
+      <c r="N178" s="68" t="n"/>
+      <c r="O178" s="69">
+        <f>IF(OR(M178="",N178="",M178=0),"",(N178/M178)/1440)</f>
+        <v/>
+      </c>
       <c r="P178" s="15" t="n"/>
       <c r="Q178" s="15" t="n"/>
       <c r="R178" s="15" t="n"/>
@@ -11383,8 +11920,11 @@
       </c>
       <c r="L179" s="15" t="n"/>
       <c r="M179" s="15" t="n"/>
-      <c r="N179" s="15" t="n"/>
-      <c r="O179" s="15" t="n"/>
+      <c r="N179" s="68" t="n"/>
+      <c r="O179" s="69">
+        <f>IF(OR(M179="",N179="",M179=0),"",(N179/M179)/1440)</f>
+        <v/>
+      </c>
       <c r="P179" s="15" t="n"/>
       <c r="Q179" s="15" t="n"/>
       <c r="R179" s="15" t="n"/>
@@ -11441,8 +11981,11 @@
       </c>
       <c r="L180" s="15" t="n"/>
       <c r="M180" s="15" t="n"/>
-      <c r="N180" s="15" t="n"/>
-      <c r="O180" s="15" t="n"/>
+      <c r="N180" s="68" t="n"/>
+      <c r="O180" s="69">
+        <f>IF(OR(M180="",N180="",M180=0),"",(N180/M180)/1440)</f>
+        <v/>
+      </c>
       <c r="P180" s="15" t="n"/>
       <c r="Q180" s="15" t="n"/>
       <c r="R180" s="15" t="n"/>
@@ -11499,8 +12042,11 @@
       </c>
       <c r="L181" s="15" t="n"/>
       <c r="M181" s="15" t="n"/>
-      <c r="N181" s="15" t="n"/>
-      <c r="O181" s="15" t="n"/>
+      <c r="N181" s="68" t="n"/>
+      <c r="O181" s="69">
+        <f>IF(OR(M181="",N181="",M181=0),"",(N181/M181)/1440)</f>
+        <v/>
+      </c>
       <c r="P181" s="15" t="n"/>
       <c r="Q181" s="15" t="n"/>
       <c r="R181" s="15" t="n"/>
@@ -11555,8 +12101,11 @@
       </c>
       <c r="L182" s="15" t="n"/>
       <c r="M182" s="15" t="n"/>
-      <c r="N182" s="15" t="n"/>
-      <c r="O182" s="15" t="n"/>
+      <c r="N182" s="68" t="n"/>
+      <c r="O182" s="69">
+        <f>IF(OR(M182="",N182="",M182=0),"",(N182/M182)/1440)</f>
+        <v/>
+      </c>
       <c r="P182" s="15" t="n"/>
       <c r="Q182" s="15" t="n"/>
       <c r="R182" s="15" t="n"/>
@@ -11611,8 +12160,11 @@
       </c>
       <c r="L183" s="15" t="n"/>
       <c r="M183" s="15" t="n"/>
-      <c r="N183" s="15" t="n"/>
-      <c r="O183" s="15" t="n"/>
+      <c r="N183" s="68" t="n"/>
+      <c r="O183" s="69">
+        <f>IF(OR(M183="",N183="",M183=0),"",(N183/M183)/1440)</f>
+        <v/>
+      </c>
       <c r="P183" s="15" t="n"/>
       <c r="Q183" s="15" t="n"/>
       <c r="R183" s="15" t="n"/>
@@ -11669,8 +12221,11 @@
       </c>
       <c r="L184" s="15" t="n"/>
       <c r="M184" s="15" t="n"/>
-      <c r="N184" s="15" t="n"/>
-      <c r="O184" s="15" t="n"/>
+      <c r="N184" s="68" t="n"/>
+      <c r="O184" s="69">
+        <f>IF(OR(M184="",N184="",M184=0),"",(N184/M184)/1440)</f>
+        <v/>
+      </c>
       <c r="P184" s="15" t="n"/>
       <c r="Q184" s="15" t="n"/>
       <c r="R184" s="15" t="n"/>
@@ -11727,8 +12282,11 @@
       </c>
       <c r="L185" s="15" t="n"/>
       <c r="M185" s="15" t="n"/>
-      <c r="N185" s="15" t="n"/>
-      <c r="O185" s="15" t="n"/>
+      <c r="N185" s="68" t="n"/>
+      <c r="O185" s="69">
+        <f>IF(OR(M185="",N185="",M185=0),"",(N185/M185)/1440)</f>
+        <v/>
+      </c>
       <c r="P185" s="15" t="n"/>
       <c r="Q185" s="15" t="n"/>
       <c r="R185" s="15" t="n"/>
@@ -11783,8 +12341,11 @@
       </c>
       <c r="L186" s="15" t="n"/>
       <c r="M186" s="15" t="n"/>
-      <c r="N186" s="15" t="n"/>
-      <c r="O186" s="15" t="n"/>
+      <c r="N186" s="68" t="n"/>
+      <c r="O186" s="69">
+        <f>IF(OR(M186="",N186="",M186=0),"",(N186/M186)/1440)</f>
+        <v/>
+      </c>
       <c r="P186" s="15" t="n"/>
       <c r="Q186" s="15" t="n"/>
       <c r="R186" s="15" t="n"/>
@@ -11841,8 +12402,11 @@
       </c>
       <c r="L187" s="15" t="n"/>
       <c r="M187" s="15" t="n"/>
-      <c r="N187" s="15" t="n"/>
-      <c r="O187" s="15" t="n"/>
+      <c r="N187" s="68" t="n"/>
+      <c r="O187" s="69">
+        <f>IF(OR(M187="",N187="",M187=0),"",(N187/M187)/1440)</f>
+        <v/>
+      </c>
       <c r="P187" s="15" t="n"/>
       <c r="Q187" s="15" t="n"/>
       <c r="R187" s="15" t="n"/>
@@ -11897,8 +12461,11 @@
       </c>
       <c r="L188" s="15" t="n"/>
       <c r="M188" s="15" t="n"/>
-      <c r="N188" s="15" t="n"/>
-      <c r="O188" s="15" t="n"/>
+      <c r="N188" s="68" t="n"/>
+      <c r="O188" s="69">
+        <f>IF(OR(M188="",N188="",M188=0),"",(N188/M188)/1440)</f>
+        <v/>
+      </c>
       <c r="P188" s="15" t="n"/>
       <c r="Q188" s="15" t="n"/>
       <c r="R188" s="15" t="n"/>
@@ -11955,8 +12522,11 @@
       </c>
       <c r="L189" s="15" t="n"/>
       <c r="M189" s="15" t="n"/>
-      <c r="N189" s="15" t="n"/>
-      <c r="O189" s="15" t="n"/>
+      <c r="N189" s="68" t="n"/>
+      <c r="O189" s="69">
+        <f>IF(OR(M189="",N189="",M189=0),"",(N189/M189)/1440)</f>
+        <v/>
+      </c>
       <c r="P189" s="15" t="n"/>
       <c r="Q189" s="15" t="n"/>
       <c r="R189" s="15" t="n"/>
@@ -12013,8 +12583,11 @@
       </c>
       <c r="L190" s="15" t="n"/>
       <c r="M190" s="15" t="n"/>
-      <c r="N190" s="15" t="n"/>
-      <c r="O190" s="15" t="n"/>
+      <c r="N190" s="68" t="n"/>
+      <c r="O190" s="69">
+        <f>IF(OR(M190="",N190="",M190=0),"",(N190/M190)/1440)</f>
+        <v/>
+      </c>
       <c r="P190" s="15" t="n"/>
       <c r="Q190" s="15" t="n"/>
       <c r="R190" s="15" t="n"/>
@@ -12071,8 +12644,11 @@
       </c>
       <c r="L191" s="15" t="n"/>
       <c r="M191" s="15" t="n"/>
-      <c r="N191" s="15" t="n"/>
-      <c r="O191" s="15" t="n"/>
+      <c r="N191" s="68" t="n"/>
+      <c r="O191" s="69">
+        <f>IF(OR(M191="",N191="",M191=0),"",(N191/M191)/1440)</f>
+        <v/>
+      </c>
       <c r="P191" s="15" t="n"/>
       <c r="Q191" s="15" t="n"/>
       <c r="R191" s="15" t="n"/>
@@ -12127,8 +12703,11 @@
       </c>
       <c r="L192" s="15" t="n"/>
       <c r="M192" s="15" t="n"/>
-      <c r="N192" s="15" t="n"/>
-      <c r="O192" s="15" t="n"/>
+      <c r="N192" s="68" t="n"/>
+      <c r="O192" s="69">
+        <f>IF(OR(M192="",N192="",M192=0),"",(N192/M192)/1440)</f>
+        <v/>
+      </c>
       <c r="P192" s="15" t="n"/>
       <c r="Q192" s="15" t="n"/>
       <c r="R192" s="15" t="n"/>
@@ -12183,8 +12762,11 @@
       </c>
       <c r="L193" s="15" t="n"/>
       <c r="M193" s="15" t="n"/>
-      <c r="N193" s="15" t="n"/>
-      <c r="O193" s="15" t="n"/>
+      <c r="N193" s="68" t="n"/>
+      <c r="O193" s="69">
+        <f>IF(OR(M193="",N193="",M193=0),"",(N193/M193)/1440)</f>
+        <v/>
+      </c>
       <c r="P193" s="15" t="n"/>
       <c r="Q193" s="15" t="n"/>
       <c r="R193" s="15" t="n"/>
@@ -12241,8 +12823,11 @@
       </c>
       <c r="L194" s="15" t="n"/>
       <c r="M194" s="15" t="n"/>
-      <c r="N194" s="15" t="n"/>
-      <c r="O194" s="15" t="n"/>
+      <c r="N194" s="68" t="n"/>
+      <c r="O194" s="69">
+        <f>IF(OR(M194="",N194="",M194=0),"",(N194/M194)/1440)</f>
+        <v/>
+      </c>
       <c r="P194" s="15" t="n"/>
       <c r="Q194" s="15" t="n"/>
       <c r="R194" s="15" t="n"/>
@@ -12299,8 +12884,11 @@
       </c>
       <c r="L195" s="15" t="n"/>
       <c r="M195" s="15" t="n"/>
-      <c r="N195" s="15" t="n"/>
-      <c r="O195" s="15" t="n"/>
+      <c r="N195" s="68" t="n"/>
+      <c r="O195" s="69">
+        <f>IF(OR(M195="",N195="",M195=0),"",(N195/M195)/1440)</f>
+        <v/>
+      </c>
       <c r="P195" s="15" t="n"/>
       <c r="Q195" s="15" t="n"/>
       <c r="R195" s="15" t="n"/>
@@ -12355,8 +12943,11 @@
       </c>
       <c r="L196" s="15" t="n"/>
       <c r="M196" s="15" t="n"/>
-      <c r="N196" s="15" t="n"/>
-      <c r="O196" s="15" t="n"/>
+      <c r="N196" s="68" t="n"/>
+      <c r="O196" s="69">
+        <f>IF(OR(M196="",N196="",M196=0),"",(N196/M196)/1440)</f>
+        <v/>
+      </c>
       <c r="P196" s="15" t="n"/>
       <c r="Q196" s="15" t="n"/>
       <c r="R196" s="15" t="n"/>
@@ -12411,8 +13002,11 @@
       </c>
       <c r="L197" s="15" t="n"/>
       <c r="M197" s="15" t="n"/>
-      <c r="N197" s="15" t="n"/>
-      <c r="O197" s="15" t="n"/>
+      <c r="N197" s="68" t="n"/>
+      <c r="O197" s="69">
+        <f>IF(OR(M197="",N197="",M197=0),"",(N197/M197)/1440)</f>
+        <v/>
+      </c>
       <c r="P197" s="15" t="n"/>
       <c r="Q197" s="15" t="n"/>
       <c r="R197" s="15" t="n"/>
@@ -12469,8 +13063,11 @@
       </c>
       <c r="L198" s="15" t="n"/>
       <c r="M198" s="15" t="n"/>
-      <c r="N198" s="15" t="n"/>
-      <c r="O198" s="15" t="n"/>
+      <c r="N198" s="68" t="n"/>
+      <c r="O198" s="69">
+        <f>IF(OR(M198="",N198="",M198=0),"",(N198/M198)/1440)</f>
+        <v/>
+      </c>
       <c r="P198" s="15" t="n"/>
       <c r="Q198" s="15" t="n"/>
       <c r="R198" s="15" t="n"/>
@@ -12527,8 +13124,11 @@
       </c>
       <c r="L199" s="15" t="n"/>
       <c r="M199" s="15" t="n"/>
-      <c r="N199" s="15" t="n"/>
-      <c r="O199" s="15" t="n"/>
+      <c r="N199" s="68" t="n"/>
+      <c r="O199" s="69">
+        <f>IF(OR(M199="",N199="",M199=0),"",(N199/M199)/1440)</f>
+        <v/>
+      </c>
       <c r="P199" s="15" t="n"/>
       <c r="Q199" s="15" t="n"/>
       <c r="R199" s="15" t="n"/>

</xml_diff>

<commit_message>
Log Mon 3 Aug: Gym Legs + easy run (4.5km, 5:40/km reported)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="dddd\,\ dd\ mmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="ddd\ dd\-mmm\-yy"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
@@ -31,7 +31,6 @@
     <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="170" formatCode="dd-mmm-yy"/>
     <numFmt numFmtId="171" formatCode="ddd dd-mmm-yy"/>
-    <numFmt numFmtId="172" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -2471,7 +2470,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L18" s="65" t="n"/>
+      <c r="L18" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M18" s="65" t="n"/>
       <c r="N18" s="66" t="n"/>
       <c r="O18" s="67">
@@ -2532,9 +2535,17 @@
           <t>Easy run</t>
         </is>
       </c>
-      <c r="L19" s="65" t="n"/>
-      <c r="M19" s="65" t="n"/>
-      <c r="N19" s="66" t="n"/>
+      <c r="L19" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M19" s="65" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N19" s="66" t="n">
+        <v>26</v>
+      </c>
       <c r="O19" s="67">
         <f>IF(AND(ISNUMBER(M19),ISNUMBER(N19),M19&gt;0),(N19/M19)/1440,"")</f>
         <v/>

</xml_diff>

<commit_message>
Log Tue 4 Aug: medium-long run, 6km in 42min (7:00/km)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2604,9 +2604,17 @@
           <t>Medium-long - steady</t>
         </is>
       </c>
-      <c r="L20" s="65" t="n"/>
-      <c r="M20" s="65" t="n"/>
-      <c r="N20" s="66" t="n"/>
+      <c r="L20" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M20" s="65" t="n">
+        <v>6</v>
+      </c>
+      <c r="N20" s="66" t="n">
+        <v>42</v>
+      </c>
       <c r="O20" s="67">
         <f>IF(AND(ISNUMBER(M20),ISNUMBER(N20),M20&gt;0),(N20/M20)/1440,"")</f>
         <v/>

</xml_diff>

<commit_message>
Log Wed 5 Aug: Gym Push skipped
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2671,7 +2671,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L21" s="65" t="n"/>
+      <c r="L21" s="65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M21" s="65" t="n"/>
       <c r="N21" s="66" t="n"/>
       <c r="O21" s="67">
@@ -2680,7 +2684,11 @@
       </c>
       <c r="P21" s="65" t="n"/>
       <c r="Q21" s="65" t="n"/>
-      <c r="R21" s="65" t="n"/>
+      <c r="R21" s="65" t="inlineStr">
+        <is>
+          <t>Skipped - no training that day</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="63" t="n">

</xml_diff>

<commit_message>
Log Thu 6 Aug: intervals completed, 6.1km in 33min
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2740,16 +2740,28 @@
           <t>6 x 400 m</t>
         </is>
       </c>
-      <c r="L22" s="65" t="n"/>
-      <c r="M22" s="65" t="n"/>
-      <c r="N22" s="66" t="n"/>
+      <c r="L22" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M22" s="65" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="N22" s="66" t="n">
+        <v>33</v>
+      </c>
       <c r="O22" s="67">
         <f>IF(AND(ISNUMBER(M22),ISNUMBER(N22),M22&gt;0),(N22/M22)/1440,"")</f>
         <v/>
       </c>
       <c r="P22" s="65" t="n"/>
       <c r="Q22" s="65" t="n"/>
-      <c r="R22" s="65" t="n"/>
+      <c r="R22" s="65" t="inlineStr">
+        <is>
+          <t>1.5km@10.5kph WU, 6x(400m@13.5kph/200m@9kph), 1km@10.5kph CD</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="63" t="n">

</xml_diff>

<commit_message>
Log Fri 7 Aug: Gym Pull completed
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2811,7 +2811,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L23" s="65" t="n"/>
+      <c r="L23" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M23" s="65" t="n"/>
       <c r="N23" s="66" t="n"/>
       <c r="O23" s="67">

</xml_diff>

<commit_message>
Log Sat 8 Aug: long run, 12km in 69min (5:45/km)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2876,9 +2876,17 @@
           <t>Long run - easy</t>
         </is>
       </c>
-      <c r="L24" s="65" t="n"/>
-      <c r="M24" s="65" t="n"/>
-      <c r="N24" s="66" t="n"/>
+      <c r="L24" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M24" s="65" t="n">
+        <v>12</v>
+      </c>
+      <c r="N24" s="66" t="n">
+        <v>69</v>
+      </c>
       <c r="O24" s="67">
         <f>IF(AND(ISNUMBER(M24),ISNUMBER(N24),M24&gt;0),(N24/M24)/1440,"")</f>
         <v/>

</xml_diff>

<commit_message>
Log Week 3 RPE: easy 5, medium-long 4, intervals 6, long run 8
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2550,7 +2550,9 @@
         <f>IF(AND(ISNUMBER(M19),ISNUMBER(N19),M19&gt;0),(N19/M19)/1440,"")</f>
         <v/>
       </c>
-      <c r="P19" s="65" t="n"/>
+      <c r="P19" s="65" t="n">
+        <v>5</v>
+      </c>
       <c r="Q19" s="65" t="n"/>
       <c r="R19" s="65" t="n"/>
     </row>
@@ -2619,7 +2621,9 @@
         <f>IF(AND(ISNUMBER(M20),ISNUMBER(N20),M20&gt;0),(N20/M20)/1440,"")</f>
         <v/>
       </c>
-      <c r="P20" s="65" t="n"/>
+      <c r="P20" s="65" t="n">
+        <v>4</v>
+      </c>
       <c r="Q20" s="65" t="n"/>
       <c r="R20" s="65" t="n"/>
     </row>
@@ -2755,7 +2759,9 @@
         <f>IF(AND(ISNUMBER(M22),ISNUMBER(N22),M22&gt;0),(N22/M22)/1440,"")</f>
         <v/>
       </c>
-      <c r="P22" s="65" t="n"/>
+      <c r="P22" s="65" t="n">
+        <v>6</v>
+      </c>
       <c r="Q22" s="65" t="n"/>
       <c r="R22" s="65" t="inlineStr">
         <is>
@@ -2891,7 +2897,9 @@
         <f>IF(AND(ISNUMBER(M24),ISNUMBER(N24),M24&gt;0),(N24/M24)/1440,"")</f>
         <v/>
       </c>
-      <c r="P24" s="65" t="n"/>
+      <c r="P24" s="65" t="n">
+        <v>8</v>
+      </c>
       <c r="Q24" s="65" t="n"/>
       <c r="R24" s="65" t="n"/>
     </row>

</xml_diff>

<commit_message>
Log Mon 10 Aug: easy run done, Gym Legs skipped
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3010,7 +3010,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L26" s="65" t="n"/>
+      <c r="L26" s="65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M26" s="65" t="n"/>
       <c r="N26" s="66" t="n"/>
       <c r="O26" s="67">
@@ -3071,8 +3075,14 @@
           <t>Easy run</t>
         </is>
       </c>
-      <c r="L27" s="65" t="n"/>
-      <c r="M27" s="65" t="n"/>
+      <c r="L27" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M27" s="65" t="n">
+        <v>4.5</v>
+      </c>
       <c r="N27" s="66" t="n"/>
       <c r="O27" s="67">
         <f>IF(AND(ISNUMBER(M27),ISNUMBER(N27),M27&gt;0),(N27/M27)/1440,"")</f>

</xml_diff>

<commit_message>
Log Mon 27 Jul (Gym skipped), Tue 11 Aug + Wed 12 Aug (done)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -1851,7 +1851,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L9" s="65" t="n"/>
+      <c r="L9" s="65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M9" s="65" t="n"/>
       <c r="N9" s="66" t="n"/>
       <c r="O9" s="67">
@@ -3142,8 +3146,14 @@
           <t>Medium-long - steady</t>
         </is>
       </c>
-      <c r="L28" s="65" t="n"/>
-      <c r="M28" s="65" t="n"/>
+      <c r="L28" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M28" s="65" t="n">
+        <v>6</v>
+      </c>
       <c r="N28" s="66" t="n"/>
       <c r="O28" s="67">
         <f>IF(AND(ISNUMBER(M28),ISNUMBER(N28),M28&gt;0),(N28/M28)/1440,"")</f>
@@ -3201,7 +3211,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L29" s="65" t="n"/>
+      <c r="L29" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M29" s="65" t="n"/>
       <c r="N29" s="66" t="n"/>
       <c r="O29" s="67">

</xml_diff>

<commit_message>
Log Thu 13 Aug (tempo done) and Fri 14 Aug (Gym Pull skipped)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3276,8 +3276,14 @@
           <t>15-min tempo</t>
         </is>
       </c>
-      <c r="L30" s="65" t="n"/>
-      <c r="M30" s="65" t="n"/>
+      <c r="L30" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M30" s="65" t="n">
+        <v>5.5</v>
+      </c>
       <c r="N30" s="66" t="n"/>
       <c r="O30" s="67">
         <f>IF(AND(ISNUMBER(M30),ISNUMBER(N30),M30&gt;0),(N30/M30)/1440,"")</f>
@@ -3335,7 +3341,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L31" s="65" t="n"/>
+      <c r="L31" s="65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M31" s="65" t="n"/>
       <c r="N31" s="66" t="n"/>
       <c r="O31" s="67">

</xml_diff>

<commit_message>
Note: Fri 14 Aug padel (90min, ~1000kcal) in place of skipped gym
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3354,7 +3354,11 @@
       </c>
       <c r="P31" s="65" t="n"/>
       <c r="Q31" s="65" t="n"/>
-      <c r="R31" s="65" t="n"/>
+      <c r="R31" s="65" t="inlineStr">
+        <is>
+          <t>Skipped gym; played padel instead (90min, ~1000kcal)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="63" t="n">

</xml_diff>

<commit_message>
Log Sat 15 Aug long run: 10km (planned 14) at 6:40/km
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3410,16 +3410,28 @@
           <t>Long run - easy</t>
         </is>
       </c>
-      <c r="L32" s="65" t="n"/>
-      <c r="M32" s="65" t="n"/>
-      <c r="N32" s="66" t="n"/>
+      <c r="L32" s="65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M32" s="65" t="n">
+        <v>10</v>
+      </c>
+      <c r="N32" s="66" t="n">
+        <v>67</v>
+      </c>
       <c r="O32" s="67">
         <f>IF(AND(ISNUMBER(M32),ISNUMBER(N32),M32&gt;0),(N32/M32)/1440,"")</f>
         <v/>
       </c>
       <c r="P32" s="65" t="n"/>
       <c r="Q32" s="65" t="n"/>
-      <c r="R32" s="65" t="n"/>
+      <c r="R32" s="65" t="inlineStr">
+        <is>
+          <t>Cut short (planned 14km) - eased off after padel the day before</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="70" t="n">

</xml_diff>

<commit_message>
Log Mon 17 Aug: Gym Legs + easy run both skipped
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3540,7 +3540,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L34" s="72" t="n"/>
+      <c r="L34" s="72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M34" s="72" t="n"/>
       <c r="N34" s="73" t="n"/>
       <c r="O34" s="74">
@@ -3601,7 +3605,11 @@
           <t>Easy run</t>
         </is>
       </c>
-      <c r="L35" s="72" t="n"/>
+      <c r="L35" s="72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="M35" s="72" t="n"/>
       <c r="N35" s="73" t="n"/>
       <c r="O35" s="74">

</xml_diff>

<commit_message>
Log Tue 18 Aug: medium-long run done (5km)
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3670,8 +3670,14 @@
           <t>Medium-long - steady</t>
         </is>
       </c>
-      <c r="L36" s="72" t="n"/>
-      <c r="M36" s="72" t="n"/>
+      <c r="L36" s="72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M36" s="72" t="n">
+        <v>5</v>
+      </c>
       <c r="N36" s="73" t="n"/>
       <c r="O36" s="74">
         <f>IF(AND(ISNUMBER(M36),ISNUMBER(N36),M36&gt;0),(N36/M36)/1440,"")</f>

</xml_diff>

<commit_message>
Log Wed 19 Aug: Gym Push done
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3735,7 +3735,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="L37" s="72" t="n"/>
+      <c r="L37" s="72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="M37" s="72" t="n"/>
       <c r="N37" s="73" t="n"/>
       <c r="O37" s="74">

</xml_diff>

<commit_message>
Fix undercounted distance on Workouts/Weekly Plan for tempo+intervals
The Workouts sheet's "Approx. km" for every broken-tempo and
intervals entry was missing the jog-recovery distance (and, for
time-based reps, computed from pace x time). Recomputed all 18
affected entries (warm-up + reps + recovery jogs + cool-down,
strides at ~0.1km each), fixed the Workouts sheet, and propagated
the corrected numbers to every Weekly Plan row referencing them via
the Workout column (16 rows; 2 entries already rounded correctly).
Biggest correction: "10 x 2 min" was listed at 7.5km, actually ~11km
given the reps + full recovery jogs.
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="H22" s="63" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I22" s="63" t="inlineStr">
         <is>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="H30" s="63" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I30" s="63" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="H38" s="75" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="I38" s="75" t="inlineStr">
         <is>
@@ -4263,7 +4263,7 @@
         </is>
       </c>
       <c r="H46" s="63" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I46" s="63" t="inlineStr">
         <is>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H54" s="63" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="I54" s="63" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="H62" s="77" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I62" s="77" t="inlineStr">
         <is>
@@ -5703,7 +5703,7 @@
         </is>
       </c>
       <c r="H70" s="77" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="I70" s="77" t="inlineStr">
         <is>
@@ -6663,7 +6663,7 @@
         </is>
       </c>
       <c r="H86" s="77" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I86" s="77" t="inlineStr">
         <is>
@@ -7143,7 +7143,7 @@
         </is>
       </c>
       <c r="H94" s="77" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I94" s="77" t="inlineStr">
         <is>
@@ -8103,7 +8103,7 @@
         </is>
       </c>
       <c r="H110" s="81" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="I110" s="81" t="inlineStr">
         <is>
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="H118" s="83" t="n">
-        <v>7.5</v>
+        <v>11</v>
       </c>
       <c r="I118" s="83" t="inlineStr">
         <is>
@@ -9063,7 +9063,7 @@
         </is>
       </c>
       <c r="H126" s="83" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="I126" s="83" t="inlineStr">
         <is>
@@ -9543,7 +9543,7 @@
         </is>
       </c>
       <c r="H134" s="83" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="I134" s="83" t="inlineStr">
         <is>
@@ -10023,7 +10023,7 @@
         </is>
       </c>
       <c r="H142" s="83" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="I142" s="83" t="inlineStr">
         <is>
@@ -10503,7 +10503,7 @@
         </is>
       </c>
       <c r="H150" s="85" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="I150" s="85" t="inlineStr">
         <is>
@@ -10983,7 +10983,7 @@
         </is>
       </c>
       <c r="H158" s="85" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="I158" s="85" t="inlineStr">
         <is>
@@ -12013,7 +12013,7 @@
         </is>
       </c>
       <c r="H14" s="43" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I14" s="43" t="inlineStr">
         <is>
@@ -12053,7 +12053,7 @@
         </is>
       </c>
       <c r="H15" s="43" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I15" s="43" t="inlineStr">
         <is>
@@ -12093,7 +12093,7 @@
         </is>
       </c>
       <c r="H16" s="43" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I16" s="43" t="inlineStr">
         <is>
@@ -12173,7 +12173,7 @@
         </is>
       </c>
       <c r="H18" s="43" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I18" s="43" t="inlineStr">
         <is>
@@ -12213,7 +12213,7 @@
         </is>
       </c>
       <c r="H19" s="43" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="I19" s="43" t="inlineStr">
         <is>
@@ -12253,7 +12253,7 @@
         </is>
       </c>
       <c r="H20" s="43" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="I20" s="43" t="inlineStr">
         <is>
@@ -12293,7 +12293,7 @@
         </is>
       </c>
       <c r="H21" s="43" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="I21" s="43" t="inlineStr">
         <is>
@@ -12333,7 +12333,7 @@
         </is>
       </c>
       <c r="H22" s="43" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="I22" s="43" t="inlineStr">
         <is>
@@ -12387,7 +12387,7 @@
         </is>
       </c>
       <c r="H24" s="43" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="I24" s="43" t="inlineStr">
         <is>
@@ -12427,7 +12427,7 @@
         </is>
       </c>
       <c r="H25" s="43" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="I25" s="43" t="inlineStr">
         <is>
@@ -12467,7 +12467,7 @@
         </is>
       </c>
       <c r="H26" s="43" t="n">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="I26" s="43" t="inlineStr">
         <is>
@@ -12507,7 +12507,7 @@
         </is>
       </c>
       <c r="H27" s="43" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="I27" s="43" t="inlineStr">
         <is>
@@ -12547,7 +12547,7 @@
         </is>
       </c>
       <c r="H28" s="43" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="I28" s="43" t="inlineStr">
         <is>
@@ -12587,7 +12587,7 @@
         </is>
       </c>
       <c r="H29" s="43" t="n">
-        <v>7.5</v>
+        <v>11</v>
       </c>
       <c r="I29" s="43" t="inlineStr">
         <is>
@@ -12627,7 +12627,7 @@
         </is>
       </c>
       <c r="H30" s="43" t="n">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="I30" s="43" t="inlineStr">
         <is>
@@ -12667,7 +12667,7 @@
         </is>
       </c>
       <c r="H31" s="43" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="I31" s="43" t="inlineStr">
         <is>
@@ -12889,6 +12889,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Log Sat 22 Aug: long run cut to 8km, significant soreness/fatigue
</commit_message>
<xml_diff>
--- a/Marathon_Training_Plan.xlsx
+++ b/Marathon_Training_Plan.xlsx
@@ -3920,16 +3920,34 @@
           <t>Long run - easy</t>
         </is>
       </c>
-      <c r="L40" s="72" t="n"/>
-      <c r="M40" s="72" t="n"/>
-      <c r="N40" s="73" t="n"/>
+      <c r="L40" s="72" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M40" s="72" t="n">
+        <v>8</v>
+      </c>
+      <c r="N40" s="73" t="n">
+        <v>63</v>
+      </c>
       <c r="O40" s="74">
         <f>IF(AND(ISNUMBER(M40),ISNUMBER(N40),M40&gt;0),(N40/M40)/1440,"")</f>
         <v/>
       </c>
-      <c r="P40" s="72" t="n"/>
-      <c r="Q40" s="72" t="n"/>
-      <c r="R40" s="72" t="n"/>
+      <c r="P40" s="72" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q40" s="72" t="inlineStr">
+        <is>
+          <t>Sore</t>
+        </is>
+      </c>
+      <c r="R40" s="72" t="inlineStr">
+        <is>
+          <t>Cut short (planned 11km): first 5km@9kph(~6:40/km), last 3km@6kph(~10:00/km) - legs very sore, felt overtrained. Walked 10km the day before.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="68" t="n">
@@ -12889,7 +12907,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>

</xml_diff>